<commit_message>
feat(crm): sincroniza 160 leads com roteiro completo de abordagem 50% OFF e modelo de site pronto
</commit_message>
<xml_diff>
--- a/prospeccao_160_leads_sp.xlsx
+++ b/prospeccao_160_leads_sp.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M161"/>
+  <dimension ref="A1:K161"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="40.83203125" customWidth="1"/>
@@ -408,10 +408,8 @@
     <col min="7" max="7" width="12.83203125" customWidth="1"/>
     <col min="8" max="8" width="20.83203125" customWidth="1"/>
     <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="35.83203125" customWidth="1"/>
-    <col min="11" max="11" width="45.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="80.83203125" customWidth="1"/>
+    <col min="10" max="10" width="50.83203125" customWidth="1"/>
+    <col min="11" max="11" width="90.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -443,16 +441,10 @@
         <v>Situação do Site</v>
       </c>
       <c r="J1" t="str">
-        <v>Link Atual</v>
+        <v>Link WhatsApp Direto</v>
       </c>
       <c r="K1" t="str">
-        <v>Endereço Completo</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Link WhatsApp Direto</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Mensagem de Abordagem (50% OFF)</v>
+        <v>Mensagem de Abordagem (50% OFF + Site Pronto)</v>
       </c>
     </row>
     <row r="2" xml:space="preserve">
@@ -484,20 +476,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J2" t="str">
-        <v>https://linktr.ee/drafefernandes</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Consultório 3 - Av. Moaci, 525 - Conj 609 - Moema, São Paulo - SP, 04081-002</v>
-      </c>
-      <c r="L2" t="str">
-        <v>https://wa.me/5511991307186?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511991307186?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Fernandes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K2" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Fernandes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -529,20 +514,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J3" t="str">
-        <v>https://linktr.ee/drasamaraoliveira_?utm_source=ig&amp;utm_medium=social&amp;utm_content=link_in_bio&amp;fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQPOTM2NjE5NzQzMzkyNDU5AAGnfH1dXc14yvpmnoJ4k1irpfNClsn3d8yKB1Fov3MFQvQ8wKwpsOIMBgLt9XQ_aem_nMyhVMbErrB6Z85L6mXYkw</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Alameda dos Jurupis, 455 - Sl 92 - Moema, São Paulo - SP, 04088-001</v>
-      </c>
-      <c r="L3" t="str">
-        <v>https://wa.me/5511964799591?text=Ol%C3%A1%2C%20Dra.%20Samara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Samara! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511964799591?text=Ol%C3%A1%2C%20Dra.%20Samara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Samara%20Oliveira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K3" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Samara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Samara Oliveira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -574,20 +552,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J4" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Alameda dos Nhambiquaras, 1770 - Cj. 209 - Moema, São Paulo - SP, 04090-004</v>
-      </c>
-      <c r="L4" t="str">
-        <v>https://wa.me/5511940394742?text=Ol%C3%A1%2C%20Odontoreli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontoreli! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511940394742?text=Ol%C3%A1%2C%20Odontoreli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontoreli%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K4" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Odontoreli! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontoreli, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -619,20 +590,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J5" t="str">
-        <v>https://www.doctoralia.com.br/marcia-ayres/dentista/sao-paulo</v>
-      </c>
-      <c r="K5" t="str">
-        <v>Av. Moema, 265 - Conj 101 - Indianópolis, São Paulo - SP, 04077-020</v>
-      </c>
-      <c r="L5" t="str">
-        <v>https://wa.me/5511971268686?text=Ol%C3%A1%2C%20Dra.%20Marcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marcia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511971268686?text=Ol%C3%A1%2C%20Dra.%20Marcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcia%20Ayres%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K5" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Marcia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcia Ayres, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -664,20 +628,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J6" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K6" t="str">
-        <v>R. Teodoro Sampaio, 2222 - 2° andar - Pinheiros, São Paulo - SP, 05406-150</v>
-      </c>
-      <c r="L6" t="str">
-        <v>https://wa.me/5511984843250?text=Ol%C3%A1%2C%20Dr.%20Paulo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. Paulo! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511984843250?text=Ol%C3%A1%2C%20Dr.%20Paulo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Dent%C3%A1rio%20Dr.%20Paulo%20Rog%C3%A9rio%20Barbosa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dr. Paulo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Dentário Dr. Paulo Rogério Barbosa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -709,20 +666,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J7" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K7" t="str">
-        <v>R. Teodoro Sampaio, 2490 - Pinheiros, São Paulo - SP, 05406-200</v>
-      </c>
-      <c r="L7" t="str">
-        <v>https://wa.me/5511925683124?text=Ol%C3%A1%2C%20Oral%20Premium!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Oral Premium! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511925683124?text=Ol%C3%A1%2C%20Oral%20Premium!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Oral%20Premium%20Implantes%20Pinheiros%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Oral Premium! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Oral Premium Implantes Pinheiros, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -754,20 +704,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J8" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K8" t="str">
-        <v>R. Pais Leme, 215 - Cj 2105 - Pinheiros, São Paulo - SP, 05424-150</v>
-      </c>
-      <c r="L8" t="str">
-        <v>https://wa.me/5511944502942?text=Ol%C3%A1%2C%20Cairo%20Martinelli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Cairo Martinelli! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511944502942?text=Ol%C3%A1%2C%20Cairo%20Martinelli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cairo%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Cairo Martinelli! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cairo Martinelli Odontologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -799,20 +742,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J9" t="str">
-        <v>http://instagram.com/dr.viniciusbibiano</v>
-      </c>
-      <c r="K9" t="str">
-        <v>R. Teodoro Sampaio, 2550 - 3 andar - conjunto 33 - Pinheiros, São Paulo - SP, 05406-200</v>
-      </c>
-      <c r="L9" t="str">
-        <v>https://wa.me/5511993616602?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M9" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993616602?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20Bibiano%20%7C%20Dentista%20em%20Pinheiros%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica Bibiano | Dentista em Pinheiros, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -844,20 +780,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J10" t="str">
-        <v>https://wa.me/message/H22QFMB4FZMYD1</v>
-      </c>
-      <c r="K10" t="str">
-        <v>Av. Paulista, 807 - Sl 618 - Cerqueira César, São Paulo - SP, 01419-002</v>
-      </c>
-      <c r="L10" t="str">
-        <v>https://wa.me/5511950060220?text=Ol%C3%A1%2C%20Dra.%20J%C3%A9ssica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Jéssica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511950060220?text=Ol%C3%A1%2C%20Dra.%20J%C3%A9ssica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20J%C3%A9ssica%20Mattos%20de%20Britto%20-%20Odontologia%20Est%C3%A9tica%20e%20Restauradora%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Jéssica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Jéssica Mattos de Britto - Odontologia Estética e Restauradora, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -889,20 +818,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J11" t="str">
-        <v>http://instagram.com/dramariagoncalves</v>
-      </c>
-      <c r="K11" t="str">
-        <v>Av. Paulista, 807 - Sl 924 - Bela Vista, São Paulo - SP, 01311-100</v>
-      </c>
-      <c r="L11" t="str">
-        <v>https://wa.me/5511910995184?text=Ol%C3%A1%2C%20Dra%20Maria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Maria! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511910995184?text=Ol%C3%A1%2C%20Dra%20Maria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Maria%20Eduarda%20Gon%C3%A7alves%20%7C%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Maria! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Maria Eduarda Gonçalves | Cirurgiã Dentista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -934,20 +856,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J12" t="str">
-        <v>https://www.instagram.com/drgalsander?igsh=MXRwZ3JlZXQ3cXN3Yg==</v>
-      </c>
-      <c r="K12" t="str">
-        <v>Itaim Bibi, São Paulo - SP, 04500-000</v>
-      </c>
-      <c r="L12" t="str">
-        <v>https://wa.me/5511976253586?text=Ol%C3%A1%2C%20Dr.%20Galsander!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. Galsander! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976253586?text=Ol%C3%A1%2C%20Dr.%20Galsander!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Galsander%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K12" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dr. Galsander! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Galsander, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -979,20 +894,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J13" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K13" t="str">
-        <v>R. Domingos de Morais, 2747 - Vila Mariana, São Paulo - SP, 04035-001</v>
-      </c>
-      <c r="L13" t="str">
-        <v>https://wa.me/5511964008778?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M13" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Odontologia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511964008778?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20AR%20Odontologia%20-%20Dr.%20C%C3%A9sar%20e%20Equipe%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K13" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica AR Odontologia - Dr. César e Equipe, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -1024,20 +932,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J14" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K14" t="str">
-        <v>R. Domingos de Morais, 1456 - Vila Mariana, São Paulo - SP, 04010-200</v>
-      </c>
-      <c r="L14" t="str">
-        <v>https://wa.me/5511947647807?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M14" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511947647807?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20LK%20%7C%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K14" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica LK | Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
@@ -1069,20 +970,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J15" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K15" t="str">
-        <v>R. Dr. Tirso Martins, 100 - Conj 107 - Vila Mariana, São Paulo - SP, 04120-050</v>
-      </c>
-      <c r="L15" t="str">
-        <v>https://wa.me/5511999919290?text=Ol%C3%A1%2C%20Dra.%20Carolina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Carolina! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511999919290?text=Ol%C3%A1%2C%20Dra.%20Carolina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Carolina%20Oliveira%20-%20Endodontia%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K15" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Carolina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Carolina Oliveira - Endodontia e Harmonização Facial na Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -1114,20 +1008,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J16" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K16" t="str">
-        <v>Rua Loefgreen, 1291 - cj93 - Vila Clementino, São Paulo - SP, 04040-031</v>
-      </c>
-      <c r="L16" t="str">
-        <v>https://wa.me/5511958187028?text=Ol%C3%A1%2C%20Odontologico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontologico! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511958187028?text=Ol%C3%A1%2C%20Odontologico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontologico%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K16" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Odontologico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontologico na Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -1159,20 +1046,13 @@
         <v>Sem site próprio (Apenas negocio)</v>
       </c>
       <c r="J17" t="str">
-        <v>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;url=https://dentista-dra-andreia-serra.negocio.site/&amp;ved=2ahUKEwjc5ueF7v_nAhWjLLkGHd-pDB0QFjAZegQIBxAB&amp;usg=AOvVaw23N10dPXvHyJEkdydgJi0X</v>
-      </c>
-      <c r="K17" t="str">
-        <v>R. Domingos de Morais, 2781 - Conj 913 - Vila Mariana, São Paulo - SP, 04035-001</v>
-      </c>
-      <c r="L17" t="str">
-        <v>https://wa.me/5511975911100?text=Ol%C3%A1%2C%20Dra.%20Andreia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Andreia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511975911100?text=Ol%C3%A1%2C%20Dra.%20Andreia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Andreia%20Serra%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K17" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Andreia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Andreia Serra, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
@@ -1204,20 +1084,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J18" t="str">
-        <v>https://l.instagram.com/?u=https://linktr.ee/dramarciaharumimurata&amp;e=AT1N9YDKEugyBbEwe94G4hO-NzSWSyHgF1RhzSumj7pTZk2roJYnt2LifhIyfVpvgBMPU_BNIypnIsxCYq9APoSsmxxIDJQmdYcOiodw1AyXxK6TeRLfyw</v>
-      </c>
-      <c r="K18" t="str">
-        <v>R. Padre Estevão Pernet, 1059 - Vila Gomes Cardim, São Paulo - SP, 03315-000</v>
-      </c>
-      <c r="L18" t="str">
-        <v>https://wa.me/5511976088594?text=Ol%C3%A1%2C%20Dentista!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976088594?text=Ol%C3%A1%2C%20Dentista!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20-%20Tatuap%C3%A9%20-%20Dra.%20Marcia%20Harumi%20Murata%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K18" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dentista! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista - Tatuapé - Dra. Marcia Harumi Murata, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
@@ -1249,20 +1122,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J19" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K19" t="str">
-        <v>R. Tuiuti, 2009 - Conj 112 - Tatuapé, São Paulo - SP, 03307-005</v>
-      </c>
-      <c r="L19" t="str">
-        <v>https://wa.me/5511930252702?text=Ol%C3%A1%2C%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M19" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontológico! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511930252702?text=Ol%C3%A1%2C%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra%20Regiane%20Carvalheiro%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K19" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Odontológico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra Regiane Carvalheiro, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
@@ -1294,20 +1160,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J20" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K20" t="str">
-        <v>R. Serra de Juréa, 54 - Tatuapé, São Paulo - SP, 03323-020</v>
-      </c>
-      <c r="L20" t="str">
-        <v>https://wa.me/5511951406244?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M20" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511951406244?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Faustino%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K20" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Faustino, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -1339,20 +1198,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J21" t="str">
-        <v>https://instagram.com/dra_annacarolina</v>
-      </c>
-      <c r="K21" t="str">
-        <v>R. Padre Estevão Pernet, 1059 - Tatuapé, São Paulo - SP, 03315-000</v>
-      </c>
-      <c r="L21" t="str">
-        <v>https://wa.me/5511985969605?text=Ol%C3%A1%2C%20Dra%20Anna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M21" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Anna! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511985969605?text=Ol%C3%A1%2C%20Dra%20Anna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Anna%20Carolina%20%7C%20Dentista%20%7C%20Harmoniza%C3%A7%C3%A3o%20%7C%20Aparelho%20invis%C3%ADvel%20-%20sousmile%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K21" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Anna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Anna Carolina | Dentista | Harmonização | Aparelho invisível - sousmile | Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1384,20 +1236,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J22" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K22" t="str">
-        <v>R. Padre Estevão Pernet, 160 - Tatuapé, São Paulo - SP, 03590-090</v>
-      </c>
-      <c r="L22" t="str">
-        <v>https://wa.me/5511985133002?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511985133002?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20S%C3%A3o%20Paulo%20Dra%20Bianca%20Assis%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K22" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista São Paulo Dra Bianca Assis Cirurgiã Dentista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -1429,20 +1274,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J23" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K23" t="str">
-        <v>R. Cel. Carlos Oliva, 113 - Sl 07 - Tatuapé, São Paulo - SP, 03067-010</v>
-      </c>
-      <c r="L23" t="str">
-        <v>https://wa.me/5511976103809?text=Ol%C3%A1%2C%20Dra.%20Daniella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M23" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Daniella! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976103809?text=Ol%C3%A1%2C%20Dra.%20Daniella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Daniella%20Plaza%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K23" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Daniella! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Daniella Plaza, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1474,20 +1312,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J24" t="str">
-        <v>https://instagram.com/dratamymenezes?igshid=MzMyNGUyNmU2YQ==</v>
-      </c>
-      <c r="K24" t="str">
-        <v>R. Apucarana, 272 - Sl 603 - Tatuapé, São Paulo - SP, 03311-000</v>
-      </c>
-      <c r="L24" t="str">
-        <v>https://wa.me/5511945231034?text=Ol%C3%A1%2C%20Clinica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clinica Odontologia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511945231034?text=Ol%C3%A1%2C%20Clinica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Odontologia%20Especializada%20-%20Dra%20Thamiris%20Menezes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K24" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clinica Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Odontologia Especializada - Dra Thamiris Menezes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1519,20 +1350,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J25" t="str">
-        <v>https://www.instagram.com/dradanielleoliveiraa?igsh=MW5oc3U0YWQ4Mmcyag==&amp;utm_source=qr</v>
-      </c>
-      <c r="K25" t="str">
-        <v>R. Dr. Homem de Melo, 644 - Perdizes, São Paulo - SP, 05007-002</v>
-      </c>
-      <c r="L25" t="str">
-        <v>https://wa.me/5511991519479?text=Ol%C3%A1%2C%20Dra.%20Danielle!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Danielle! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511991519479?text=Ol%C3%A1%2C%20Dra.%20Danielle!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Danielle%20Oliveira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K25" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Danielle! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Danielle Oliveira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1564,20 +1388,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J26" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K26" t="str">
-        <v>R. Cardoso de Almeida - Perdizes, São Paulo - SP, 05013-001</v>
-      </c>
-      <c r="L26" t="str">
-        <v>https://wa.me/5511992918335?text=Ol%C3%A1%2C%20Dra.%20Isadora!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M26" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Isadora! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511992918335?text=Ol%C3%A1%2C%20Dra.%20Isadora!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Isadora%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K26" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Isadora! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Isadora Martinelli Odontologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1609,20 +1426,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J27" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K27" t="str">
-        <v>R. Bocaina, 108 - Sl 01 - Perdizes, São Paulo - SP, 05013-030</v>
-      </c>
-      <c r="L27" t="str">
-        <v>https://wa.me/5511963239000?text=Ol%C3%A1%2C%20Dra%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Helena! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511963239000?text=Ol%C3%A1%2C%20Dra%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Helena%20Pires%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K27" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Helena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Helena Pires, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1654,20 +1464,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J28" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K28" t="str">
-        <v>R. Turiassu, n° 591 - Conj 25 - Perdizes, São Paulo - SP, 05005-001</v>
-      </c>
-      <c r="L28" t="str">
-        <v>https://wa.me/5511939011103?text=Ol%C3%A1%2C%20Dra%20Giovanna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Giovanna! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511939011103?text=Ol%C3%A1%2C%20Dra%20Giovanna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Giovanna%20Dourado%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K28" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Giovanna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Giovanna Dourado, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -1699,20 +1502,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J29" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K29" t="str">
-        <v>R. Piracuama, 280 - Perdizes, São Paulo - SP, 05017-040</v>
-      </c>
-      <c r="L29" t="str">
-        <v>https://wa.me/5511988877098?text=Ol%C3%A1%2C%20Dra.Leticia%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra.Leticia Morais! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511988877098?text=Ol%C3%A1%2C%20Dra.Leticia%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Leticia%20Morais%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K29" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra.Leticia Morais! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Leticia Morais, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -1744,20 +1540,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J30" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K30" t="str">
-        <v>R. João Ramalho, 1222 - Perdizes, São Paulo - SP, 05008-002</v>
-      </c>
-      <c r="L30" t="str">
-        <v>https://wa.me/5511996040673?text=Ol%C3%A1%2C%20Dra.%20Monique!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M30" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Monique! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511996040673?text=Ol%C3%A1%2C%20Dra.%20Monique!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Monique%20Fai%C3%A3o%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K30" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Monique! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Monique Faião, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -1789,20 +1578,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J31" t="str">
-        <v>https://www.instagram.com/dra.luanavieiraa?igsh=cGRzNHNpOTJ4MXkw&amp;utm_source=qr</v>
-      </c>
-      <c r="K31" t="str">
-        <v>R. Voluntários da Pátria, 654 - Sl 414 - Santana, São Paulo - SP, 02010-000</v>
-      </c>
-      <c r="L31" t="str">
-        <v>https://wa.me/5511978738749?text=Ol%C3%A1%2C%20Dentista%20Santana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Santana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M31" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista Santana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511978738749?text=Ol%C3%A1%2C%20Dentista%20Santana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20Santana%20-%20Dra%20Luana%20Vieira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K31" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dentista Santana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Santana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em Santana - Dra Luana Vieira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="32" xml:space="preserve">
@@ -1834,20 +1616,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J32" t="str">
-        <v>https://instagram.com/dralourdesspereira?igshid=MzRlODBiNWFlZA==</v>
-      </c>
-      <c r="K32" t="str">
-        <v>Escritório Santana - R. Dr. César, 1368 - Sl 508 - Santana, São Paulo - SP, 02013-004</v>
-      </c>
-      <c r="L32" t="str">
-        <v>https://wa.me/5511956566650?text=Ol%C3%A1%2C%20Odontologia%20%2FSa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Santana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M32" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontologia /Saúde! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511956566650?text=Ol%C3%A1%2C%20Odontologia%20%2FSa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontologia%20%2FSa%C3%BAde%20e%20bem%20estar%20Dra%20Lourdes%20S.Pereira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K32" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Odontologia /Saúde! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Santana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontologia /Saúde e bem estar Dra Lourdes S.Pereira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -1879,20 +1654,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J33" t="str">
-        <v>https://www.instagram.com/draluciana.dentista</v>
-      </c>
-      <c r="K33" t="str">
-        <v>R. Duarte de Azevedo, 431 - Sl 16 - Santana, São Paulo - SP, 02036-021</v>
-      </c>
-      <c r="L33" t="str">
-        <v>https://wa.me/5511993273559?text=Ol%C3%A1%2C%20Dra%20Luciana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Santana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M33" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Luciana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993273559?text=Ol%C3%A1%2C%20Dra%20Luciana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luciana%20Espejo%20%7C%20Dentista%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K33" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Luciana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Santana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luciana Espejo | Dentista em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -1924,20 +1692,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J34" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K34" t="str">
-        <v>R. Augusto Tolle, 767 - Conj 301 - Santana, São Paulo - SP, 02405-001</v>
-      </c>
-      <c r="L34" t="str">
-        <v>https://wa.me/5511991252211?text=Ol%C3%A1%2C%20Dra%20Alessandra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Santana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M34" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Alessandra! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511991252211?text=Ol%C3%A1%2C%20Dra%20Alessandra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Alessandra%20Parisi%20%7C%20Dentista%20%7C%20Santana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K34" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Alessandra! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Santana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Alessandra Parisi | Dentista | Santana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -1969,20 +1730,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J35" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K35" t="str">
-        <v>R. Voluntários da Pátria, 560 - Sl 304 - Santana, São Paulo - SP, 02011-000</v>
-      </c>
-      <c r="L35" t="str">
-        <v>https://wa.me/5511915333818?text=Ol%C3%A1%2C%20Dra.%20Thabata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Santana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M35" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Thabata! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511915333818?text=Ol%C3%A1%2C%20Dra.%20Thabata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra.%20Thabata%20L%C3%ADvia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K35" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Thabata! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Santana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra. Thabata Lívia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
@@ -2014,20 +1768,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J36" t="str">
-        <v>https://www.instagram.com/centroodontomorumbi/</v>
-      </c>
-      <c r="K36" t="str">
-        <v>Condomínio West Tower - centrodontomorumbi@centrodontomorumbi.com.br, Rua dos Três Irmãos, 62 - 1307 - Morumbi, São Paulo - SP, 05615-190</v>
-      </c>
-      <c r="L36" t="str">
-        <v>https://wa.me/5511966400022?text=Ol%C3%A1%2C%20Centro%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Morumbi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M36" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Centro Odontológico! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511966400022?text=Ol%C3%A1%2C%20Centro%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20Odontol%C3%B3gico%20Morumbi%20-%20Dra%20Renata%20Ramos%20e%20Equipe%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K36" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Centro Odontológico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Morumbi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro Odontológico Morumbi - Dra Renata Ramos e Equipe, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -2059,20 +1806,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J37" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K37" t="str">
-        <v>Rua Edward Joseph, 122 - Conj 82 - Morumbi, São Paulo - SP, 05709-020</v>
-      </c>
-      <c r="L37" t="str">
-        <v>https://wa.me/5511951307605?text=Ol%C3%A1%2C%20Dentista%20Morumbi%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Morumbi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista Morumbi,! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511951307605?text=Ol%C3%A1%2C%20Dentista%20Morumbi%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Morumbi%2C%20S%C3%A3o%20Paulo%20-%20Dra%20Larissa%20Tavares%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K37" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dentista Morumbi,! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Morumbi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Morumbi, São Paulo - Dra Larissa Tavares, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -2104,20 +1844,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J38" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K38" t="str">
-        <v>Rua dos Três Irmãos, 201 - Morumbi, São Paulo - SP, 05615-190</v>
-      </c>
-      <c r="L38" t="str">
-        <v>https://wa.me/5511959391155?text=Ol%C3%A1%2C%20Dr.%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Morumbi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M38" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. João! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511959391155?text=Ol%C3%A1%2C%20Dr.%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Dr.%20Jo%C3%A3o%20Vila%20-%20Morumbi%20-%20Vila%20Progredior%20-%20Jd%20Guedala%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K38" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dr. João! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Morumbi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Dr. João Vila - Morumbi - Vila Progredior - Jd Guedala, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -2149,20 +1882,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J39" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K39" t="str">
-        <v>Rua Dr. Luiz Migliano, 1986 - Parque Bairro Morumbi, São Paulo - SP, 05711-001</v>
-      </c>
-      <c r="L39" t="str">
-        <v>https://wa.me/5511958978174?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Morumbi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511958978174?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20S%C3%A3o%20Paulo%20-%20Dra%20Bruna%20Del%20Mestre%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K39" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,7★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Morumbi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em São Paulo - Dra Bruna Del Mestre, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -2194,20 +1920,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J40" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K40" t="str">
-        <v>Rua Dr. Luiz Migliano, 1986 - Vila Andrade, São Paulo - SP, 05711-001</v>
-      </c>
-      <c r="L40" t="str">
-        <v>https://wa.me/5511949420235?text=Ol%C3%A1%2C%20Dra.%20Tayna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Morumbi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M40" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Tayna! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511949420235?text=Ol%C3%A1%2C%20Dra.%20Tayna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Tayna%20Bastos%20%7C%20Dentista%20no%20Morumbi%20-%20S%C3%A3o%20Paulo%20%7C%20Pr%C3%B3tese%2C%20est%C3%A9tica%20e%20urg%C3%AAncia.%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K40" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Tayna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Morumbi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Tayna Bastos | Dentista no Morumbi - São Paulo | Prótese, estética e urgência., pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -2239,20 +1958,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J41" t="str">
-        <v>https://www.instagram.com/dra_mayaracardoso/</v>
-      </c>
-      <c r="K41" t="str">
-        <v>Av. Higienópolis, 195 - Higienópolis, São Paulo - SP, 01238-001</v>
-      </c>
-      <c r="L41" t="str">
-        <v>https://wa.me/5511947930542?text=Ol%C3%A1%2C%20Dra%20Mayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M41" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Mayara! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511947930542?text=Ol%C3%A1%2C%20Dra%20Mayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Mayara%20Cardoso%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K41" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Mayara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Mayara Cardoso, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -2284,20 +1996,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J42" t="str">
-        <v>https://www.doctoralia.com.br/nayara-freitas/dentista/sao-paulo</v>
-      </c>
-      <c r="K42" t="str">
-        <v>Av. Higienópolis, 195 - Higienópolis, São Paulo - SP, 01238-001</v>
-      </c>
-      <c r="L42" t="str">
-        <v>https://wa.me/5511972871378?text=Ol%C3%A1%2C%20Dra%20Nayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M42" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Nayara! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511972871378?text=Ol%C3%A1%2C%20Dra%20Nayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Nayara%20Freitas%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K42" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Nayara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Nayara Freitas, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="43" xml:space="preserve">
@@ -2329,20 +2034,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J43" t="str">
-        <v>https://www.instagram.com/dr.alexandrewon/</v>
-      </c>
-      <c r="K43" t="str">
-        <v>R. Martinico Prado, 167 - Sl 71 - Higienópolis, São Paulo - SP, 01224-011</v>
-      </c>
-      <c r="L43" t="str">
-        <v>https://wa.me/5511940696509?text=Ol%C3%A1%2C%20Won%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M43" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Won Odontologia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511940696509?text=Ol%C3%A1%2C%20Won%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Won%20Odontologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K43" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Won Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Won Odontologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
@@ -2374,20 +2072,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J44" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K44" t="str">
-        <v>R. Maranhão, 554 - Conj 63 - Higienópolis, São Paulo - SP, 01240-000</v>
-      </c>
-      <c r="L44" t="str">
-        <v>https://wa.me/5511945216642?text=Ol%C3%A1%2C%20Dr.%20Marcello!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M44" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. Marcello! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511945216642?text=Ol%C3%A1%2C%20Dr.%20Marcello!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Marcello%20Barone%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%20e%20Odontologia%20est%C3%A9tica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K44" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dr. Marcello! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Marcello Barone - Harmonização Orofacial e Odontologia estética, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
@@ -2419,20 +2110,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J45" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K45" t="str">
-        <v>R. Sabará, 566 - Higienópolis, São Paulo - SP, 01239-010</v>
-      </c>
-      <c r="L45" t="str">
-        <v>https://wa.me/5511998978621?text=Ol%C3%A1%2C%20Dra.%20Cecilia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M45" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Cecilia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511998978621?text=Ol%C3%A1%2C%20Dra.%20Cecilia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cecilia%20Sena%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K45" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Cecilia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cecilia Sena, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -2464,20 +2148,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J46" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K46" t="str">
-        <v>Av. Angélica, 501 - Conjunto 806 - Higienópolis, São Paulo - SP, 01228-200</v>
-      </c>
-      <c r="L46" t="str">
-        <v>https://wa.me/5511984157966?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511984157966?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Rodrigues%20Santos%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K46" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Rodrigues Santos, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -2509,20 +2186,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J47" t="str">
-        <v>https://instagram.com/drasilviaarruda?utm_medium=copy_link</v>
-      </c>
-      <c r="K47" t="str">
-        <v>R. Dona Antônia de Queirós, 549 - conj. 901 - Higienópolis, São Paulo - SP, 01307-014</v>
-      </c>
-      <c r="L47" t="str">
-        <v>https://wa.me/5511998439008?text=Ol%C3%A1%2C%20Dra%20Silvia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C3%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Odontologia%20no%20Google%20em%20Higien%C3%B3polis%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M47" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Silvia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511998439008?text=Ol%C3%A1%2C%20Dra%20Silvia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C3%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Silvia%20Gajardoni%20Arruda%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K47" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Silvia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 4,3★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Odontologia no Google em Higienópolis, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Silvia Gajardoni Arruda, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -2554,20 +2224,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J48" t="str">
-        <v>https://www.instagram.com/draraphaela.maia/</v>
-      </c>
-      <c r="K48" t="str">
-        <v>Alameda dos Nhambiquaras, 1770 - Sl 505 - Moema, São Paulo - SP, 04090-003</v>
-      </c>
-      <c r="L48" t="str">
-        <v>https://wa.me/5511993878167?text=Ol%C3%A1%2C%20Dra%20Raphaela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Raphaela! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993878167?text=Ol%C3%A1%2C%20Dra%20Raphaela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raphaela%20Maia%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20em%20Moema%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K48" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Raphaela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raphaela Maia - Harmonização Facial em Moema, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="49" xml:space="preserve">
@@ -2599,20 +2262,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J49" t="str">
-        <v>https://linktr.ee/drafeliramonteiro</v>
-      </c>
-      <c r="K49" t="str">
-        <v>Alameda dos Maracatins, 426 - Moema, São Paulo - SP, 04089-000</v>
-      </c>
-      <c r="L49" t="str">
-        <v>https://wa.me/5511988571847?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M49" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511988571847?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Lira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Zona%20Sul%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K49" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Lira | Harmonização Facial | Zona Sul São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -2644,20 +2300,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J50" t="str">
-        <v>https://www.instagram.com/dramendoncagabriela?igsh=MTE5MThiMGVhcXV2MQ==</v>
-      </c>
-      <c r="K50" t="str">
-        <v>R. Itapeva, 518 - 15º andar - Bela Vista, São Paulo - SP, 01332-000</v>
-      </c>
-      <c r="L50" t="str">
-        <v>https://wa.me/5511965850611?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M50" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511965850611?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Mendon%C3%A7a%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K50" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Mendonça - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">
@@ -2689,20 +2338,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J51" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K51" t="str">
-        <v>Av. Paulista, 2001 - Jardim Paulista, São Paulo - SP, 01311-931</v>
-      </c>
-      <c r="L51" t="str">
-        <v>https://wa.me/5511975815099?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Avan%C3%A7ada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M51" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Estética Avançada! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511975815099?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Avan%C3%A7ada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20AC%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K51" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Estética Avançada! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para AC Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="52" xml:space="preserve">
@@ -2734,20 +2376,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J52" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K52" t="str">
-        <v>Rua Peixoto Gomide, 219 - Conj. 102 Sala 108 - Jardim Paulista, São Paulo - SP, 01409-001</v>
-      </c>
-      <c r="L52" t="str">
-        <v>https://wa.me/5511958882681?text=Ol%C3%A1%2C%20Dra%20Fl%C3%A1via!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Flávia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511958882681?text=Ol%C3%A1%2C%20Dra%20Fl%C3%A1via!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Fl%C3%A1via%20Roma%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K52" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Flávia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Flávia Roma Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="53" xml:space="preserve">
@@ -2779,20 +2414,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J53" t="str">
-        <v>https://www.instagram.com/estetica_monicamuchante?igsh=M2syNWtzY2t3b3k4</v>
-      </c>
-      <c r="K53" t="str">
-        <v>Alameda Joaquim Eugênio de Lima, 1756 - Sl 1 - Jardim Paulista, São Paulo - SP, 01403-002</v>
-      </c>
-      <c r="L53" t="str">
-        <v>https://wa.me/5511951008872?text=Ol%C3%A1%2C%20Dra.%20M%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M53" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Mônica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511951008872?text=Ol%C3%A1%2C%20Dra.%20M%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20M%C3%B4nica%20Muchante%20Biom%C3%A9dica%20Esteta%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K53" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Mônica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Mônica Muchante Biomédica Esteta | Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="54" xml:space="preserve">
@@ -2824,20 +2452,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J54" t="str">
-        <v>https://www.instagram.com/dragiulianafranca/</v>
-      </c>
-      <c r="K54" t="str">
-        <v>Av. Paulista, 807 - Sl 816 - Bela Vista, São Paulo - SP, 01311-915</v>
-      </c>
-      <c r="L54" t="str">
-        <v>https://wa.me/5511977440161?text=Ol%C3%A1%2C%20Dra.%20Giuliana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M54" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Giuliana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511977440161?text=Ol%C3%A1%2C%20Dra.%20Giuliana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Giuliana%20Fran%C3%A7a%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K54" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Giuliana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Giuliana França Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="55" xml:space="preserve">
@@ -2869,20 +2490,13 @@
         <v>Sem site próprio (Apenas api)</v>
       </c>
       <c r="J55" t="str">
-        <v>https://api.whatsapp.com/message/CDJPK6KBGJXNE1?autoload=1&amp;app_absent=0</v>
-      </c>
-      <c r="K55" t="str">
-        <v>Av. Paulista, 1048 - Bela Vista, São Paulo - SP, 01310-100</v>
-      </c>
-      <c r="L55" t="str">
-        <v>https://wa.me/5511966291967?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M55" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511966291967?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Mello%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K55" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Mello | Estética Avançada SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="56" xml:space="preserve">
@@ -2914,20 +2528,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J56" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K56" t="str">
-        <v>R. Teodoro Sampaio, 2767 - 8° andar, Conj 82 - Pinheiros, São Paulo - SP, 05406-150</v>
-      </c>
-      <c r="L56" t="str">
-        <v>https://wa.me/5511952805419?text=Ol%C3%A1%2C%20Dra%20Leticia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Leticia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511952805419?text=Ol%C3%A1%2C%20Dra%20Leticia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Leticia%20Papp%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K56" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Leticia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Leticia Papp - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="57" xml:space="preserve">
@@ -2959,20 +2566,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J57" t="str">
-        <v>https://www.instagram.com/dra_amandaomartins/</v>
-      </c>
-      <c r="K57" t="str">
-        <v>R. Bela Cintra, 968 - conj 51 - Cerqueira César, São Paulo - SP, 01415-002</v>
-      </c>
-      <c r="L57" t="str">
-        <v>https://wa.me/5511975791298?text=Ol%C3%A1%2C%20Lemu%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M57" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Lemu Clinic! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511975791298?text=Ol%C3%A1%2C%20Lemu%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Lemu%20Clinic%20%7C%20Dra.%20Amanda%20Martins%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K57" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Lemu Clinic! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Lemu Clinic | Dra. Amanda Martins | Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="58" xml:space="preserve">
@@ -3004,20 +2604,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J58" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K58" t="str">
-        <v>Av. Paulista, 2064 - Cerqueira César, São Paulo - SP, 01310-200</v>
-      </c>
-      <c r="L58" t="str">
-        <v>https://wa.me/5511976971573?text=Ol%C3%A1%2C%20Dra%20Stephanie!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M58" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Stephanie! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976971573?text=Ol%C3%A1%2C%20Dra%20Stephanie!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Stephanie%20Milagre%20-%20Cl%C3%ADnica%20de%20est%C3%A9tica%20avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K58" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Stephanie! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Stephanie Milagre - Clínica de estética avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -3049,20 +2642,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J59" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K59" t="str">
-        <v>Av. Francisco Matarazzo, 229 - Conj. 58 - Água Branca, São Paulo - SP, 05001-000</v>
-      </c>
-      <c r="L59" t="str">
-        <v>https://wa.me/5511954537661?text=Ol%C3%A1%2C%20Dra%20Renata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Renata! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511954537661?text=Ol%C3%A1%2C%20Dra%20Renata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Renata%20Queiroz%20-%20Biomedicina%20Est%C3%A9tica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K59" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Renata! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Renata Queiroz - Biomedicina Estética, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="60" xml:space="preserve">
@@ -3094,20 +2680,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J60" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K60" t="str">
-        <v>Av. Angélica, 2491 - Conj 9 - Bela Vista, São Paulo - SP, 01227-200</v>
-      </c>
-      <c r="L60" t="str">
-        <v>https://wa.me/5511962612208?text=Ol%C3%A1%2C%20Nathalia%20Nastri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Nathalia Nastri! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511962612208?text=Ol%C3%A1%2C%20Nathalia%20Nastri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr%20Nathalia%20Nastri%20-%20Biomedicina%20Est%C3%A9tica-%20Pinheiros%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K60" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Nathalia Nastri! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr Nathalia Nastri - Biomedicina Estética- Pinheiros São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="61" xml:space="preserve">
@@ -3139,20 +2718,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J61" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K61" t="str">
-        <v>R. Joaquim Floriano, 820 - Itaim Bibi, São Paulo - SP, 04534-003</v>
-      </c>
-      <c r="L61" t="str">
-        <v>https://wa.me/5511914566745?text=Ol%C3%A1%2C%20Dra.Igma%20Araujo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M61" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra.Igma Araujo! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511914566745?text=Ol%C3%A1%2C%20Dra.Igma%20Araujo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Igma%20Araujo%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K61" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra.Igma Araujo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Igma Araujo | Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="62" xml:space="preserve">
@@ -3184,20 +2756,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J62" t="str">
-        <v>https://wa.me/5511988399169</v>
-      </c>
-      <c r="K62" t="str">
-        <v>R. Joaquim Floriano, 820 - 10 andar - Itaim Bibi, São Paulo - SP, 04534-003</v>
-      </c>
-      <c r="L62" t="str">
-        <v>https://wa.me/5511991646740?text=Ol%C3%A1%2C%20Dra%20Carmen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Carmen! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511991646740?text=Ol%C3%A1%2C%20Dra%20Carmen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carmen%20Barge%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Corporal%20%7C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K62" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Carmen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carmen Barge | Harmonização Facial e Corporal | São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="63" xml:space="preserve">
@@ -3229,20 +2794,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J63" t="str">
-        <v>https://www.instagram.com/dralaismarquesa/</v>
-      </c>
-      <c r="K63" t="str">
-        <v>R. Pedroso Alvarenga, 584 - Itaim Bibi, São Paulo - SP, 04531-001</v>
-      </c>
-      <c r="L63" t="str">
-        <v>https://wa.me/5511954742132?text=Ol%C3%A1%2C%20Dra.%20La%C3%ADs!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M63" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Laís! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511954742132?text=Ol%C3%A1%2C%20Dra.%20La%C3%ADs!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20La%C3%ADs%20Marques%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K63" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Laís! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Laís Marques - Harmonização Orofacial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="64" xml:space="preserve">
@@ -3274,20 +2832,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J64" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K64" t="str">
-        <v>Av. São Gabriel, 149 - Conj 1001 - Itaim Bibi, São Paulo - SP, 01435-001</v>
-      </c>
-      <c r="L64" t="str">
-        <v>https://wa.me/5511944625222?text=Ol%C3%A1%2C%20Clinica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M64" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clinica Estética! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511944625222?text=Ol%C3%A1%2C%20Clinica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Est%C3%A9tica-%20Elaine%20Vasconcelos-%20Harmoniza%C3%A7%C3%A3o%20Facial-%20Itaim%20Bibi%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K64" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clinica Estética! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Estética- Elaine Vasconcelos- Harmonização Facial- Itaim Bibi, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="65" xml:space="preserve">
@@ -3319,20 +2870,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J65" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K65" t="str">
-        <v>R. Fidêncio Ramos, 100 - 5 andar - Vila Olímpia, São Paulo - SP, 04551-010</v>
-      </c>
-      <c r="L65" t="str">
-        <v>https://wa.me/5511961662005?text=Ol%C3%A1%2C%20Dra.%20Alyne!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Alyne! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511961662005?text=Ol%C3%A1%2C%20Dra.%20Alyne!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Alyne%20Souza%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20-%20Vila%20Ol%C3%ADmpia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K65" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Alyne! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Alyne Souza | Harmonização Facial - Vila Olímpia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="66" xml:space="preserve">
@@ -3364,20 +2908,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J66" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K66" t="str">
-        <v>Trade Building - R. Funchal, 375 - And 1 - Sala 11 - Vila Olímpia, São Paulo - SP, 04551-060</v>
-      </c>
-      <c r="L66" t="str">
-        <v>https://wa.me/5511917440783?text=Ol%C3%A1%2C%20Dra.%20Thayn%C3%A1!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M66" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Thayná! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511917440783?text=Ol%C3%A1%2C%20Dra.%20Thayn%C3%A1!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Thayn%C3%A1%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K66" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Thayná! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Thayná Rosa | Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="67" xml:space="preserve">
@@ -3409,20 +2946,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J67" t="str">
-        <v>https://www.instagram.com/clinicabellalinea?igsh=MXVmMngxNm05aXdlZQ%3D%3D&amp;utm_source=qr</v>
-      </c>
-      <c r="K67" t="str">
-        <v>Rua Luís Góis, 832 - Mirandópolis, São Paulo - SP, 04043-050</v>
-      </c>
-      <c r="L67" t="str">
-        <v>https://wa.me/5511991236080?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Bella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M67" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Bella! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511991236080?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Bella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Bella%20Linea%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K67" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica Bella! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 4,7★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Bella Linea, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="68" xml:space="preserve">
@@ -3454,20 +2984,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J68" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K68" t="str">
-        <v>R. Domingos de Morais, 2781 - Conj 314 - Vila Mariana, São Paulo - SP, 04035-001</v>
-      </c>
-      <c r="L68" t="str">
-        <v>https://wa.me/5511992442685?text=Ol%C3%A1%2C%20Dra%20Raquel!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Raquel! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511992442685?text=Ol%C3%A1%2C%20Dra%20Raquel!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raquel%20Camargo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K68" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Raquel! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raquel Camargo - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="69" xml:space="preserve">
@@ -3499,20 +3022,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J69" t="str">
-        <v>https://wa.me/5511965833614</v>
-      </c>
-      <c r="K69" t="str">
-        <v>Rua Vergueiro, 2279 - Sl 913 - Vila Mariana, São Paulo - SP, 04101-100</v>
-      </c>
-      <c r="L69" t="str">
-        <v>https://wa.me/5511965833614?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M69" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511965833614?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Botox%20na%20Vila%20Mariana%20Dra.%20Bruna%20Ferreira%20Esteta%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K69" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Botox na Vila Mariana Dra. Bruna Ferreira Esteta, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="70" xml:space="preserve">
@@ -3544,20 +3060,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J70" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K70" t="str">
-        <v>R. Santa Cruz, 722 - Sl 410 - Vila Mariana, São Paulo - SP, 04122-000</v>
-      </c>
-      <c r="L70" t="str">
-        <v>https://wa.me/5511994003820?text=Ol%C3%A1%2C%20Nadia%20Ces%C3%A1rio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Nadia Cesário! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511994003820?text=Ol%C3%A1%2C%20Nadia%20Ces%C3%A1rio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nadia%20Ces%C3%A1rio%20-%20Est%C3%A9tica%20Especializada%20%7CDrenagem%20Linf%C3%A1tica%20Vila%20Mariana%20%7CLimpeza%20de%20pele%20%7CLipedema%7C%20P%C3%B3s%20Operat%C3%B3rio%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K70" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Nadia Cesário! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nadia Cesário - Estética Especializada |Drenagem Linfática Vila Mariana |Limpeza de pele |Lipedema| Pós Operatório, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="71" xml:space="preserve">
@@ -3589,20 +3098,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J71" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K71" t="str">
-        <v>R. Domingos de Morais, 2781 - Vila Mariana, São Paulo - SP, 04035-001</v>
-      </c>
-      <c r="L71" t="str">
-        <v>https://wa.me/5511999985553?text=Ol%C3%A1%2C%20Dra.%20Mage!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Mage! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511999985553?text=Ol%C3%A1%2C%20Dra.%20Mage!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Dra.%20Mage%20Mantovani%20Est%C3%A9tica%20Avan%C3%A7ada%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K71" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Mage! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Dra. Mage Mantovani Estética Avançada Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="72" xml:space="preserve">
@@ -3634,20 +3136,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J72" t="str">
-        <v>https://www.instagram.com/dra.amandarubio?igsh=MTI5NmJkZWU2d2VlMw==&amp;utm_source=qr</v>
-      </c>
-      <c r="K72" t="str">
-        <v>Rua Vergueiro, 2279 - Sl 913 - Vila Mariana, São Paulo - SP, 04101-100</v>
-      </c>
-      <c r="L72" t="str">
-        <v>https://wa.me/5511974771241?text=Ol%C3%A1%2C%20Dra%20Amanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Amanda! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511974771241?text=Ol%C3%A1%2C%20Dra%20Amanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Amanda%20Rubio%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K72" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Amanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Amanda Rubio - Harmonização Facial e Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -3679,20 +3174,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J73" t="str">
-        <v>https://wa.me//5511993736844?text=Ol%C3%A1!%20Encontrei%20no%20Google%20e%20quero%20saber%20mais.</v>
-      </c>
-      <c r="K73" t="str">
-        <v>Edifício Platina - R. Bom Sucesso, 220 - Sl 1210 – 12º andar - Tatuapé, São Paulo - SP, 03305-000</v>
-      </c>
-      <c r="L73" t="str">
-        <v>https://wa.me/5511993736844?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993736844?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Bruna%20Martinez%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K73" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Bruna Martinez - Harmonização Facial Tatuapé SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="74" xml:space="preserve">
@@ -3724,20 +3212,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J74" t="str">
-        <v>https://wa.me/message/CIUHJ3HBXIETA1</v>
-      </c>
-      <c r="K74" t="str">
-        <v>R. Cantagalo, 692 - Sl 714 - Vila Gomes Cardim, São Paulo - SP, 03319-000</v>
-      </c>
-      <c r="L74" t="str">
-        <v>https://wa.me/5511994073067?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M74" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511994073067?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Guimar%C3%A3es%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K74" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Guimarães Rosa | Harmonização Facial Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="75" xml:space="preserve">
@@ -3769,20 +3250,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J75" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K75" t="str">
-        <v>R. Padre Estevão Pernet, 160 - Tatuapé, São Paulo - SP, 03315-000</v>
-      </c>
-      <c r="L75" t="str">
-        <v>https://wa.me/5511953634975?text=Ol%C3%A1%2C%20Dra.%20Vit%C3%B3ria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Vitória! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511953634975?text=Ol%C3%A1%2C%20Dra.%20Vit%C3%B3ria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Vit%C3%B3ria%20Caldeira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K75" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Vitória! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Vitória Caldeira | Harmonização Facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="76" xml:space="preserve">
@@ -3814,20 +3288,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J76" t="str">
-        <v>https://wa.me/5511945950480</v>
-      </c>
-      <c r="K76" t="str">
-        <v>R. Cantagalo, 692 - Sl 1313 - Tatuapé, São Paulo - SP, 03319-000</v>
-      </c>
-      <c r="L76" t="str">
-        <v>https://wa.me/5511945950480?text=Ol%C3%A1%2C%20Dra.%20Gisele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M76" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Gisele! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511945950480?text=Ol%C3%A1%2C%20Dra.%20Gisele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Gisele%20Neves%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%20%7C%20Botox%20%7C%20Ultraformer%20%7C%20Sculptra%20%7C%20Radiesse%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K76" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Gisele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Gisele Neves - Harmonização Facial no Tatuapé | Botox | Ultraformer | Sculptra | Radiesse, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="77" xml:space="preserve">
@@ -3859,20 +3326,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J77" t="str">
-        <v>https://linktr.ee/dracarla.bocuto?fbclid=PAAabVkC7D5GvCg526Viljb7iD7leQoFXx5zYuUVFUNXw_8gCHOeAkCW2DXSw</v>
-      </c>
-      <c r="K77" t="str">
-        <v>R. Itapura, 239 - Vila Gomes Cardim, São Paulo - SP, 03310-000</v>
-      </c>
-      <c r="L77" t="str">
-        <v>https://wa.me/5511982885834?text=Ol%C3%A1%2C%20Dra%20Carla!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M77" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Carla! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511982885834?text=Ol%C3%A1%2C%20Dra%20Carla!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carla%20Bocuto%20Harmoniza%C3%A7%C3%A3o%20Natural%20-%20Botox%20Tatuap%C3%A9%2C%20Mind%20Est%C3%A9tica.%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K77" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Carla! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carla Bocuto Harmonização Natural - Botox Tatuapé, Mind Estética., pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="78" xml:space="preserve">
@@ -3904,20 +3364,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J78" t="str">
-        <v>https://www.instagram.com/dra.marinaferreira</v>
-      </c>
-      <c r="K78" t="str">
-        <v>R. Itapura, 239 - Vila Gomes Cardim, São Paulo - SP, 03310-000</v>
-      </c>
-      <c r="L78" t="str">
-        <v>https://wa.me/5511983714557?text=Ol%C3%A1%2C%20Dra.%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M78" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marina! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511983714557?text=Ol%C3%A1%2C%20Dra.%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marina%20Ferreira%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20%7C%20Tatuap%C3%A9%2FAn%C3%A1lia%20Franco%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K78" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Marina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marina Ferreira | Harmonização facial | Tatuapé/Anália Franco SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="79" xml:space="preserve">
@@ -3949,20 +3402,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J79" t="str">
-        <v>https://www.instagram.com/dra.leticiaforstner/</v>
-      </c>
-      <c r="K79" t="str">
-        <v>edificio ferrara - R. Padre Estevão Pernet, 718 - Sl 2504 - Tatuapé, São Paulo - SP, 03315-000</v>
-      </c>
-      <c r="L79" t="str">
-        <v>https://wa.me/5511963070502?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M79" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511963070502?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Forstner%20%7C%20Otomodela%C3%A7%C3%A3o%20%E2%80%A2%20Preenchimento%20Labial%20%E2%80%A2%20Botox%20%E2%80%A2%20Harmoniza%C3%A7%C3%A3o%20Facial%20%E2%80%93%20Tatuap%C3%A9%20SP%20%7C%20Line%20Skin%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K79" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Forstner | Otomodelação • Preenchimento Labial • Botox • Harmonização Facial – Tatuapé SP | Line Skin, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="80" xml:space="preserve">
@@ -3994,20 +3440,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J80" t="str">
-        <v>https://instagram.com/dra.carolinelopess?igshid=MzMyNGUyNmU2YQ==</v>
-      </c>
-      <c r="K80" t="str">
-        <v>R. Tijuco Preto, 393 - Sala 148 - Tatuapé, São Paulo - SP, 03316-000</v>
-      </c>
-      <c r="L80" t="str">
-        <v>https://wa.me/5511969170606?text=Ol%C3%A1%2C%20Dra.%20Caroline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M80" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Caroline! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511969170606?text=Ol%C3%A1%2C%20Dra.%20Caroline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Caroline%20Lopes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K80" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Caroline! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Caroline Lopes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="81" xml:space="preserve">
@@ -4039,20 +3478,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J81" t="str">
-        <v>https://www.instagram.com/dra.micheleneri?igsh=ajcyeXp0Nm1xM3Zk&amp;utm_source=qr</v>
-      </c>
-      <c r="K81" t="str">
-        <v>Rua Catiguá, 159 - Tatuapé, São Paulo - SP, 03065-030</v>
-      </c>
-      <c r="L81" t="str">
-        <v>https://wa.me/5511942945433?text=Ol%C3%A1%2C%20Dra.%20Michele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M81" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Michele! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511942945433?text=Ol%C3%A1%2C%20Dra.%20Michele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Michele%20Neri%20%E2%80%93%20Harmoniza%C3%A7%C3%A3o%20Facial%20%26%20Corporal%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K81" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Michele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Michele Neri – Harmonização Facial &amp; Corporal | Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="82" xml:space="preserve">
@@ -4084,20 +3516,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J82" t="str">
-        <v>http://www.instagram.com/draandressalopes</v>
-      </c>
-      <c r="K82" t="str">
-        <v>R. Vilela, 665 - 8º andar - Tatuapé, São Paulo - SP, 03314-000</v>
-      </c>
-      <c r="L82" t="str">
-        <v>https://wa.me/5511932253874?text=Ol%C3%A1%2C%20Dra%20Andressa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Andressa! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511932253874?text=Ol%C3%A1%2C%20Dra%20Andressa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Andressa%20Lopes%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K82" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Andressa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Andressa Lopes - Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="83" xml:space="preserve">
@@ -4129,20 +3554,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J83" t="str">
-        <v>https://www.instagram.com/drasuellenalbuquerque/</v>
-      </c>
-      <c r="K83" t="str">
-        <v>R. Apucarana, 272 - Sl 1004 - Vila Carrão, São Paulo - SP, 03311-000</v>
-      </c>
-      <c r="L83" t="str">
-        <v>https://wa.me/5511918467067?text=Ol%C3%A1%2C%20Dra%20Su%C3%A9llen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M83" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Suéllen! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511918467067?text=Ol%C3%A1%2C%20Dra%20Su%C3%A9llen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Su%C3%A9llen%20Albuquerque%20-%20Cl%C3%ADnica%20de%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K83" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Suéllen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Suéllen Albuquerque - Clínica de Harmonização Facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="84" xml:space="preserve">
@@ -4174,20 +3592,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J84" t="str">
-        <v>https://www.instagram.com/dratalita.trevisan/</v>
-      </c>
-      <c r="K84" t="str">
-        <v>R. Bom Sucesso, 220 - Tatuapé, São Paulo - SP, 03305-000</v>
-      </c>
-      <c r="L84" t="str">
-        <v>https://wa.me/5511913257440?text=Ol%C3%A1%2C%20Dra%20Talita!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M84" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Talita! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511913257440?text=Ol%C3%A1%2C%20Dra%20Talita!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Talita%20Trevisan%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K84" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Talita! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Talita Trevisan | Harmonização facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="85" xml:space="preserve">
@@ -4219,20 +3630,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J85" t="str">
-        <v>https://www.instagram.com/dragreicekelli?igsh=MWFicHZibDl6bjJ3dw%3D%3D&amp;utm_source=qr</v>
-      </c>
-      <c r="K85" t="str">
-        <v>R. Demétrio Ribeiro, 575 - Vila Reg. Feijó, São Paulo - SP, 03332-000</v>
-      </c>
-      <c r="L85" t="str">
-        <v>https://wa.me/5511999627447?text=Ol%C3%A1%2C%20Dra.%20Greice!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M85" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Greice! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511999627447?text=Ol%C3%A1%2C%20Dra.%20Greice!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Greice%20Keli-%20Est%C3%A9tica%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K85" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Greice! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Greice Keli- Estética e Harmonização Facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -4264,20 +3668,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J86" t="str">
-        <v>https://linktr.ee/dra.cristinaizabel.s</v>
-      </c>
-      <c r="K86" t="str">
-        <v>R. Padre Chico, no 85 - Perdizes, São Paulo - SP, 05008-010</v>
-      </c>
-      <c r="L86" t="str">
-        <v>https://wa.me/5511962892115?text=Ol%C3%A1%2C%20Dra.%20Cristina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M86" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Cristina! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511962892115?text=Ol%C3%A1%2C%20Dra.%20Cristina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cristina%20Silva%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K86" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Cristina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cristina Silva - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -4309,20 +3706,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J87" t="str">
-        <v>https://www.instagram.com/yvya_estetica/</v>
-      </c>
-      <c r="K87" t="str">
-        <v>Rua Bartira, 805 - Perdizes, São Paulo - SP, 05009-000</v>
-      </c>
-      <c r="L87" t="str">
-        <v>https://wa.me/5511975740970?text=Ol%C3%A1%2C%20YvYa%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M87" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, YvYa Clínica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511975740970?text=Ol%C3%A1%2C%20YvYa%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20YvYa%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20em%20Perdizes%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Limpeza%20de%20Pele%20%7C%20Preenchimento%20Facial%20%7C%20Ultrassom%20Microfocado%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K87" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, YvYa Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para YvYa Clínica de Estética em Perdizes | Harmonização Facial | Limpeza de Pele | Preenchimento Facial | Ultrassom Microfocado, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="88" xml:space="preserve">
@@ -4354,20 +3744,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J88" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K88" t="str">
-        <v>Rua Apinajés, 816 - Perdizes, São Paulo - SP, 05017-000</v>
-      </c>
-      <c r="L88" t="str">
-        <v>https://wa.me/5511913567195?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M88" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Estética! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511913567195?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20avan%C3%A7ada%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K88" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica Estética! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Estética avançada Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="89" xml:space="preserve">
@@ -4399,20 +3782,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J89" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K89" t="str">
-        <v>In Office - R. Min. Ferreira Alves, 97 - Sl 301 Ed - Perdizes, São Paulo - SP, 05009-060</v>
-      </c>
-      <c r="L89" t="str">
-        <v>https://wa.me/5511914800366?text=Ol%C3%A1%2C%20FIG%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M89" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, FIG Clinic! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511914800366?text=Ol%C3%A1%2C%20FIG%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20FIG%20Clinic%20-%20Dra.%20Manuela%20de%20Souza%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K89" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, FIG Clinic! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para FIG Clinic - Dra. Manuela de Souza, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -4444,20 +3820,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J90" t="str">
-        <v>https://www.instagram.com/dramadigiacomo?igsh=MTQzcHJnaXMxYnpiMQ==&amp;utm_source=qr</v>
-      </c>
-      <c r="K90" t="str">
-        <v>Av. Antártica, 675 - 19º andar - Água Branca, São Paulo - SP, 05003-020</v>
-      </c>
-      <c r="L90" t="str">
-        <v>https://wa.me/5511972848524?text=Ol%C3%A1%2C%20Dra.%20Marcela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M90" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marcela! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511972848524?text=Ol%C3%A1%2C%20Dra.%20Marcela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcela%20Di%20Giacomo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K90" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Marcela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcela Di Giacomo - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="91" xml:space="preserve">
@@ -4489,20 +3858,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J91" t="str">
-        <v>https://www.instagram.com/dra.clairpessoa/</v>
-      </c>
-      <c r="K91" t="str">
-        <v>Av. Antártica, 675 - 19° andar - Perdizes, São Paulo - SP, 05003-020</v>
-      </c>
-      <c r="L91" t="str">
-        <v>https://wa.me/5511954221740?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Facial!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M91" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Estética Facial! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511954221740?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Facial!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Est%C3%A9tica%20Facial%20%26%20Rejuvenescimento%20%7C%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K91" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Estética Facial! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Estética Facial &amp; Rejuvenescimento | Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="92" xml:space="preserve">
@@ -4534,20 +3896,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J92" t="str">
-        <v>https://www.doctoralia.com.br/ana-regina-alencar-santos/dermatologista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=50473&amp;utm_content=website</v>
-      </c>
-      <c r="K92" t="str">
-        <v>Av. Ibirapuera, 2907 - 2 andar - Conjunto 223 - Moema, São Paulo - SP, 04029-200</v>
-      </c>
-      <c r="L92" t="str">
-        <v>https://wa.me/5511960447173?text=Ol%C3%A1%2C%20Dra.%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C2%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M92" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Ana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511960447173?text=Ol%C3%A1%2C%20Dra.%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C2%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Ana%20Regina%20Alencar%20Santos%2C%20Dermatologista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K92" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Ana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,2★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Ana Regina Alencar Santos, Dermatologista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="93" xml:space="preserve">
@@ -4579,20 +3934,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J93" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K93" t="str">
-        <v>R. Min. Gabriel de Rezende Passos, 500 - 9º andar - Moema, São Paulo - SP, 04521-022</v>
-      </c>
-      <c r="L93" t="str">
-        <v>https://wa.me/5511910324225?text=Ol%C3%A1%2C%20Dra%20Elisabeth!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M93" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Elisabeth! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511910324225?text=Ol%C3%A1%2C%20Dra%20Elisabeth!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Elisabeth%20Silveira%20-%20Dermatologia%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K93" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Elisabeth! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Elisabeth Silveira - Dermatologia em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="94" xml:space="preserve">
@@ -4624,20 +3972,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J94" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K94" t="str">
-        <v>R. Graúna, 315 - Moema, São Paulo - SP, 04514-001</v>
-      </c>
-      <c r="L94" t="str">
-        <v>https://wa.me/5511993053569?text=Ol%C3%A1%2C%20Fernanda%20Lima!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M94" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Fernanda Lima! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993053569?text=Ol%C3%A1%2C%20Fernanda%20Lima!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Lima%20Queiroz%20Noya%20de%20Abreu%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K94" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Fernanda Lima! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Estética &amp; Harmonização no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Lima Queiroz Noya de Abreu, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="95" xml:space="preserve">
@@ -4669,20 +4010,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J95" t="str">
-        <v>https://www.instagram.com/nutri.malubraidotti/</v>
-      </c>
-      <c r="K95" t="str">
-        <v>Av. Rouxinol, 84 - Moema, São Paulo - SP, 04516-000</v>
-      </c>
-      <c r="L95" t="str">
-        <v>https://wa.me/5511945167295?text=Ol%C3%A1%2C%20Malu!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M95" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Malu! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511945167295?text=Ol%C3%A1%2C%20Malu!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Malu%20Braidotti%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K95" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Malu! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Malu Braidotti, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="96" xml:space="preserve">
@@ -4714,20 +4048,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J96" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K96" t="str">
-        <v>Av. Rouxinol, 55 - Sl 104 - Moema, São Paulo - SP, 04516-000</v>
-      </c>
-      <c r="L96" t="str">
-        <v>https://wa.me/5511937287838?text=Ol%C3%A1%2C%20Centro%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M96" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Centro Nutrição! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511937287838?text=Ol%C3%A1%2C%20Centro%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20de%20Nutri%C3%A7%C3%A3o%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K96" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Centro Nutrição! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro de Nutrição, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="97" xml:space="preserve">
@@ -4759,20 +4086,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J97" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K97" t="str">
-        <v>Av. Rouxinol, 84 - 67 - Moema, São Paulo - SP, 04516-000</v>
-      </c>
-      <c r="L97" t="str">
-        <v>https://wa.me/5511997196772?text=Ol%C3%A1%2C%20Nutri%C3%A7%C3%A3o%20Personalizada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M97" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Nutrição Personalizada! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511997196772?text=Ol%C3%A1%2C%20Nutri%C3%A7%C3%A3o%20Personalizada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutri%C3%A7%C3%A3o%20Personalizada%20-%20Dra%20Fab%C3%ADola%20Estela%20Domingues%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K97" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Nutrição Personalizada! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutrição Personalizada - Dra Fabíola Estela Domingues, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="98" xml:space="preserve">
@@ -4804,20 +4124,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J98" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K98" t="str">
-        <v>R. Américo Brasiliense, 1765 - Conj 43-44 - Granja Julieta, São Paulo - SP, 04715-000</v>
-      </c>
-      <c r="L98" t="str">
-        <v>https://wa.me/5511985928451?text=Ol%C3%A1%2C%20Esportivo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M98" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Esportivo! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511985928451?text=Ol%C3%A1%2C%20Esportivo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportivo%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K98" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Esportivo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportivo em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="99" xml:space="preserve">
@@ -4849,20 +4162,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J99" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K99" t="str">
-        <v>Av. Rouxinol, 84 - 2° Andar, cj 27 - Moema, São Paulo - SP, 04516-000</v>
-      </c>
-      <c r="L99" t="str">
-        <v>https://wa.me/5511974981031?text=Ol%C3%A1%2C%20Wesen%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C1%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M99" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Wesen Clínica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511974981031?text=Ol%C3%A1%2C%20Wesen%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C1%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Wesen%20Cl%C3%ADnica%20de%20Emagrecimento%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K99" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Wesen Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 4,1★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Wesen Clínica de Emagrecimento, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="100" xml:space="preserve">
@@ -4894,20 +4200,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J100" t="str">
-        <v>https://www.instagram.com/larissafranco.nutri?igsh=MTE1MGZjenZvY3g3cw%3D%3D&amp;utm_source=qr</v>
-      </c>
-      <c r="K100" t="str">
-        <v>Av. Rebouças, 499 - Conj 605 - Jardins, São Paulo - SP, 05401-050</v>
-      </c>
-      <c r="L100" t="str">
-        <v>https://wa.me/5511988957410?text=Ol%C3%A1%2C%20Larissa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Larissa! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511988957410?text=Ol%C3%A1%2C%20Larissa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Larissa%20Franco%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K100" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Larissa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Larissa Franco, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="101" xml:space="preserve">
@@ -4939,20 +4238,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J101" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K101" t="str">
-        <v>R. Bento de Andrade, 598 - Jardim Paulista, São Paulo - SP, 04503-001</v>
-      </c>
-      <c r="L101" t="str">
-        <v>https://wa.me/5511922183012?text=Ol%C3%A1%2C%20Larissa%20Monteiro!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Larissa Monteiro! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511922183012?text=Ol%C3%A1%2C%20Larissa%20Monteiro!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Larissa%20Monteiro%20Nutricionista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K101" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Larissa Monteiro! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Larissa Monteiro Nutricionista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="102" xml:space="preserve">
@@ -4984,20 +4276,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J102" t="str">
-        <v>https://www.instagram.com/nathalia.nutri/</v>
-      </c>
-      <c r="K102" t="str">
-        <v>Alameda Gabriel Monteiro da Silva, 429 - Jardim America, São Paulo - SP, 01441-000</v>
-      </c>
-      <c r="L102" t="str">
-        <v>https://wa.me/5511976575363?text=Ol%C3%A1%2C%20nos!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M102" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, nos! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976575363?text=Ol%C3%A1%2C%20nos!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20nos%20Jardins%20-%20Nath%C3%A1lia%20D'Abruzzo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K102" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, nos! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista nos Jardins - Nathália D'Abruzzo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="103" xml:space="preserve">
@@ -5029,20 +4314,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J103" t="str">
-        <v>https://www.doctoralia.com.br/marisa-graca/nutricionista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=705957&amp;utm_content=website</v>
-      </c>
-      <c r="K103" t="str">
-        <v>R. Cincinato Braga, 37 - Conj 51 - Bela Vista, São Paulo - SP, 01333-011</v>
-      </c>
-      <c r="L103" t="str">
-        <v>https://wa.me/5511934427007?text=Ol%C3%A1%2C%20Dra.%20Marisa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M103" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marisa! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511934427007?text=Ol%C3%A1%2C%20Dra.%20Marisa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marisa%20Diniz%20Gra%C3%A7a%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K103" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra. Marisa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marisa Diniz Graça, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="104" xml:space="preserve">
@@ -5074,20 +4352,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J104" t="str">
-        <v>https://wa.me/5511921795550?text=Ol%C3%A1!%20Vim%20pelo%20Google%20e%20gostaria%20de%20mais%20informa%C3%A7%C3%B5es%20sobre%20a%20consulta%20nutricional!</v>
-      </c>
-      <c r="K104" t="str">
-        <v>Rua Tabapuã, 888 - Itaim Bibi, São Paulo - SP, 04533-002</v>
-      </c>
-      <c r="L104" t="str">
-        <v>https://wa.me/5511921795550?text=Ol%C3%A1%2C%20Rafael%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M104" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Rafael Morais! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511921795550?text=Ol%C3%A1%2C%20Rafael%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Rafael%20Morais%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K104" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Rafael Morais! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Rafael Morais, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="105" xml:space="preserve">
@@ -5119,20 +4390,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J105" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K105" t="str">
-        <v>R. Comendador Miguel Calfat, 128 - Sl 210 - Itaim Bibi, São Paulo - SP, 04537-080</v>
-      </c>
-      <c r="L105" t="str">
-        <v>https://wa.me/5511980982327?text=Ol%C3%A1%2C%20Dra%20Daniela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M105" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Daniela! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511980982327?text=Ol%C3%A1%2C%20Dra%20Daniela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Daniela%20Mendon%C3%A7a%20-%20Nutricionista%20Esportiva%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K105" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Daniela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Daniela Mendonça - Nutricionista Esportiva, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="106" xml:space="preserve">
@@ -5164,20 +4428,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J106" t="str">
-        <v>https://wa.me/5511964236252</v>
-      </c>
-      <c r="K106" t="str">
-        <v>Rua Urussuí, 92 - Conj 91 - Itaim Bibi, São Paulo - SP, 04542-050</v>
-      </c>
-      <c r="L106" t="str">
-        <v>https://wa.me/5511964236252?text=Ol%C3%A1%2C%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M106" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, João! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511964236252?text=Ol%C3%A1%2C%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Jo%C3%A3o%20Pinheiro%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K106" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, João! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista João Pinheiro, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="107" xml:space="preserve">
@@ -5209,20 +4466,13 @@
         <v>Sem site próprio (Apenas api)</v>
       </c>
       <c r="J107" t="str">
-        <v>https://api.whatsapp.com/send?phone=5511981267772&amp;text=Ol%C3%A1%2C%20Andrea!%20Te%20encontrei%20no%20Google%20e%20gostaria%20de%20mais%20informa%C3%A7%C3%B5es%20sobre%20a%20consulta%20com%20voc%C3%AA.%20Obrigado.</v>
-      </c>
-      <c r="K107" t="str">
-        <v>Rua Tabapuã, 111 - CJ 51-52 - Itaim Bibi, São Paulo - SP, 04533-010</v>
-      </c>
-      <c r="L107" t="str">
-        <v>https://wa.me/5511981267772?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M107" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511981267772?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Andrea%20Garrett%20Nutricionista%20no%20Itaim%20Bibi%20CRN3%2090979%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K107" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Andrea Garrett Nutricionista no Itaim Bibi CRN3 90979, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="108" xml:space="preserve">
@@ -5254,20 +4504,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J108" t="str">
-        <v>https://www.instagram.com/nutricionistaveronicanovais/</v>
-      </c>
-      <c r="K108" t="str">
-        <v>Edifício Thera Faria Lima, R. Amaro Cavalheiro, 347 - conjunto 913 - Pinheiros, São Paulo - SP, 05425-011</v>
-      </c>
-      <c r="L108" t="str">
-        <v>https://wa.me/5511952251414?text=Ol%C3%A1%2C%20Ver%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M108" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Verônica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511952251414?text=Ol%C3%A1%2C%20Ver%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ver%C3%B4nica%20Novais%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K108" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Verônica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Verônica Novais, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="109" xml:space="preserve">
@@ -5299,20 +4542,13 @@
         <v>Sem site próprio (Apenas api)</v>
       </c>
       <c r="J109" t="str">
-        <v>https://api.whatsapp.com/send?phone=5511972163767</v>
-      </c>
-      <c r="K109" t="str">
-        <v>Av. Brig. Faria Lima, 1461 - Pinheiros, São Paulo - SP, 01452-002</v>
-      </c>
-      <c r="L109" t="str">
-        <v>https://wa.me/5511972163767?text=Ol%C3%A1%2C%20Yuri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M109" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Yuri! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511972163767?text=Ol%C3%A1%2C%20Yuri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Yuri%20Gomes%20-%20Nutricionista%20Esportivo%20em%20Pinheiros%2C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K109" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Yuri! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Yuri Gomes - Nutricionista Esportivo em Pinheiros, São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="110" xml:space="preserve">
@@ -5344,20 +4580,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J110" t="str">
-        <v>https://www.doctoralia.com.br/ellen-cortezi/nutricionista/sao-paulo</v>
-      </c>
-      <c r="K110" t="str">
-        <v>R. Cônego Eugênio Leite, 1166 - Pinheiros, São Paulo - SP, 05414-001</v>
-      </c>
-      <c r="L110" t="str">
-        <v>https://wa.me/5511971308828?text=Ol%C3%A1%2C%20Ellen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M110" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Ellen! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511971308828?text=Ol%C3%A1%2C%20Ellen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ellen%20Hiromi%20Cortezi%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K110" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Ellen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Ellen Hiromi Cortezi, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="111" xml:space="preserve">
@@ -5389,20 +4618,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J111" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K111" t="str">
-        <v>R. Pais Leme, 215 - Pinheiros, São Paulo - SP, 05424-150</v>
-      </c>
-      <c r="L111" t="str">
-        <v>https://wa.me/5511982923609?text=Ol%C3%A1%2C%20Aline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M111" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Aline! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511982923609?text=Ol%C3%A1%2C%20Aline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Aline%20Rodrigues%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K111" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Aline! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Aline Rodrigues, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="112" xml:space="preserve">
@@ -5434,20 +4656,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J112" t="str">
-        <v>https://www.instagram.com/mayrachamas?igsh=MXN2M2xyeXB4Z28xcw%3D%3D&amp;utm_source=qr</v>
-      </c>
-      <c r="K112" t="str">
-        <v>Thera Office Faria Lima - R. Pais Leme, 215 - Pinheiros, São Paulo - SP, 05424-150</v>
-      </c>
-      <c r="L112" t="str">
-        <v>https://wa.me/5511995262251?text=Ol%C3%A1%2C%20Mayra%20Chamas!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M112" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Mayra Chamas! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511995262251?text=Ol%C3%A1%2C%20Mayra%20Chamas!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mayra%20Chamas%20Nutricionista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K112" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Mayra Chamas! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mayra Chamas Nutricionista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="113" xml:space="preserve">
@@ -5479,20 +4694,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J113" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K113" t="str">
-        <v>R. Domingos de Morais, 2781 - Vila Mariana, São Paulo - SP, 04035-001</v>
-      </c>
-      <c r="L113" t="str">
-        <v>https://wa.me/5511948082545?text=Ol%C3%A1%2C%20Mariana%20Sena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M113" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Mariana Sena! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511948082545?text=Ol%C3%A1%2C%20Mariana%20Sena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Sena%20-%20Nutricionista%20Cl%C3%ADnica%20Funcional%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K113" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Mariana Sena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Sena - Nutricionista Clínica Funcional, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="114" xml:space="preserve">
@@ -5524,20 +4732,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J114" t="str">
-        <v>https://www.instagram.com/nutri_primazza/?hl=pt-br</v>
-      </c>
-      <c r="K114" t="str">
-        <v>Rua: Baltazar Lisboa, 322 - Vila Mariana, São Paulo - SP, 04110-061</v>
-      </c>
-      <c r="L114" t="str">
-        <v>https://wa.me/5511996792653?text=Ol%C3%A1%2C%20Vegetariana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M114" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Vegetariana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511996792653?text=Ol%C3%A1%2C%20Vegetariana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Vegetariana%2F%20Vegana%20Priscilla%20Mazza%20(Vila%20Mariana)%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K114" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Vegetariana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Vegetariana/ Vegana Priscilla Mazza (Vila Mariana), pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="115" xml:space="preserve">
@@ -5569,20 +4770,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J115" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K115" t="str">
-        <v>R. Domingos de Morais, 2781 - 14º andar - Vila Mariana, São Paulo - SP, 04035-001</v>
-      </c>
-      <c r="L115" t="str">
-        <v>https://wa.me/5511942228782?text=Ol%C3%A1%2C%20Priscila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M115" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Priscila! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511942228782?text=Ol%C3%A1%2C%20Priscila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Priscila%20Raso%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K115" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Priscila! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Priscila Raso, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="116" xml:space="preserve">
@@ -5614,20 +4808,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J116" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K116" t="str">
-        <v>R. Domingos de Morais, 348 - Vila Mariana, São Paulo - SP, 04011-000</v>
-      </c>
-      <c r="L116" t="str">
-        <v>https://wa.me/5511947936739?text=Ol%C3%A1%2C%20Camila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M116" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Camila! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511947936739?text=Ol%C3%A1%2C%20Camila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Camila%20Hidani%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K116" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Camila! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Camila Hidani, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="117" xml:space="preserve">
@@ -5659,20 +4846,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J117" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K117" t="str">
-        <v>R. Agostinho Rodrigues Filho, 550 - Vila Mariana, São Paulo - SP, 04026-040</v>
-      </c>
-      <c r="L117" t="str">
-        <v>https://wa.me/5511989456640?text=Ol%C3%A1%2C%20Dra%20Pollana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M117" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Pollana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511989456640?text=Ol%C3%A1%2C%20Dra%20Pollana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Pollana%20Campos%20Moreira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K117" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra Pollana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Pollana Campos Moreira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="118" xml:space="preserve">
@@ -5704,20 +4884,13 @@
         <v>Sem site próprio (Apenas wixsite)</v>
       </c>
       <c r="J118" t="str">
-        <v>https://julianagasulla.wixsite.com/nutricao</v>
-      </c>
-      <c r="K118" t="str">
-        <v>Rua Soriano de Sousa, 189 - Tatuapé, São Paulo - SP, 03066-020</v>
-      </c>
-      <c r="L118" t="str">
-        <v>https://wa.me/5511975438419?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M118" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Esportiva! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511975438419?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportiva%20Tatuap%C3%A9%20-%20Juliana%20Gasulla%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K118" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Esportiva! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportiva Tatuapé - Juliana Gasulla, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="119" xml:space="preserve">
@@ -5749,20 +4922,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J119" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K119" t="str">
-        <v>Rua Catiguá, 159 - Tatuapé, São Paulo - SP, 03065-030</v>
-      </c>
-      <c r="L119" t="str">
-        <v>https://wa.me/5511950262944?text=Ol%C3%A1%2C%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M119" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511950262944?text=Ol%C3%A1%2C%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Cl%C3%ADnica%20e%20Esportiva%20-%20Mariana%20Saito%20-%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K119" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Clínica e Esportiva - Mariana Saito - Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="120" xml:space="preserve">
@@ -5794,20 +4960,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J120" t="str">
-        <v>https://instagram.com/nutrijessicanogueira?r=nametag</v>
-      </c>
-      <c r="K120" t="str">
-        <v>Condomínio Higgs Empresarial - R. Serra de Botucatu, 880 - Sl 201 - Tatuapé, São Paulo - SP, 03317-000</v>
-      </c>
-      <c r="L120" t="str">
-        <v>https://wa.me/5511940152184?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M120" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511940152184?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20no%20Tatuap%C3%A9%20%7C%20J%C3%A9ssica%20Nogueira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K120" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista no Tatuapé | Jéssica Nogueira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="121" xml:space="preserve">
@@ -5839,20 +4998,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J121" t="str">
-        <v>https://wa.me/message/5PEST3D4ANFQB1</v>
-      </c>
-      <c r="K121" t="str">
-        <v>R. Itapura, 239 - Vila Gomes Cardim, São Paulo - SP, 03310-000</v>
-      </c>
-      <c r="L121" t="str">
-        <v>https://wa.me/5511976671105?text=Ol%C3%A1%2C%20Jessica%20Nascimento!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M121" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Jessica Nascimento! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976671105?text=Ol%C3%A1%2C%20Jessica%20Nascimento!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Jessica%20Nascimento%20%7C%20Nutricionista%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K121" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Jessica Nascimento! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Jessica Nascimento | Nutricionista Tatuapé SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="122" xml:space="preserve">
@@ -5884,20 +5036,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J122" t="str">
-        <v>https://www.instagram.com/nutrijulialinhares/</v>
-      </c>
-      <c r="K122" t="str">
-        <v>R. Vilela, 665 - Tatuapé, São Paulo - SP, 03314-000</v>
-      </c>
-      <c r="L122" t="str">
-        <v>https://wa.me/5511933768718?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M122" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Julia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511933768718?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Julia%20Linhares%20-%20Cl%C3%ADnica%20e%20Esportiva%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K122" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Julia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Julia Linhares - Clínica e Esportiva, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="123" xml:space="preserve">
@@ -5929,20 +5074,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J123" t="str">
-        <v>https://www.doctoralia.com.br/susan-franca-guimaraes/nutricionista/sao-paulo</v>
-      </c>
-      <c r="K123" t="str">
-        <v>R. Serra de Juréa, 396 - Tatuapé, São Paulo - SP, 03323-020</v>
-      </c>
-      <c r="L123" t="str">
-        <v>https://wa.me/5511993881567?text=Ol%C3%A1%2C%20Tatuap%C3%A9!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M123" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Tatuapé! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993881567?text=Ol%C3%A1%2C%20Tatuap%C3%A9!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Tatuap%C3%A9%20%7C%20Susan%20Fran%C3%A7a%20Guimar%C3%A3es%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K123" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Tatuapé! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 4,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Tatuapé | Susan França Guimarães, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="124" xml:space="preserve">
@@ -5974,20 +5112,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J124" t="str">
-        <v>http://linktr.ee/victorpiekny</v>
-      </c>
-      <c r="K124" t="str">
-        <v>R. Restinga, 113 - Tatuapé, São Paulo - SP, 03065-020</v>
-      </c>
-      <c r="L124" t="str">
-        <v>https://wa.me/5511942591826?text=Ol%C3%A1%2C%20Victor!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M124" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Victor! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511942591826?text=Ol%C3%A1%2C%20Victor!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Victor%20Piekny%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K124" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Victor! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Victor Piekny, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="125" xml:space="preserve">
@@ -6019,20 +5150,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J125" t="str">
-        <v>http://instagram.com/nutri.bruantonietti</v>
-      </c>
-      <c r="K125" t="str">
-        <v>R. Vilela, 652 - Tatuapé, São Paulo - SP, 03314-000</v>
-      </c>
-      <c r="L125" t="str">
-        <v>https://wa.me/5511951573284?text=Ol%C3%A1%2C%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M125" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Bruna! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511951573284?text=Ol%C3%A1%2C%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Bruna%20Antonietti%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K125" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Bruna Antonietti, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="126" xml:space="preserve">
@@ -6064,20 +5188,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J126" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K126" t="str">
-        <v>Rua Apinajés, 1.100 - Conj 301A - Perdizes, São Paulo - SP, 05017-000</v>
-      </c>
-      <c r="L126" t="str">
-        <v>https://wa.me/5511976893728?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M126" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Nutrição! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511976893728?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Nutri%C3%A7%C3%A3o%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K126" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica Nutrição! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Nutrição Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="127" xml:space="preserve">
@@ -6109,20 +5226,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J127" t="str">
-        <v>https://instagram.com/monicaunzueta.nutri?igshid=1glrwzy5tmocd</v>
-      </c>
-      <c r="K127" t="str">
-        <v>R. Monte Alegre, 428 - Perdizes, São Paulo - SP, 05019-010</v>
-      </c>
-      <c r="L127" t="str">
-        <v>https://wa.me/5511932300359?text=Ol%C3%A1%2C%20Emagrecimento%20Sa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M127" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Emagrecimento Saúde! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511932300359?text=Ol%C3%A1%2C%20Emagrecimento%20Sa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Emagrecimento%20e%20Sa%C3%BAde%20da%20Mulher%2035%2B%20%7C%20Nutricionista%20Monica%20Valeria%20Palenque%20Unzueta%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K127" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Emagrecimento Saúde! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Emagrecimento e Saúde da Mulher 35+ | Nutricionista Monica Valeria Palenque Unzueta, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="128" xml:space="preserve">
@@ -6154,20 +5264,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J128" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K128" t="str">
-        <v>Rua Federação Paulista de Futebol, 799 - Ed. Top Office Tower - Conj 1107/1108 - Barra Funda, São Paulo - SP, 01141-040</v>
-      </c>
-      <c r="L128" t="str">
-        <v>https://wa.me/5511916477655?text=Ol%C3%A1%2C%20Dra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M128" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511916477655?text=Ol%C3%A1%2C%20Dra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Dra%20Patr%C3%ADcia%20Neri%20Cavalcanti%20%7C%20Transformo%20a%20Sa%C3%BAde%20de%20Mulheres%20com%20Ci%C3%AAncia%20e%20Acolhimento.%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K128" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Dra! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Dra Patrícia Neri Cavalcanti | Transformo a Saúde de Mulheres com Ciência e Acolhimento., pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -6199,20 +5302,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J129" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K129" t="str">
-        <v>R. Palestra Itália, 73 - Conj 147 - Perdizes, São Paulo - SP, 05005-000</v>
-      </c>
-      <c r="L129" t="str">
-        <v>https://wa.me/5511992192552?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M129" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Esportiva! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511992192552?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Camila%20Moreira%20Nutricionista%20Esportiva%20Funcional%20-%20Cl%C3%ADnica%20Endocor%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K129" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Esportiva! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Camila Moreira Nutricionista Esportiva Funcional - Clínica Endocor, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="130" xml:space="preserve">
@@ -6244,20 +5340,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J130" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K130" t="str">
-        <v>R. Monte Alegre, 428 - Conj 26 - Perdizes, São Paulo - SP, 05014-000</v>
-      </c>
-      <c r="L130" t="str">
-        <v>https://wa.me/5511932613077?text=Ol%C3%A1%2C%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Nutri%C3%A7%C3%A3o%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M130" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Helena! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511932613077?text=Ol%C3%A1%2C%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Helena%20Fioravanti%20%7C%20Nutricionista%20em%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K130" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Helena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Nutrição no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Helena Fioravanti | Nutricionista em Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="131" xml:space="preserve">
@@ -6289,20 +5378,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J131" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K131" t="str">
-        <v>Av. Francisco Matarazzo - Água Branca, São Paulo - SP, 05003-020</v>
-      </c>
-      <c r="L131" t="str">
-        <v>https://wa.me/5511972437354?text=Ol%C3%A1%2C%20Psi%20Yara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M131" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Psi Yara! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511972437354?text=Ol%C3%A1%2C%20Psi%20Yara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psi%20Yara%20Rodrigues%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K131" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Psi Yara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psi Yara Rodrigues, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="132" xml:space="preserve">
@@ -6334,20 +5416,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J132" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K132" t="str">
-        <v>Rua Tuim, 380 - 2° andar - Moema, São Paulo - SP, 04514-100</v>
-      </c>
-      <c r="L132" t="str">
-        <v>https://wa.me/5511995828384?text=Ol%C3%A1%2C%20Luciane%20Bonfanti!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M132" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Luciane Bonfanti! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511995828384?text=Ol%C3%A1%2C%20Luciane%20Bonfanti!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Luciane%20Bonfanti%20%7C%20Psic%C3%B3loga%20em%20Moema%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K132" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Luciane Bonfanti! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Luciane Bonfanti | Psicóloga em Moema, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="133" xml:space="preserve">
@@ -6379,20 +5454,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J133" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K133" t="str">
-        <v>Av. Lavandisca, 741 - Moema, São Paulo - SP, 04515-011</v>
-      </c>
-      <c r="L133" t="str">
-        <v>https://wa.me/5511952911744?text=Ol%C3%A1%2C%20Mariana%20Honorio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M133" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Mariana Honorio! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511952911744?text=Ol%C3%A1%2C%20Mariana%20Honorio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Honorio%20Psicologa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K133" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Mariana Honorio! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Honorio Psicologa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -6424,20 +5492,13 @@
         <v>Sem site próprio (Apenas wixsite)</v>
       </c>
       <c r="J134" t="str">
-        <v>https://psicologatayane.wixsite.com/website</v>
-      </c>
-      <c r="K134" t="str">
-        <v>Estação Eucaliptos - Av. Rouxinol, 1041 - Moema, São Paulo - SP, 04516-001</v>
-      </c>
-      <c r="L134" t="str">
-        <v>https://wa.me/5511961879290?text=Ol%C3%A1%2C%20Tayane%20Teizen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M134" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Tayane Teizen! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511961879290?text=Ol%C3%A1%2C%20Tayane%20Teizen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Tayane%20Teizen%20-%20Psic%C3%B3loga%20Psicodin%C3%A2mica%20Psicanal%C3%ADtica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K134" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Tayane Teizen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Tayane Teizen - Psicóloga Psicodinâmica Psicanalítica, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="135" xml:space="preserve">
@@ -6469,20 +5530,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J135" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K135" t="str">
-        <v>Av. Chibarás, 75 - Moema, São Paulo - SP, 04076-000</v>
-      </c>
-      <c r="L135" t="str">
-        <v>https://wa.me/5511989304882?text=Ol%C3%A1%2C%20Adele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M135" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Adele! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511989304882?text=Ol%C3%A1%2C%20Adele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Adele%20Cestari%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K135" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Adele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Adele Cestari, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="136" xml:space="preserve">
@@ -6514,20 +5568,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J136" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K136" t="str">
-        <v>Av. Rouxinol, 84 - Moema, São Paulo - SP, 04516-000</v>
-      </c>
-      <c r="L136" t="str">
-        <v>https://wa.me/5511993376425?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M136" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica psicologia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993376425?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20psicologia%20%7C%20Gabriela%20Vaz%20Grzegorzewska%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K136" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Clínica psicologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de psicologia | Gabriela Vaz Grzegorzewska, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="137" xml:space="preserve">
@@ -6559,20 +5606,13 @@
         <v>Sem site próprio (Apenas linktr)</v>
       </c>
       <c r="J137" t="str">
-        <v>https://linktr.ee/psi.giopermac</v>
-      </c>
-      <c r="K137" t="str">
-        <v>Av. Bem-te-vi, 333 - Moema, São Paulo - SP, 04524-913</v>
-      </c>
-      <c r="L137" t="str">
-        <v>https://wa.me/5511998106227?text=Ol%C3%A1%2C%20Giovana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20um%20link%20de%20Linktree%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Moema%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M137" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Giovana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511998106227?text=Ol%C3%A1%2C%20Giovana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Giovana%20Pereira%20Macedo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K137" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Giovana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas um link de Linktree, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Moema, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Giovana Pereira Macedo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="138" xml:space="preserve">
@@ -6604,20 +5644,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J138" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K138" t="str">
-        <v>Avenida Paulista, 2073 Conjunto Nacional - Horsa II, Cj 101 - Jardins, São Paulo - SP, 01311-940</v>
-      </c>
-      <c r="L138" t="str">
-        <v>https://wa.me/5511948764737?text=Ol%C3%A1%2C%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M138" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Psicologia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511948764737?text=Ol%C3%A1%2C%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologia%20-%20Profa%20Dra%20Gabriella%20Alvarenga%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K138" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Psicologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologia - Profa Dra Gabriella Alvarenga, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="139" xml:space="preserve">
@@ -6649,20 +5682,13 @@
         <v>Sem site próprio (Apenas wa)</v>
       </c>
       <c r="J139" t="str">
-        <v>https://wa.me/5511943493132</v>
-      </c>
-      <c r="K139" t="str">
-        <v>Rua Haddock Lobo, 578 - Jardim Paulista, São Paulo - SP, 01414-000</v>
-      </c>
-      <c r="L139" t="str">
-        <v>https://wa.me/5511943493132?text=Ol%C3%A1%2C%20CLAUDIO%20CARLOS!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20direcionando%20apenas%20para%20o%20WhatsApp%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M139" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, CLAUDIO CARLOS! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511943493132?text=Ol%C3%A1%2C%20CLAUDIO%20CARLOS!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20CLAUDIO%20CARLOS%20DE%20SOUZA%20-%20Psic%C3%B3logo%20Jardins%20Av.%20Paulista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K139" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, CLAUDIO CARLOS! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está direcionando apenas para o WhatsApp, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para CLAUDIO CARLOS DE SOUZA - Psicólogo Jardins Av. Paulista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="140" xml:space="preserve">
@@ -6694,20 +5720,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J140" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K140" t="str">
-        <v>Av. Paulista, 807 - Conj 1001 - Bela Vista, São Paulo - SP, 01311-100</v>
-      </c>
-      <c r="L140" t="str">
-        <v>https://wa.me/5511996717876?text=Ol%C3%A1%2C%20Psicologa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M140" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Psicologa! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511996717876?text=Ol%C3%A1%2C%20Psicologa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K140" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Psicologa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="141" xml:space="preserve">
@@ -6739,20 +5758,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J141" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K141" t="str">
-        <v>R. Pamplona, 1445 - Conj 21 - Jardins, São Paulo - SP, 01405-002</v>
-      </c>
-      <c r="L141" t="str">
-        <v>https://wa.me/5511994413787?text=Ol%C3%A1%2C%20Fortun%C3%A9e%20Josiane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M141" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Fortunée Josiane! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511994413787?text=Ol%C3%A1%2C%20Fortun%C3%A9e%20Josiane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fortun%C3%A9e%20Josiane%20Zagha%20-%20Psic%C3%B3loga%20e%20Psicoterapeuta%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K141" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Fortunée Josiane! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fortunée Josiane Zagha - Psicóloga e Psicoterapeuta, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="142" xml:space="preserve">
@@ -6784,20 +5796,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J142" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K142" t="str">
-        <v>Av. Brig. Faria Lima, 1982 - Conj 701 - Jardim Paulistano, São Paulo - SP, 01451-000</v>
-      </c>
-      <c r="L142" t="str">
-        <v>https://wa.me/5511974992088?text=Ol%C3%A1%2C%20Marcela%20Pitombo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Jardins%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M142" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Marcela Pitombo! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511974992088?text=Ol%C3%A1%2C%20Marcela%20Pitombo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Marcela%20Pitombo%20Seixas%20-%20Psicologia%20Cl%C3%ADnica%20e%20Neuropsicologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K142" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Marcela Pitombo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Jardins, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Marcela Pitombo Seixas - Psicologia Clínica e Neuropsicologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="143" xml:space="preserve">
@@ -6829,20 +5834,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J143" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K143" t="str">
-        <v>R. dos Pinheiros, 240 - Conj 11 - Pinheiros, São Paulo - SP, 05422-010</v>
-      </c>
-      <c r="L143" t="str">
-        <v>https://wa.me/5511982031569?text=Ol%C3%A1%2C%20Patr%C3%ADcia%20Camelatto!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M143" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Patrícia Camelatto! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511982031569?text=Ol%C3%A1%2C%20Patr%C3%ADcia%20Camelatto!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Patr%C3%ADcia%20Camelatto%20-%20Psic%C3%B3loga%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K143" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Patrícia Camelatto! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Patrícia Camelatto - Psicóloga, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="144" xml:space="preserve">
@@ -6874,20 +5872,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J144" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K144" t="str">
-        <v>Av. Pedroso de Morais, 240 - Pinheiros, São Paulo - SP, 05420-903</v>
-      </c>
-      <c r="L144" t="str">
-        <v>https://wa.me/5511981559609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M144" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511981559609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20e%20Psicanalista%20Thaina%20Santos%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K144" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga e Psicanalista Thaina Santos, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="145" xml:space="preserve">
@@ -6919,20 +5910,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J145" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K145" t="str">
-        <v>Condomínio Edifício Executive Tower - R. Francisco Leitão, 469 - Pinheiros, São Paulo - SP, 05414-020</v>
-      </c>
-      <c r="L145" t="str">
-        <v>https://wa.me/5511995316010?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M145" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511995316010?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cristina%20Galv%C3%A3o%20Psic%C3%B3loga%20e%20Neuropsic%C3%B3loga%20Pinheiros%2FSP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K145" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cristina Galvão Psicóloga e Neuropsicóloga Pinheiros/SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="146" xml:space="preserve">
@@ -6964,20 +5948,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J146" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K146" t="str">
-        <v>R. Cônego Eugênio Leite, 933 - 45 - Pinheiros, São Paulo - SP, 05406-060</v>
-      </c>
-      <c r="L146" t="str">
-        <v>https://wa.me/5511986209818?text=Ol%C3%A1%2C%20Psicologia%20Pinheiros!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%203%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M146" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Psicologia Pinheiros! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511986209818?text=Ol%C3%A1%2C%20Psicologia%20Pinheiros!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%203%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologia%20Pinheiros%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K146" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Psicologia Pinheiros! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 3,7★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologia Pinheiros, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="147" xml:space="preserve">
@@ -7009,20 +5986,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J147" t="str">
-        <v>https://www.doctoralia.com.br/z/YixYVw</v>
-      </c>
-      <c r="K147" t="str">
-        <v>R. Pais Leme, 136 - 5° andar - sala 506 - Pinheiros, São Paulo - SP, 05424-010</v>
-      </c>
-      <c r="L147" t="str">
-        <v>https://wa.me/5511984804578?text=Ol%C3%A1%2C%20em!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Pinheiros%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M147" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, em! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511984804578?text=Ol%C3%A1%2C%20em!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20em%20Pinheiros%20-%20Elianai%20Holanda%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K147" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, em! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Pinheiros, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga em Pinheiros - Elianai Holanda, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="148" xml:space="preserve">
@@ -7054,20 +6024,13 @@
         <v>Sem site próprio (Apenas wixsite)</v>
       </c>
       <c r="J148" t="str">
-        <v>https://fernandaataidepsic.wixsite.com/my-site-1</v>
-      </c>
-      <c r="K148" t="str">
-        <v>Atendimentos On-line - R. Joaquim Floriano, 413 - Itaim Bibi, São Paulo - SP, 04534-011</v>
-      </c>
-      <c r="L148" t="str">
-        <v>https://wa.me/5511993286995?text=Ol%C3%A1%2C%20Fernanda%20Ataide!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M148" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Fernanda Ataide! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511993286995?text=Ol%C3%A1%2C%20Fernanda%20Ataide!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Ataide%20Psicologa%20Cl%C3%ADnica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K148" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Fernanda Ataide! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Ataide Psicologa Clínica, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="149" xml:space="preserve">
@@ -7099,20 +6062,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J149" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K149" t="str">
-        <v>R. Joaquim Floriano, 413 - Itaim Bibi, São Paulo - SP, 04534-011</v>
-      </c>
-      <c r="L149" t="str">
-        <v>https://wa.me/5511917252484?text=Ol%C3%A1%2C%20ZIL%C3%81%20GUIMAR%C3%83ES!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M149" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, ZILÁ GUIMARÃES! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511917252484?text=Ol%C3%A1%2C%20ZIL%C3%81%20GUIMAR%C3%83ES!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20ZIL%C3%81%20GUIMAR%C3%83ES-%20PSIC%C3%93LOGA-%20SP%20ITAIM%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K149" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, ZILÁ GUIMARÃES! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para ZILÁ GUIMARÃES- PSICÓLOGA- SP ITAIM, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="150" xml:space="preserve">
@@ -7144,20 +6100,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J150" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K150" t="str">
-        <v>R. Pedroso Alvarenga, 1062 - Conj 106 - Itaim Bibi, São Paulo - SP, 04531-010</v>
-      </c>
-      <c r="L150" t="str">
-        <v>https://wa.me/5511964682000?text=Ol%C3%A1%2C%20Consultorio%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M150" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Consultorio Psicologia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511964682000?text=Ol%C3%A1%2C%20Consultorio%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consultorio%20de%20Psicologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K150" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Consultorio Psicologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultorio de Psicologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="151" xml:space="preserve">
@@ -7189,20 +6138,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J151" t="str">
-        <v>https://www.doctoralia.com.br/eric-heibel/psicologo-psicanalista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=711270&amp;utm_content=website</v>
-      </c>
-      <c r="K151" t="str">
-        <v>Rua Urussuí, 92 - Conj 15 - Itaim Bibi, São Paulo - SP, 04542-050</v>
-      </c>
-      <c r="L151" t="str">
-        <v>https://wa.me/5511983831705?text=Ol%C3%A1%2C%20Eric%20Heibel%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Itaim%20Bibi%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M151" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Eric Heibel,! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511983831705?text=Ol%C3%A1%2C%20Eric%20Heibel%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Eric%20Heibel%2C%20Psic%C3%B3logo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K151" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Eric Heibel,! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Itaim Bibi, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Eric Heibel, Psicólogo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="152" xml:space="preserve">
@@ -7234,20 +6176,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J152" t="str">
-        <v>https://www.instagram.com/psicocamilasantos</v>
-      </c>
-      <c r="K152" t="str">
-        <v>R. Bartolomeu de Gusmão, 394 - Vila Mariana, São Paulo - SP, 04111-021</v>
-      </c>
-      <c r="L152" t="str">
-        <v>https://wa.me/5511987335609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M152" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511987335609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20e%20neuropsic%C3%B3loga%20Camila%20Santos%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K152" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga e neuropsicóloga Camila Santos, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="153" xml:space="preserve">
@@ -7279,20 +6214,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J153" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K153" t="str">
-        <v>Rua Teodoro Sampaio, 417, R. Domingos de Morais, 2132 - Vila Mariana, São Paulo - SP, 05405-000</v>
-      </c>
-      <c r="L153" t="str">
-        <v>https://wa.me/5511983635226?text=Ol%C3%A1%2C%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Vila%20Mariana%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M153" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Ana! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511983635226?text=Ol%C3%A1%2C%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Ana%20Florentino%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K153" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Ana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Vila Mariana, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Ana Florentino, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="154" xml:space="preserve">
@@ -7324,20 +6252,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J154" t="str">
-        <v>https://www.instagram.com/psicologasuzane/</v>
-      </c>
-      <c r="K154" t="str">
-        <v>Rua Catiguá, 159 - Tatuapé, São Paulo - SP, 03065-030</v>
-      </c>
-      <c r="L154" t="str">
-        <v>https://wa.me/5511987797093?text=Ol%C3%A1%2C%20Suzane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M154" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Suzane! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511987797093?text=Ol%C3%A1%2C%20Suzane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Suzane%20Rayssa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K154" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Suzane! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Suzane Rayssa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="155" xml:space="preserve">
@@ -7369,20 +6290,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J155" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K155" t="str">
-        <v>R. Francisco Marengo, 189 - Tatuapé, São Paulo - SP, 03355-020</v>
-      </c>
-      <c r="L155" t="str">
-        <v>https://wa.me/5511987208987?text=Ol%C3%A1%2C%20Lilian!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M155" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Lilian! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511987208987?text=Ol%C3%A1%2C%20Lilian!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Lilian%20Izzo%20%7C%20Tatuap%C3%A9%20-%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K155" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Lilian! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Lilian Izzo | Tatuapé - São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="156" xml:space="preserve">
@@ -7414,20 +6328,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J156" t="str">
-        <v>https://www.instagram.com/solangemedina.psico/</v>
-      </c>
-      <c r="K156" t="str">
-        <v>Rua Vilela, 665, 8º andar Edificio Crona - Tatuapé, São Paulo - SP, 03213-050</v>
-      </c>
-      <c r="L156" t="str">
-        <v>https://wa.me/5511982743076?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M156" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511982743076?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20no%20Tatuap%C3%A9%20SP%20%7C%20Terapia%20de%20Casal%2C%20Ansiedade%2C%20Depress%C3%A3o%20e%20Autoconhecimento%20-%20Solange%20Medina%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K156" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga no Tatuapé SP | Terapia de Casal, Ansiedade, Depressão e Autoconhecimento - Solange Medina, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="157" xml:space="preserve">
@@ -7459,20 +6366,13 @@
         <v>Sem site próprio (Apenas instagram)</v>
       </c>
       <c r="J157" t="str">
-        <v>https://www.instagram.com/psi.daylanesilva/</v>
-      </c>
-      <c r="K157" t="str">
-        <v>Rua Catiguá, 159 - Tatuapé, São Paulo - SP, 03065-030</v>
-      </c>
-      <c r="L157" t="str">
-        <v>https://wa.me/5511983150090?text=Ol%C3%A1%2C%20Daylane%20Silva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20o%20perfil%20do%20Instagram%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M157" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Daylane Silva! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511983150090?text=Ol%C3%A1%2C%20Daylane%20Silva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Daylane%20Silva%20%7C%20Psic%C3%B3loga%20Cl%C3%ADnica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K157" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Daylane Silva! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas o perfil do Instagram, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Daylane Silva | Psicóloga Clínica, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="158" xml:space="preserve">
@@ -7504,20 +6404,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J158" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K158" t="str">
-        <v>Rua Soriano de Sousa, 189 - Tatuapé, São Paulo - SP, 03066-020</v>
-      </c>
-      <c r="L158" t="str">
-        <v>https://wa.me/5511974441262?text=Ol%C3%A1%2C%20La%C3%ADs%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Tatuap%C3%A9%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M158" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Laís Fernandes! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511974441262?text=Ol%C3%A1%2C%20La%C3%ADs%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20La%C3%ADs%20Fernandes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K158" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Laís Fernandes! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Tatuapé, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Laís Fernandes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="159" xml:space="preserve">
@@ -7549,20 +6442,13 @@
         <v>Sem site próprio (Apenas doctoralia)</v>
       </c>
       <c r="J159" t="str">
-        <v>https://www.doctoralia.com.br/z/woij1Y</v>
-      </c>
-      <c r="K159" t="str">
-        <v>R. Cardoso de Almeida, 1005 - Perdizes, São Paulo - SP, 05013-001</v>
-      </c>
-      <c r="L159" t="str">
-        <v>https://wa.me/5511994158972?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20usando%20apenas%20a%20p%C3%A1gina%20do%20Doctoralia%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M159" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Julia! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511994158972?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Julia%20Ribas%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K159" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Julia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está usando apenas a página do Doctoralia, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Julia Ribas, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="160" xml:space="preserve">
@@ -7594,20 +6480,13 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J160" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K160" t="str">
-        <v>Edifício Adesso - Rua Cayowaá, 1071 - conj. 124 - Perdizes, São Paulo - SP, 05018-001</v>
-      </c>
-      <c r="L160" t="str">
-        <v>https://wa.me/5511987558867?text=Ol%C3%A1%2C%20Valquiria%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M160" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Valquiria Fernandes! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511987558867?text=Ol%C3%A1%2C%20Valquiria%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Valquiria%20Fernandes%20-%20Psic%C3%B3loga%20Integrativa%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K160" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Valquiria Fernandes! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Valquiria Fernandes - Psicóloga Integrativa em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="161" xml:space="preserve">
@@ -7639,25 +6518,18 @@
         <v>Sem site próprio (Sem site cadastrado)</v>
       </c>
       <c r="J161" t="str">
-        <v>Nenhum site cadastrado</v>
-      </c>
-      <c r="K161" t="str">
-        <v>R. Prof. Pedro da Cunha, 65 - Perdizes, São Paulo - SP, 05010-020</v>
-      </c>
-      <c r="L161" t="str">
-        <v>https://wa.me/5511987046526?text=Ol%C3%A1%2C%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%20da%20GS%20Dev%20Studio.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ANotei%20que%20hoje%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20sem%20um%20site%20institucional%20pr%C3%B3prio%20com%20agendamento%20direto.%20Quando%20algu%C3%A9m%20pesquisa%20por%20Psicologia%20no%20Google%20em%20Perdizes%2C%20quem%20tem%20site%20profissional%20passa%20muito%20mais%20credibilidade%20e%20recebe%20o%20contato%20antes.%0A%0ASelecionei%20o%20seu%20perfil%20para%20a%20nossa%20*a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20OFF%20nesta%20semana%20em%20S%C3%A3o%20Paulo*%3A%20desenvolvemos%20a%20sua%20p%C3%A1gina%20profissional%20de%20alta%20convers%C3%A3o%20para%20celular%20com%2050%25%20de%20desconto%20no%20setup%2C%20com%20bot%C3%A3o%20direto%20de%20WhatsApp%20e%20manuten%C3%A7%C3%A3o%20t%C3%A9cnica%20cont%C3%ADnua%20inclusa%20para%20voc%C3%AA%20n%C3%A3o%20se%20preocupar%20com%20nada.%0A%0APosso%20te%20mandar%20uma%20demonstra%C3%A7%C3%A3o%20visual%20de%201%20minuto%20sem%20compromisso%20para%20voc%C3%AA%20ver%20como%20ficaria%3F</v>
-      </c>
-      <c r="M161" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Marina! Tudo bem? Sou o Gabriel da GS Dev Studio.
+        <v>https://wa.me/5511987046526?text=Ol%C3%A1%2C%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Marina%20Araujo%20%7C%20Perdizes%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+      </c>
+      <c r="K161" t="str" xml:space="preserve">
+        <v xml:space="preserve">Olá, Marina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
 Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Notei que hoje você está sem uma página oficial própria cadastrada no Google, sem um site institucional próprio com agendamento direto. Quando alguém pesquisa por Psicologia no Google em Perdizes, quem tem site profissional passa muito mais credibilidade e recebe o contato antes.
-Selecionei o seu perfil para a nossa *ação promocional exclusiva de 50% OFF nesta semana em São Paulo*: desenvolvemos a sua página profissional de alta conversão para celular com 50% de desconto no setup, com botão direto de WhatsApp e manutenção técnica contínua inclusa para você não se preocupar com nada.
-Posso te mandar uma demonstração visual de 1 minuto sem compromisso para você ver como ficaria?</v>
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Marina Araujo | Perdizes SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M161"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K161"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(prospeccao): corrige classificação e badges de empresas sem site (elimina falso 'possui site' e adiciona filtros puros de zero link)
</commit_message>
<xml_diff>
--- a/prospeccao_160_leads_sp.xlsx
+++ b/prospeccao_160_leads_sp.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="160 Leads SP - 50% OFF" sheetId="1" r:id="rId1"/>
+    <sheet name="Leads Sem Site SP" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -398,19 +398,6 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K161"/>
-  <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="25.83203125" customWidth="1"/>
-    <col min="5" max="5" width="15.83203125" customWidth="1"/>
-    <col min="6" max="6" width="18.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
-    <col min="8" max="8" width="20.83203125" customWidth="1"/>
-    <col min="9" max="9" width="30.83203125" customWidth="1"/>
-    <col min="10" max="10" width="50.83203125" customWidth="1"/>
-    <col min="11" max="11" width="90.83203125" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -435,10 +422,10 @@
         <v>Nota Google</v>
       </c>
       <c r="H1" t="str">
-        <v>Avaliações</v>
+        <v>Situação do Site</v>
       </c>
       <c r="I1" t="str">
-        <v>Situação do Site</v>
+        <v>Link Cadastrado no Google</v>
       </c>
       <c r="J1" t="str">
         <v>Link WhatsApp Direto</v>
@@ -470,19 +457,19 @@
         <v>5,0</v>
       </c>
       <c r="H2" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I2" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>https://linktr.ee/drafefernandes</v>
       </c>
       <c r="J2" t="str">
-        <v>https://wa.me/5511991307186?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Fernandes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991307186?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Fernandes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K2" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Fernandes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Fernandes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -508,19 +495,19 @@
         <v>5,0</v>
       </c>
       <c r="H3" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I3" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>https://linktr.ee/drasamaraoliveira_?utm_source=ig&amp;utm_medium=social&amp;utm_content=link_in_bio&amp;fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQPOTM2NjE5NzQzMzkyNDU5AAGnfH1dXc14yvpmnoJ4k1irpfNClsn3d8yKB1Fov3MFQvQ8wKwpsOIMBgLt9XQ_aem_nMyhVMbErrB6Z85L6mXYkw</v>
       </c>
       <c r="J3" t="str">
-        <v>https://wa.me/5511964799591?text=Ol%C3%A1%2C%20Dra.%20Samara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Samara%20Oliveira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964799591?text=Ol%C3%A1%2C%20Dra.%20Samara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Samara%20Oliveira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K3" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Samara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Samara Oliveira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Samara Oliveira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -546,19 +533,19 @@
         <v>5,0</v>
       </c>
       <c r="H4" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I4" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J4" t="str">
-        <v>https://wa.me/5511940394742?text=Ol%C3%A1%2C%20Odontoreli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontoreli%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11940394742?text=Ol%C3%A1%2C%20Odontoreli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontoreli%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K4" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Odontoreli! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontoreli, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontoreli, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -584,19 +571,19 @@
         <v>5,0</v>
       </c>
       <c r="H5" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I5" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/marcia-ayres/dentista/sao-paulo</v>
       </c>
       <c r="J5" t="str">
-        <v>https://wa.me/5511971268686?text=Ol%C3%A1%2C%20Dra.%20Marcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcia%20Ayres%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11971268686?text=Ol%C3%A1%2C%20Dra.%20Marcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcia%20Ayres%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K5" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Marcia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcia Ayres, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcia Ayres, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -622,19 +609,19 @@
         <v>5,0</v>
       </c>
       <c r="H6" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I6" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J6" t="str">
-        <v>https://wa.me/5511984843250?text=Ol%C3%A1%2C%20Dr.%20Paulo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Dent%C3%A1rio%20Dr.%20Paulo%20Rog%C3%A9rio%20Barbosa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11984843250?text=Ol%C3%A1%2C%20Dr.%20Paulo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Dent%C3%A1rio%20Dr.%20Paulo%20Rog%C3%A9rio%20Barbosa%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K6" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dr. Paulo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Dentário Dr. Paulo Rogério Barbosa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Dentário Dr. Paulo Rogério Barbosa, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -660,19 +647,19 @@
         <v>5,0</v>
       </c>
       <c r="H7" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I7" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J7" t="str">
-        <v>https://wa.me/5511925683124?text=Ol%C3%A1%2C%20Oral%20Premium!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Oral%20Premium%20Implantes%20Pinheiros%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11925683124?text=Ol%C3%A1%2C%20Oral%20Premium!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Oral%20Premium%20Implantes%20Pinheiros%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K7" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Oral Premium! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Oral Premium Implantes Pinheiros, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Oral Premium Implantes Pinheiros, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -698,19 +685,19 @@
         <v>5,0</v>
       </c>
       <c r="H8" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I8" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J8" t="str">
-        <v>https://wa.me/5511944502942?text=Ol%C3%A1%2C%20Cairo%20Martinelli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cairo%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11944502942?text=Ol%C3%A1%2C%20Cairo%20Martinelli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cairo%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K8" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Cairo Martinelli! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cairo Martinelli Odontologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cairo Martinelli Odontologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -736,19 +723,19 @@
         <v>4,9</v>
       </c>
       <c r="H9" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I9" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>http://instagram.com/dr.viniciusbibiano</v>
       </c>
       <c r="J9" t="str">
-        <v>https://wa.me/5511993616602?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20Bibiano%20%7C%20Dentista%20em%20Pinheiros%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993616602?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20Bibiano%20%7C%20Dentista%20em%20Pinheiros%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K9" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica Bibiano | Dentista em Pinheiros, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica Bibiano | Dentista em Pinheiros, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -774,19 +761,19 @@
         <v>5,0</v>
       </c>
       <c r="H10" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I10" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/message/H22QFMB4FZMYD1</v>
       </c>
       <c r="J10" t="str">
-        <v>https://wa.me/5511950060220?text=Ol%C3%A1%2C%20Dra.%20J%C3%A9ssica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20J%C3%A9ssica%20Mattos%20de%20Britto%20-%20Odontologia%20Est%C3%A9tica%20e%20Restauradora%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11950060220?text=Ol%C3%A1%2C%20Dra.%20J%C3%A9ssica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20J%C3%A9ssica%20Mattos%20de%20Britto%20-%20Odontologia%20Est%C3%A9tica%20e%20Restauradora%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K10" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Jéssica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Jéssica Mattos de Britto - Odontologia Estética e Restauradora, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Jéssica Mattos de Britto - Odontologia Estética e Restauradora, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -812,19 +799,19 @@
         <v>5,0</v>
       </c>
       <c r="H11" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I11" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>http://instagram.com/dramariagoncalves</v>
       </c>
       <c r="J11" t="str">
-        <v>https://wa.me/5511910995184?text=Ol%C3%A1%2C%20Dra%20Maria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Maria%20Eduarda%20Gon%C3%A7alves%20%7C%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11910995184?text=Ol%C3%A1%2C%20Dra%20Maria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Maria%20Eduarda%20Gon%C3%A7alves%20%7C%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K11" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Maria! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Maria Eduarda Gonçalves | Cirurgiã Dentista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Maria Eduarda Gonçalves | Cirurgiã Dentista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -850,19 +837,19 @@
         <v>5,0</v>
       </c>
       <c r="H12" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I12" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/drgalsander?igsh=MXRwZ3JlZXQ3cXN3Yg==</v>
       </c>
       <c r="J12" t="str">
-        <v>https://wa.me/5511976253586?text=Ol%C3%A1%2C%20Dr.%20Galsander!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Galsander%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976253586?text=Ol%C3%A1%2C%20Dr.%20Galsander!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Galsander%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K12" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dr. Galsander! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Galsander, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Galsander, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -888,19 +875,19 @@
         <v>4,9</v>
       </c>
       <c r="H13" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I13" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J13" t="str">
-        <v>https://wa.me/5511964008778?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20AR%20Odontologia%20-%20Dr.%20C%C3%A9sar%20e%20Equipe%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964008778?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20AR%20Odontologia%20-%20Dr.%20C%C3%A9sar%20e%20Equipe%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K13" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica AR Odontologia - Dr. César e Equipe, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica AR Odontologia - Dr. César e Equipe, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -926,19 +913,19 @@
         <v>5,0</v>
       </c>
       <c r="H14" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I14" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J14" t="str">
-        <v>https://wa.me/5511947647807?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20LK%20%7C%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11947647807?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20LK%20%7C%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K14" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica LK | Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica LK | Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
@@ -964,19 +951,19 @@
         <v>5,0</v>
       </c>
       <c r="H15" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I15" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J15" t="str">
-        <v>https://wa.me/5511999919290?text=Ol%C3%A1%2C%20Dra.%20Carolina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Carolina%20Oliveira%20-%20Endodontia%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11999919290?text=Ol%C3%A1%2C%20Dra.%20Carolina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Carolina%20Oliveira%20-%20Endodontia%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K15" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Carolina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Carolina Oliveira - Endodontia e Harmonização Facial na Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Carolina Oliveira - Endodontia e Harmonização Facial na Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -1002,19 +989,19 @@
         <v>5,0</v>
       </c>
       <c r="H16" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I16" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J16" t="str">
-        <v>https://wa.me/5511958187028?text=Ol%C3%A1%2C%20Odontologico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontologico%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11958187028?text=Ol%C3%A1%2C%20Odontologico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontologico%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K16" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Odontologico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontologico na Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontologico na Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -1040,19 +1027,19 @@
         <v>4,9</v>
       </c>
       <c r="H17" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Google negocio.site desativado)</v>
       </c>
       <c r="I17" t="str">
-        <v>Sem site próprio (Apenas negocio)</v>
+        <v>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;url=https://dentista-dra-andreia-serra.negocio.site/&amp;ved=2ahUKEwjc5ueF7v_nAhWjLLkGHd-pDB0QFjAZegQIBxAB&amp;usg=AOvVaw23N10dPXvHyJEkdydgJi0X</v>
       </c>
       <c r="J17" t="str">
-        <v>https://wa.me/5511975911100?text=Ol%C3%A1%2C%20Dra.%20Andreia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Andreia%20Serra%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975911100?text=Ol%C3%A1%2C%20Dra.%20Andreia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Andreia%20Serra%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K17" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Andreia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Andreia Serra, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Andreia Serra, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
@@ -1078,19 +1065,19 @@
         <v>5,0</v>
       </c>
       <c r="H18" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I18" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://l.instagram.com/?u=https://linktr.ee/dramarciaharumimurata&amp;e=AT1N9YDKEugyBbEwe94G4hO-NzSWSyHgF1RhzSumj7pTZk2roJYnt2LifhIyfVpvgBMPU_BNIypnIsxCYq9APoSsmxxIDJQmdYcOiodw1AyXxK6TeRLfyw</v>
       </c>
       <c r="J18" t="str">
-        <v>https://wa.me/5511976088594?text=Ol%C3%A1%2C%20Dentista!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20-%20Tatuap%C3%A9%20-%20Dra.%20Marcia%20Harumi%20Murata%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976088594?text=Ol%C3%A1%2C%20Dentista!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20-%20Tatuap%C3%A9%20-%20Dra.%20Marcia%20Harumi%20Murata%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K18" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dentista! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista - Tatuapé - Dra. Marcia Harumi Murata, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista - Tatuapé - Dra. Marcia Harumi Murata, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
@@ -1116,19 +1103,19 @@
         <v>4,9</v>
       </c>
       <c r="H19" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I19" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J19" t="str">
-        <v>https://wa.me/5511930252702?text=Ol%C3%A1%2C%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra%20Regiane%20Carvalheiro%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11930252702?text=Ol%C3%A1%2C%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra%20Regiane%20Carvalheiro%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K19" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Odontológico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra Regiane Carvalheiro, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra Regiane Carvalheiro, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
@@ -1154,19 +1141,19 @@
         <v>4,9</v>
       </c>
       <c r="H20" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I20" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J20" t="str">
-        <v>https://wa.me/5511951406244?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Faustino%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951406244?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Faustino%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K20" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Faustino, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Faustino, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -1192,19 +1179,19 @@
         <v>5,0</v>
       </c>
       <c r="H21" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I21" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/dra_annacarolina</v>
       </c>
       <c r="J21" t="str">
-        <v>https://wa.me/5511985969605?text=Ol%C3%A1%2C%20Dra%20Anna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Anna%20Carolina%20%7C%20Dentista%20%7C%20Harmoniza%C3%A7%C3%A3o%20%7C%20Aparelho%20invis%C3%ADvel%20-%20sousmile%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11985969605?text=Ol%C3%A1%2C%20Dra%20Anna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Anna%20Carolina%20%7C%20Dentista%20%7C%20Harmoniza%C3%A7%C3%A3o%20%7C%20Aparelho%20invis%C3%ADvel%20-%20sousmile%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K21" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Anna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Anna Carolina | Dentista | Harmonização | Aparelho invisível - sousmile | Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Anna Carolina | Dentista | Harmonização | Aparelho invisível - sousmile | Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1230,19 +1217,19 @@
         <v>5,0</v>
       </c>
       <c r="H22" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I22" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J22" t="str">
-        <v>https://wa.me/5511985133002?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20S%C3%A3o%20Paulo%20Dra%20Bianca%20Assis%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11985133002?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20S%C3%A3o%20Paulo%20Dra%20Bianca%20Assis%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K22" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista São Paulo Dra Bianca Assis Cirurgiã Dentista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista São Paulo Dra Bianca Assis Cirurgiã Dentista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -1268,19 +1255,19 @@
         <v>4,9</v>
       </c>
       <c r="H23" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I23" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J23" t="str">
-        <v>https://wa.me/5511976103809?text=Ol%C3%A1%2C%20Dra.%20Daniella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Daniella%20Plaza%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976103809?text=Ol%C3%A1%2C%20Dra.%20Daniella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Daniella%20Plaza%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K23" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Daniella! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Daniella Plaza, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Daniella Plaza, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1306,19 +1293,19 @@
         <v>4,8</v>
       </c>
       <c r="H24" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I24" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/dratamymenezes?igshid=MzMyNGUyNmU2YQ==</v>
       </c>
       <c r="J24" t="str">
-        <v>https://wa.me/5511945231034?text=Ol%C3%A1%2C%20Clinica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Odontologia%20Especializada%20-%20Dra%20Thamiris%20Menezes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945231034?text=Ol%C3%A1%2C%20Clinica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Odontologia%20Especializada%20-%20Dra%20Thamiris%20Menezes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K24" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clinica Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Odontologia Especializada - Dra Thamiris Menezes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Odontologia Especializada - Dra Thamiris Menezes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1344,19 +1331,19 @@
         <v>5,0</v>
       </c>
       <c r="H25" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I25" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dradanielleoliveiraa?igsh=MW5oc3U0YWQ4Mmcyag==&amp;utm_source=qr</v>
       </c>
       <c r="J25" t="str">
-        <v>https://wa.me/5511991519479?text=Ol%C3%A1%2C%20Dra.%20Danielle!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Danielle%20Oliveira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991519479?text=Ol%C3%A1%2C%20Dra.%20Danielle!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Danielle%20Oliveira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K25" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Danielle! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Danielle Oliveira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Danielle Oliveira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1382,19 +1369,19 @@
         <v>5,0</v>
       </c>
       <c r="H26" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I26" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J26" t="str">
-        <v>https://wa.me/5511992918335?text=Ol%C3%A1%2C%20Dra.%20Isadora!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Isadora%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11992918335?text=Ol%C3%A1%2C%20Dra.%20Isadora!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Isadora%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K26" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Isadora! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Isadora Martinelli Odontologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Isadora Martinelli Odontologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1420,19 +1407,19 @@
         <v>5,0</v>
       </c>
       <c r="H27" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I27" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J27" t="str">
-        <v>https://wa.me/5511963239000?text=Ol%C3%A1%2C%20Dra%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Helena%20Pires%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11963239000?text=Ol%C3%A1%2C%20Dra%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Helena%20Pires%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K27" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Helena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Helena Pires, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Helena Pires, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1458,19 +1445,19 @@
         <v>4,8</v>
       </c>
       <c r="H28" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I28" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J28" t="str">
-        <v>https://wa.me/5511939011103?text=Ol%C3%A1%2C%20Dra%20Giovanna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Giovanna%20Dourado%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11939011103?text=Ol%C3%A1%2C%20Dra%20Giovanna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Giovanna%20Dourado%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K28" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Giovanna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Giovanna Dourado, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Giovanna Dourado, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -1496,19 +1483,19 @@
         <v>4,8</v>
       </c>
       <c r="H29" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I29" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J29" t="str">
-        <v>https://wa.me/5511988877098?text=Ol%C3%A1%2C%20Dra.Leticia%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Leticia%20Morais%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11988877098?text=Ol%C3%A1%2C%20Dra.Leticia%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Leticia%20Morais%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K29" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra.Leticia Morais! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Leticia Morais, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Leticia Morais, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -1534,19 +1521,19 @@
         <v>4,9</v>
       </c>
       <c r="H30" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I30" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J30" t="str">
-        <v>https://wa.me/5511996040673?text=Ol%C3%A1%2C%20Dra.%20Monique!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Monique%20Fai%C3%A3o%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11996040673?text=Ol%C3%A1%2C%20Dra.%20Monique!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Monique%20Fai%C3%A3o%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K30" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Monique! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Monique Faião, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Monique Faião, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -1572,19 +1559,19 @@
         <v>5,0</v>
       </c>
       <c r="H31" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I31" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra.luanavieiraa?igsh=cGRzNHNpOTJ4MXkw&amp;utm_source=qr</v>
       </c>
       <c r="J31" t="str">
-        <v>https://wa.me/5511978738749?text=Ol%C3%A1%2C%20Dentista%20Santana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20Santana%20-%20Dra%20Luana%20Vieira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11978738749?text=Ol%C3%A1%2C%20Dentista%20Santana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20Santana%20-%20Dra%20Luana%20Vieira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K31" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dentista Santana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em Santana - Dra Luana Vieira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em Santana - Dra Luana Vieira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="32" xml:space="preserve">
@@ -1610,19 +1597,19 @@
         <v>5,0</v>
       </c>
       <c r="H32" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I32" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/dralourdesspereira?igshid=MzRlODBiNWFlZA==</v>
       </c>
       <c r="J32" t="str">
-        <v>https://wa.me/5511956566650?text=Ol%C3%A1%2C%20Odontologia%20%2FSa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontologia%20%2FSa%C3%BAde%20e%20bem%20estar%20Dra%20Lourdes%20S.Pereira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11956566650?text=Ol%C3%A1%2C%20Odontologia%20%2FSa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontologia%20%2FSa%C3%BAde%20e%20bem%20estar%20Dra%20Lourdes%20S.Pereira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K32" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Odontologia /Saúde! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontologia /Saúde e bem estar Dra Lourdes S.Pereira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontologia /Saúde e bem estar Dra Lourdes S.Pereira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -1648,19 +1635,19 @@
         <v>5,0</v>
       </c>
       <c r="H33" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I33" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/draluciana.dentista</v>
       </c>
       <c r="J33" t="str">
-        <v>https://wa.me/5511993273559?text=Ol%C3%A1%2C%20Dra%20Luciana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luciana%20Espejo%20%7C%20Dentista%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993273559?text=Ol%C3%A1%2C%20Dra%20Luciana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luciana%20Espejo%20%7C%20Dentista%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K33" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Luciana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luciana Espejo | Dentista em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luciana Espejo | Dentista em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -1686,19 +1673,19 @@
         <v>5,0</v>
       </c>
       <c r="H34" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I34" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J34" t="str">
-        <v>https://wa.me/5511991252211?text=Ol%C3%A1%2C%20Dra%20Alessandra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Alessandra%20Parisi%20%7C%20Dentista%20%7C%20Santana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991252211?text=Ol%C3%A1%2C%20Dra%20Alessandra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Alessandra%20Parisi%20%7C%20Dentista%20%7C%20Santana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K34" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Alessandra! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Alessandra Parisi | Dentista | Santana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Alessandra Parisi | Dentista | Santana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -1724,19 +1711,19 @@
         <v>5,0</v>
       </c>
       <c r="H35" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I35" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J35" t="str">
-        <v>https://wa.me/5511915333818?text=Ol%C3%A1%2C%20Dra.%20Thabata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra.%20Thabata%20L%C3%ADvia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11915333818?text=Ol%C3%A1%2C%20Dra.%20Thabata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra.%20Thabata%20L%C3%ADvia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K35" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Thabata! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra. Thabata Lívia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra. Thabata Lívia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
@@ -1762,19 +1749,19 @@
         <v>4,9</v>
       </c>
       <c r="H36" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I36" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/centroodontomorumbi/</v>
       </c>
       <c r="J36" t="str">
-        <v>https://wa.me/5511966400022?text=Ol%C3%A1%2C%20Centro%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20Odontol%C3%B3gico%20Morumbi%20-%20Dra%20Renata%20Ramos%20e%20Equipe%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11966400022?text=Ol%C3%A1%2C%20Centro%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20Odontol%C3%B3gico%20Morumbi%20-%20Dra%20Renata%20Ramos%20e%20Equipe%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K36" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Centro Odontológico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro Odontológico Morumbi - Dra Renata Ramos e Equipe, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro Odontológico Morumbi - Dra Renata Ramos e Equipe, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -1800,19 +1787,19 @@
         <v>5,0</v>
       </c>
       <c r="H37" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I37" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J37" t="str">
-        <v>https://wa.me/5511951307605?text=Ol%C3%A1%2C%20Dentista%20Morumbi%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Morumbi%2C%20S%C3%A3o%20Paulo%20-%20Dra%20Larissa%20Tavares%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951307605?text=Ol%C3%A1%2C%20Dentista%20Morumbi%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Morumbi%2C%20S%C3%A3o%20Paulo%20-%20Dra%20Larissa%20Tavares%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K37" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dentista Morumbi,! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Morumbi, São Paulo - Dra Larissa Tavares, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Morumbi, São Paulo - Dra Larissa Tavares, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -1838,19 +1825,19 @@
         <v>5,0</v>
       </c>
       <c r="H38" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I38" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J38" t="str">
-        <v>https://wa.me/5511959391155?text=Ol%C3%A1%2C%20Dr.%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Dr.%20Jo%C3%A3o%20Vila%20-%20Morumbi%20-%20Vila%20Progredior%20-%20Jd%20Guedala%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11959391155?text=Ol%C3%A1%2C%20Dr.%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Dr.%20Jo%C3%A3o%20Vila%20-%20Morumbi%20-%20Vila%20Progredior%20-%20Jd%20Guedala%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K38" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dr. João! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Dr. João Vila - Morumbi - Vila Progredior - Jd Guedala, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Dr. João Vila - Morumbi - Vila Progredior - Jd Guedala, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -1876,19 +1863,19 @@
         <v>4,7</v>
       </c>
       <c r="H39" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I39" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J39" t="str">
-        <v>https://wa.me/5511958978174?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20S%C3%A3o%20Paulo%20-%20Dra%20Bruna%20Del%20Mestre%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11958978174?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20S%C3%A3o%20Paulo%20-%20Dra%20Bruna%20Del%20Mestre%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K39" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,7★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em São Paulo - Dra Bruna Del Mestre, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,7★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em São Paulo - Dra Bruna Del Mestre, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -1914,19 +1901,19 @@
         <v>5,0</v>
       </c>
       <c r="H40" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I40" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J40" t="str">
-        <v>https://wa.me/5511949420235?text=Ol%C3%A1%2C%20Dra.%20Tayna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Tayna%20Bastos%20%7C%20Dentista%20no%20Morumbi%20-%20S%C3%A3o%20Paulo%20%7C%20Pr%C3%B3tese%2C%20est%C3%A9tica%20e%20urg%C3%AAncia.%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11949420235?text=Ol%C3%A1%2C%20Dra.%20Tayna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Tayna%20Bastos%20%7C%20Dentista%20no%20Morumbi%20-%20S%C3%A3o%20Paulo%20%7C%20Pr%C3%B3tese%2C%20est%C3%A9tica%20e%20urg%C3%AAncia.%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K40" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Tayna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Tayna Bastos | Dentista no Morumbi - São Paulo | Prótese, estética e urgência., pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Tayna Bastos | Dentista no Morumbi - São Paulo | Prótese, estética e urgência., pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -1952,19 +1939,19 @@
         <v>5,0</v>
       </c>
       <c r="H41" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I41" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra_mayaracardoso/</v>
       </c>
       <c r="J41" t="str">
-        <v>https://wa.me/5511947930542?text=Ol%C3%A1%2C%20Dra%20Mayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Mayara%20Cardoso%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11947930542?text=Ol%C3%A1%2C%20Dra%20Mayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Mayara%20Cardoso%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K41" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Mayara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Mayara Cardoso, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Mayara Cardoso, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -1990,19 +1977,19 @@
         <v>5,0</v>
       </c>
       <c r="H42" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I42" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/nayara-freitas/dentista/sao-paulo</v>
       </c>
       <c r="J42" t="str">
-        <v>https://wa.me/5511972871378?text=Ol%C3%A1%2C%20Dra%20Nayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Nayara%20Freitas%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972871378?text=Ol%C3%A1%2C%20Dra%20Nayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Nayara%20Freitas%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K42" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Nayara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Nayara Freitas, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Nayara Freitas, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="43" xml:space="preserve">
@@ -2028,19 +2015,19 @@
         <v>5,0</v>
       </c>
       <c r="H43" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I43" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dr.alexandrewon/</v>
       </c>
       <c r="J43" t="str">
-        <v>https://wa.me/5511940696509?text=Ol%C3%A1%2C%20Won%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Won%20Odontologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11940696509?text=Ol%C3%A1%2C%20Won%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Won%20Odontologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K43" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Won Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Won Odontologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Won Odontologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
@@ -2066,19 +2053,19 @@
         <v>5,0</v>
       </c>
       <c r="H44" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I44" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J44" t="str">
-        <v>https://wa.me/5511945216642?text=Ol%C3%A1%2C%20Dr.%20Marcello!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Marcello%20Barone%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%20e%20Odontologia%20est%C3%A9tica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945216642?text=Ol%C3%A1%2C%20Dr.%20Marcello!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Marcello%20Barone%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%20e%20Odontologia%20est%C3%A9tica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K44" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dr. Marcello! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Marcello Barone - Harmonização Orofacial e Odontologia estética, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Marcello Barone - Harmonização Orofacial e Odontologia estética, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
@@ -2104,19 +2091,19 @@
         <v>5,0</v>
       </c>
       <c r="H45" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I45" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J45" t="str">
-        <v>https://wa.me/5511998978621?text=Ol%C3%A1%2C%20Dra.%20Cecilia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cecilia%20Sena%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11998978621?text=Ol%C3%A1%2C%20Dra.%20Cecilia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cecilia%20Sena%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K45" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Cecilia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cecilia Sena, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cecilia Sena, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -2142,19 +2129,19 @@
         <v>5,0</v>
       </c>
       <c r="H46" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I46" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J46" t="str">
-        <v>https://wa.me/5511984157966?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Rodrigues%20Santos%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11984157966?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Rodrigues%20Santos%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K46" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Rodrigues Santos, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Rodrigues Santos, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -2180,19 +2167,19 @@
         <v>4,3</v>
       </c>
       <c r="H47" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I47" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/drasilviaarruda?utm_medium=copy_link</v>
       </c>
       <c r="J47" t="str">
-        <v>https://wa.me/5511998439008?text=Ol%C3%A1%2C%20Dra%20Silvia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C3%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Silvia%20Gajardoni%20Arruda%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11998439008?text=Ol%C3%A1%2C%20Dra%20Silvia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C3%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Silvia%20Gajardoni%20Arruda%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K47" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Silvia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 4,3★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Silvia Gajardoni Arruda, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 4,3★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Silvia Gajardoni Arruda, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -2218,19 +2205,19 @@
         <v>5,0</v>
       </c>
       <c r="H48" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I48" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/draraphaela.maia/</v>
       </c>
       <c r="J48" t="str">
-        <v>https://wa.me/5511993878167?text=Ol%C3%A1%2C%20Dra%20Raphaela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raphaela%20Maia%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20em%20Moema%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993878167?text=Ol%C3%A1%2C%20Dra%20Raphaela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raphaela%20Maia%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20em%20Moema%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K48" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Raphaela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raphaela Maia - Harmonização Facial em Moema, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raphaela Maia - Harmonização Facial em Moema, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="49" xml:space="preserve">
@@ -2256,19 +2243,19 @@
         <v>5,0</v>
       </c>
       <c r="H49" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I49" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>https://linktr.ee/drafeliramonteiro</v>
       </c>
       <c r="J49" t="str">
-        <v>https://wa.me/5511988571847?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Lira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Zona%20Sul%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11988571847?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Lira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Zona%20Sul%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K49" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Lira | Harmonização Facial | Zona Sul São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Lira | Harmonização Facial | Zona Sul São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -2294,19 +2281,19 @@
         <v>5,0</v>
       </c>
       <c r="H50" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I50" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dramendoncagabriela?igsh=MTE5MThiMGVhcXV2MQ==</v>
       </c>
       <c r="J50" t="str">
-        <v>https://wa.me/5511965850611?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Mendon%C3%A7a%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11965850611?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Mendon%C3%A7a%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K50" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Mendonça - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Mendonça - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">
@@ -2332,19 +2319,19 @@
         <v>4,9</v>
       </c>
       <c r="H51" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I51" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J51" t="str">
-        <v>https://wa.me/5511975815099?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Avan%C3%A7ada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20AC%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975815099?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Avan%C3%A7ada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20AC%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K51" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Estética Avançada! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para AC Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para AC Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="52" xml:space="preserve">
@@ -2370,19 +2357,19 @@
         <v>5,0</v>
       </c>
       <c r="H52" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I52" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J52" t="str">
-        <v>https://wa.me/5511958882681?text=Ol%C3%A1%2C%20Dra%20Fl%C3%A1via!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Fl%C3%A1via%20Roma%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11958882681?text=Ol%C3%A1%2C%20Dra%20Fl%C3%A1via!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Fl%C3%A1via%20Roma%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K52" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Flávia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Flávia Roma Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Flávia Roma Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="53" xml:space="preserve">
@@ -2408,19 +2395,19 @@
         <v>5,0</v>
       </c>
       <c r="H53" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I53" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/estetica_monicamuchante?igsh=M2syNWtzY2t3b3k4</v>
       </c>
       <c r="J53" t="str">
-        <v>https://wa.me/5511951008872?text=Ol%C3%A1%2C%20Dra.%20M%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20M%C3%B4nica%20Muchante%20Biom%C3%A9dica%20Esteta%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951008872?text=Ol%C3%A1%2C%20Dra.%20M%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20M%C3%B4nica%20Muchante%20Biom%C3%A9dica%20Esteta%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K53" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Mônica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Mônica Muchante Biomédica Esteta | Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Mônica Muchante Biomédica Esteta | Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="54" xml:space="preserve">
@@ -2446,19 +2433,19 @@
         <v>5,0</v>
       </c>
       <c r="H54" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I54" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dragiulianafranca/</v>
       </c>
       <c r="J54" t="str">
-        <v>https://wa.me/5511977440161?text=Ol%C3%A1%2C%20Dra.%20Giuliana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Giuliana%20Fran%C3%A7a%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11977440161?text=Ol%C3%A1%2C%20Dra.%20Giuliana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Giuliana%20Fran%C3%A7a%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K54" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Giuliana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Giuliana França Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Giuliana França Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="55" xml:space="preserve">
@@ -2484,19 +2471,19 @@
         <v>5,0</v>
       </c>
       <c r="H55" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I55" t="str">
-        <v>Sem site próprio (Apenas api)</v>
+        <v>https://api.whatsapp.com/message/CDJPK6KBGJXNE1?autoload=1&amp;app_absent=0</v>
       </c>
       <c r="J55" t="str">
-        <v>https://wa.me/5511966291967?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Mello%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11966291967?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Mello%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K55" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Mello | Estética Avançada SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Mello | Estética Avançada SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="56" xml:space="preserve">
@@ -2522,19 +2509,19 @@
         <v>5,0</v>
       </c>
       <c r="H56" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I56" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J56" t="str">
-        <v>https://wa.me/5511952805419?text=Ol%C3%A1%2C%20Dra%20Leticia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Leticia%20Papp%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11952805419?text=Ol%C3%A1%2C%20Dra%20Leticia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Leticia%20Papp%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K56" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Leticia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Leticia Papp - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Leticia Papp - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="57" xml:space="preserve">
@@ -2560,19 +2547,19 @@
         <v>5,0</v>
       </c>
       <c r="H57" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I57" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra_amandaomartins/</v>
       </c>
       <c r="J57" t="str">
-        <v>https://wa.me/5511975791298?text=Ol%C3%A1%2C%20Lemu%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Lemu%20Clinic%20%7C%20Dra.%20Amanda%20Martins%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975791298?text=Ol%C3%A1%2C%20Lemu%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Lemu%20Clinic%20%7C%20Dra.%20Amanda%20Martins%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K57" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Lemu Clinic! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Lemu Clinic | Dra. Amanda Martins | Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Lemu Clinic | Dra. Amanda Martins | Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="58" xml:space="preserve">
@@ -2598,19 +2585,19 @@
         <v>5,0</v>
       </c>
       <c r="H58" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I58" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J58" t="str">
-        <v>https://wa.me/5511976971573?text=Ol%C3%A1%2C%20Dra%20Stephanie!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Stephanie%20Milagre%20-%20Cl%C3%ADnica%20de%20est%C3%A9tica%20avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976971573?text=Ol%C3%A1%2C%20Dra%20Stephanie!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Stephanie%20Milagre%20-%20Cl%C3%ADnica%20de%20est%C3%A9tica%20avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K58" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Stephanie! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Stephanie Milagre - Clínica de estética avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Stephanie Milagre - Clínica de estética avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2636,19 +2623,19 @@
         <v>5,0</v>
       </c>
       <c r="H59" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I59" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J59" t="str">
-        <v>https://wa.me/5511954537661?text=Ol%C3%A1%2C%20Dra%20Renata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Renata%20Queiroz%20-%20Biomedicina%20Est%C3%A9tica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11954537661?text=Ol%C3%A1%2C%20Dra%20Renata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Renata%20Queiroz%20-%20Biomedicina%20Est%C3%A9tica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K59" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Renata! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Renata Queiroz - Biomedicina Estética, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Renata Queiroz - Biomedicina Estética, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="60" xml:space="preserve">
@@ -2674,19 +2661,19 @@
         <v>5,0</v>
       </c>
       <c r="H60" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I60" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J60" t="str">
-        <v>https://wa.me/5511962612208?text=Ol%C3%A1%2C%20Nathalia%20Nastri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr%20Nathalia%20Nastri%20-%20Biomedicina%20Est%C3%A9tica-%20Pinheiros%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11962612208?text=Ol%C3%A1%2C%20Nathalia%20Nastri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr%20Nathalia%20Nastri%20-%20Biomedicina%20Est%C3%A9tica-%20Pinheiros%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K60" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Nathalia Nastri! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr Nathalia Nastri - Biomedicina Estética- Pinheiros São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr Nathalia Nastri - Biomedicina Estética- Pinheiros São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="61" xml:space="preserve">
@@ -2712,19 +2699,19 @@
         <v>5,0</v>
       </c>
       <c r="H61" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I61" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J61" t="str">
-        <v>https://wa.me/5511914566745?text=Ol%C3%A1%2C%20Dra.Igma%20Araujo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Igma%20Araujo%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11914566745?text=Ol%C3%A1%2C%20Dra.Igma%20Araujo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Igma%20Araujo%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K61" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra.Igma Araujo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Igma Araujo | Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Igma Araujo | Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="62" xml:space="preserve">
@@ -2750,19 +2737,19 @@
         <v>5,0</v>
       </c>
       <c r="H62" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I62" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/5511988399169</v>
       </c>
       <c r="J62" t="str">
-        <v>https://wa.me/5511991646740?text=Ol%C3%A1%2C%20Dra%20Carmen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carmen%20Barge%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Corporal%20%7C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991646740?text=Ol%C3%A1%2C%20Dra%20Carmen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carmen%20Barge%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Corporal%20%7C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K62" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Carmen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carmen Barge | Harmonização Facial e Corporal | São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carmen Barge | Harmonização Facial e Corporal | São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="63" xml:space="preserve">
@@ -2788,19 +2775,19 @@
         <v>5,0</v>
       </c>
       <c r="H63" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I63" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dralaismarquesa/</v>
       </c>
       <c r="J63" t="str">
-        <v>https://wa.me/5511954742132?text=Ol%C3%A1%2C%20Dra.%20La%C3%ADs!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20La%C3%ADs%20Marques%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11954742132?text=Ol%C3%A1%2C%20Dra.%20La%C3%ADs!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20La%C3%ADs%20Marques%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K63" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Laís! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Laís Marques - Harmonização Orofacial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Laís Marques - Harmonização Orofacial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="64" xml:space="preserve">
@@ -2826,19 +2813,19 @@
         <v>5,0</v>
       </c>
       <c r="H64" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I64" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J64" t="str">
-        <v>https://wa.me/5511944625222?text=Ol%C3%A1%2C%20Clinica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Est%C3%A9tica-%20Elaine%20Vasconcelos-%20Harmoniza%C3%A7%C3%A3o%20Facial-%20Itaim%20Bibi%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11944625222?text=Ol%C3%A1%2C%20Clinica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Est%C3%A9tica-%20Elaine%20Vasconcelos-%20Harmoniza%C3%A7%C3%A3o%20Facial-%20Itaim%20Bibi%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K64" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clinica Estética! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Estética- Elaine Vasconcelos- Harmonização Facial- Itaim Bibi, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Estética- Elaine Vasconcelos- Harmonização Facial- Itaim Bibi, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="65" xml:space="preserve">
@@ -2864,19 +2851,19 @@
         <v>5,0</v>
       </c>
       <c r="H65" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I65" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J65" t="str">
-        <v>https://wa.me/5511961662005?text=Ol%C3%A1%2C%20Dra.%20Alyne!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Alyne%20Souza%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20-%20Vila%20Ol%C3%ADmpia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11961662005?text=Ol%C3%A1%2C%20Dra.%20Alyne!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Alyne%20Souza%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20-%20Vila%20Ol%C3%ADmpia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K65" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Alyne! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Alyne Souza | Harmonização Facial - Vila Olímpia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Alyne Souza | Harmonização Facial - Vila Olímpia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="66" xml:space="preserve">
@@ -2902,19 +2889,19 @@
         <v>5,0</v>
       </c>
       <c r="H66" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I66" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J66" t="str">
-        <v>https://wa.me/5511917440783?text=Ol%C3%A1%2C%20Dra.%20Thayn%C3%A1!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Thayn%C3%A1%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11917440783?text=Ol%C3%A1%2C%20Dra.%20Thayn%C3%A1!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Thayn%C3%A1%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K66" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Thayná! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Thayná Rosa | Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Thayná Rosa | Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="67" xml:space="preserve">
@@ -2940,19 +2927,19 @@
         <v>4,7</v>
       </c>
       <c r="H67" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I67" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/clinicabellalinea?igsh=MXVmMngxNm05aXdlZQ%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J67" t="str">
-        <v>https://wa.me/5511991236080?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Bella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Bella%20Linea%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991236080?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Bella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Bella%20Linea%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K67" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica Bella! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 4,7★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Bella Linea, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 4,7★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Bella Linea, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="68" xml:space="preserve">
@@ -2978,19 +2965,19 @@
         <v>5,0</v>
       </c>
       <c r="H68" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I68" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J68" t="str">
-        <v>https://wa.me/5511992442685?text=Ol%C3%A1%2C%20Dra%20Raquel!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raquel%20Camargo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11992442685?text=Ol%C3%A1%2C%20Dra%20Raquel!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raquel%20Camargo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K68" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Raquel! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raquel Camargo - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raquel Camargo - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="69" xml:space="preserve">
@@ -3016,19 +3003,19 @@
         <v>5,0</v>
       </c>
       <c r="H69" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I69" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/5511965833614</v>
       </c>
       <c r="J69" t="str">
-        <v>https://wa.me/5511965833614?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Botox%20na%20Vila%20Mariana%20Dra.%20Bruna%20Ferreira%20Esteta%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11965833614?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Botox%20na%20Vila%20Mariana%20Dra.%20Bruna%20Ferreira%20Esteta%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K69" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Botox na Vila Mariana Dra. Bruna Ferreira Esteta, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Botox na Vila Mariana Dra. Bruna Ferreira Esteta, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="70" xml:space="preserve">
@@ -3054,19 +3041,19 @@
         <v>5,0</v>
       </c>
       <c r="H70" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I70" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J70" t="str">
-        <v>https://wa.me/5511994003820?text=Ol%C3%A1%2C%20Nadia%20Ces%C3%A1rio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nadia%20Ces%C3%A1rio%20-%20Est%C3%A9tica%20Especializada%20%7CDrenagem%20Linf%C3%A1tica%20Vila%20Mariana%20%7CLimpeza%20de%20pele%20%7CLipedema%7C%20P%C3%B3s%20Operat%C3%B3rio%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11994003820?text=Ol%C3%A1%2C%20Nadia%20Ces%C3%A1rio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nadia%20Ces%C3%A1rio%20-%20Est%C3%A9tica%20Especializada%20%7CDrenagem%20Linf%C3%A1tica%20Vila%20Mariana%20%7CLimpeza%20de%20pele%20%7CLipedema%7C%20P%C3%B3s%20Operat%C3%B3rio%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K70" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Nadia Cesário! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nadia Cesário - Estética Especializada |Drenagem Linfática Vila Mariana |Limpeza de pele |Lipedema| Pós Operatório, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nadia Cesário - Estética Especializada |Drenagem Linfática Vila Mariana |Limpeza de pele |Lipedema| Pós Operatório, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="71" xml:space="preserve">
@@ -3092,19 +3079,19 @@
         <v>5,0</v>
       </c>
       <c r="H71" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I71" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J71" t="str">
-        <v>https://wa.me/5511999985553?text=Ol%C3%A1%2C%20Dra.%20Mage!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Dra.%20Mage%20Mantovani%20Est%C3%A9tica%20Avan%C3%A7ada%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11999985553?text=Ol%C3%A1%2C%20Dra.%20Mage!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Dra.%20Mage%20Mantovani%20Est%C3%A9tica%20Avan%C3%A7ada%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K71" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Mage! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Dra. Mage Mantovani Estética Avançada Vila Mariana, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Dra. Mage Mantovani Estética Avançada Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="72" xml:space="preserve">
@@ -3130,19 +3117,19 @@
         <v>5,0</v>
       </c>
       <c r="H72" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I72" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra.amandarubio?igsh=MTI5NmJkZWU2d2VlMw==&amp;utm_source=qr</v>
       </c>
       <c r="J72" t="str">
-        <v>https://wa.me/5511974771241?text=Ol%C3%A1%2C%20Dra%20Amanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Amanda%20Rubio%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11974771241?text=Ol%C3%A1%2C%20Dra%20Amanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Amanda%20Rubio%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K72" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Amanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Amanda Rubio - Harmonização Facial e Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Amanda Rubio - Harmonização Facial e Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -3168,19 +3155,19 @@
         <v>5,0</v>
       </c>
       <c r="H73" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I73" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me//5511993736844?text=Ol%C3%A1!%20Encontrei%20no%20Google%20e%20quero%20saber%20mais.</v>
       </c>
       <c r="J73" t="str">
-        <v>https://wa.me/5511993736844?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Bruna%20Martinez%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993736844?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Bruna%20Martinez%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K73" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Bruna Martinez - Harmonização Facial Tatuapé SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Bruna Martinez - Harmonização Facial Tatuapé SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="74" xml:space="preserve">
@@ -3206,19 +3193,19 @@
         <v>4,9</v>
       </c>
       <c r="H74" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I74" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/message/CIUHJ3HBXIETA1</v>
       </c>
       <c r="J74" t="str">
-        <v>https://wa.me/5511994073067?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Guimar%C3%A3es%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11994073067?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Guimar%C3%A3es%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K74" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Guimarães Rosa | Harmonização Facial Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Guimarães Rosa | Harmonização Facial Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="75" xml:space="preserve">
@@ -3244,19 +3231,19 @@
         <v>5,0</v>
       </c>
       <c r="H75" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I75" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J75" t="str">
-        <v>https://wa.me/5511953634975?text=Ol%C3%A1%2C%20Dra.%20Vit%C3%B3ria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Vit%C3%B3ria%20Caldeira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11953634975?text=Ol%C3%A1%2C%20Dra.%20Vit%C3%B3ria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Vit%C3%B3ria%20Caldeira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K75" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Vitória! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Vitória Caldeira | Harmonização Facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Vitória Caldeira | Harmonização Facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="76" xml:space="preserve">
@@ -3282,19 +3269,19 @@
         <v>5,0</v>
       </c>
       <c r="H76" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I76" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/5511945950480</v>
       </c>
       <c r="J76" t="str">
-        <v>https://wa.me/5511945950480?text=Ol%C3%A1%2C%20Dra.%20Gisele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Gisele%20Neves%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%20%7C%20Botox%20%7C%20Ultraformer%20%7C%20Sculptra%20%7C%20Radiesse%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945950480?text=Ol%C3%A1%2C%20Dra.%20Gisele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Gisele%20Neves%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%20%7C%20Botox%20%7C%20Ultraformer%20%7C%20Sculptra%20%7C%20Radiesse%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K76" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Gisele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Gisele Neves - Harmonização Facial no Tatuapé | Botox | Ultraformer | Sculptra | Radiesse, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Gisele Neves - Harmonização Facial no Tatuapé | Botox | Ultraformer | Sculptra | Radiesse, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="77" xml:space="preserve">
@@ -3320,19 +3307,19 @@
         <v>5,0</v>
       </c>
       <c r="H77" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I77" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>https://linktr.ee/dracarla.bocuto?fbclid=PAAabVkC7D5GvCg526Viljb7iD7leQoFXx5zYuUVFUNXw_8gCHOeAkCW2DXSw</v>
       </c>
       <c r="J77" t="str">
-        <v>https://wa.me/5511982885834?text=Ol%C3%A1%2C%20Dra%20Carla!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carla%20Bocuto%20Harmoniza%C3%A7%C3%A3o%20Natural%20-%20Botox%20Tatuap%C3%A9%2C%20Mind%20Est%C3%A9tica.%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11982885834?text=Ol%C3%A1%2C%20Dra%20Carla!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carla%20Bocuto%20Harmoniza%C3%A7%C3%A3o%20Natural%20-%20Botox%20Tatuap%C3%A9%2C%20Mind%20Est%C3%A9tica.%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K77" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Carla! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carla Bocuto Harmonização Natural - Botox Tatuapé, Mind Estética., pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carla Bocuto Harmonização Natural - Botox Tatuapé, Mind Estética., pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="78" xml:space="preserve">
@@ -3358,19 +3345,19 @@
         <v>5,0</v>
       </c>
       <c r="H78" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I78" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra.marinaferreira</v>
       </c>
       <c r="J78" t="str">
-        <v>https://wa.me/5511983714557?text=Ol%C3%A1%2C%20Dra.%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marina%20Ferreira%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20%7C%20Tatuap%C3%A9%2FAn%C3%A1lia%20Franco%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11983714557?text=Ol%C3%A1%2C%20Dra.%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marina%20Ferreira%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20%7C%20Tatuap%C3%A9%2FAn%C3%A1lia%20Franco%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K78" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Marina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marina Ferreira | Harmonização facial | Tatuapé/Anália Franco SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marina Ferreira | Harmonização facial | Tatuapé/Anália Franco SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="79" xml:space="preserve">
@@ -3396,19 +3383,19 @@
         <v>5,0</v>
       </c>
       <c r="H79" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I79" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra.leticiaforstner/</v>
       </c>
       <c r="J79" t="str">
-        <v>https://wa.me/5511963070502?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Forstner%20%7C%20Otomodela%C3%A7%C3%A3o%20%E2%80%A2%20Preenchimento%20Labial%20%E2%80%A2%20Botox%20%E2%80%A2%20Harmoniza%C3%A7%C3%A3o%20Facial%20%E2%80%93%20Tatuap%C3%A9%20SP%20%7C%20Line%20Skin%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11963070502?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Forstner%20%7C%20Otomodela%C3%A7%C3%A3o%20%E2%80%A2%20Preenchimento%20Labial%20%E2%80%A2%20Botox%20%E2%80%A2%20Harmoniza%C3%A7%C3%A3o%20Facial%20%E2%80%93%20Tatuap%C3%A9%20SP%20%7C%20Line%20Skin%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K79" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Forstner | Otomodelação • Preenchimento Labial • Botox • Harmonização Facial – Tatuapé SP | Line Skin, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Forstner | Otomodelação • Preenchimento Labial • Botox • Harmonização Facial – Tatuapé SP | Line Skin, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="80" xml:space="preserve">
@@ -3434,19 +3421,19 @@
         <v>5,0</v>
       </c>
       <c r="H80" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I80" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/dra.carolinelopess?igshid=MzMyNGUyNmU2YQ==</v>
       </c>
       <c r="J80" t="str">
-        <v>https://wa.me/5511969170606?text=Ol%C3%A1%2C%20Dra.%20Caroline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Caroline%20Lopes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11969170606?text=Ol%C3%A1%2C%20Dra.%20Caroline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Caroline%20Lopes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K80" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Caroline! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Caroline Lopes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Caroline Lopes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="81" xml:space="preserve">
@@ -3472,19 +3459,19 @@
         <v>5,0</v>
       </c>
       <c r="H81" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I81" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra.micheleneri?igsh=ajcyeXp0Nm1xM3Zk&amp;utm_source=qr</v>
       </c>
       <c r="J81" t="str">
-        <v>https://wa.me/5511942945433?text=Ol%C3%A1%2C%20Dra.%20Michele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Michele%20Neri%20%E2%80%93%20Harmoniza%C3%A7%C3%A3o%20Facial%20%26%20Corporal%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11942945433?text=Ol%C3%A1%2C%20Dra.%20Michele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Michele%20Neri%20%E2%80%93%20Harmoniza%C3%A7%C3%A3o%20Facial%20%26%20Corporal%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K81" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Michele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Michele Neri – Harmonização Facial &amp; Corporal | Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Michele Neri – Harmonização Facial &amp; Corporal | Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="82" xml:space="preserve">
@@ -3510,19 +3497,19 @@
         <v>5,0</v>
       </c>
       <c r="H82" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I82" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>http://www.instagram.com/draandressalopes</v>
       </c>
       <c r="J82" t="str">
-        <v>https://wa.me/5511932253874?text=Ol%C3%A1%2C%20Dra%20Andressa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Andressa%20Lopes%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11932253874?text=Ol%C3%A1%2C%20Dra%20Andressa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Andressa%20Lopes%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K82" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Andressa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Andressa Lopes - Harmonização Facial, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Andressa Lopes - Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="83" xml:space="preserve">
@@ -3548,19 +3535,19 @@
         <v>5,0</v>
       </c>
       <c r="H83" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I83" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/drasuellenalbuquerque/</v>
       </c>
       <c r="J83" t="str">
-        <v>https://wa.me/5511918467067?text=Ol%C3%A1%2C%20Dra%20Su%C3%A9llen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Su%C3%A9llen%20Albuquerque%20-%20Cl%C3%ADnica%20de%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11918467067?text=Ol%C3%A1%2C%20Dra%20Su%C3%A9llen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Su%C3%A9llen%20Albuquerque%20-%20Cl%C3%ADnica%20de%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K83" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Suéllen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Suéllen Albuquerque - Clínica de Harmonização Facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Suéllen Albuquerque - Clínica de Harmonização Facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="84" xml:space="preserve">
@@ -3586,19 +3573,19 @@
         <v>5,0</v>
       </c>
       <c r="H84" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I84" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dratalita.trevisan/</v>
       </c>
       <c r="J84" t="str">
-        <v>https://wa.me/5511913257440?text=Ol%C3%A1%2C%20Dra%20Talita!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Talita%20Trevisan%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11913257440?text=Ol%C3%A1%2C%20Dra%20Talita!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Talita%20Trevisan%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K84" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Talita! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Talita Trevisan | Harmonização facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Talita Trevisan | Harmonização facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="85" xml:space="preserve">
@@ -3624,19 +3611,19 @@
         <v>5,0</v>
       </c>
       <c r="H85" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I85" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dragreicekelli?igsh=MWFicHZibDl6bjJ3dw%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J85" t="str">
-        <v>https://wa.me/5511999627447?text=Ol%C3%A1%2C%20Dra.%20Greice!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Greice%20Keli-%20Est%C3%A9tica%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11999627447?text=Ol%C3%A1%2C%20Dra.%20Greice!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Greice%20Keli-%20Est%C3%A9tica%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K85" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Greice! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Greice Keli- Estética e Harmonização Facial no Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Greice Keli- Estética e Harmonização Facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -3662,19 +3649,19 @@
         <v>5,0</v>
       </c>
       <c r="H86" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I86" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>https://linktr.ee/dra.cristinaizabel.s</v>
       </c>
       <c r="J86" t="str">
-        <v>https://wa.me/5511962892115?text=Ol%C3%A1%2C%20Dra.%20Cristina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cristina%20Silva%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11962892115?text=Ol%C3%A1%2C%20Dra.%20Cristina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cristina%20Silva%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K86" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Cristina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cristina Silva - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cristina Silva - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -3700,19 +3687,19 @@
         <v>4,9</v>
       </c>
       <c r="H87" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I87" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/yvya_estetica/</v>
       </c>
       <c r="J87" t="str">
-        <v>https://wa.me/5511975740970?text=Ol%C3%A1%2C%20YvYa%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20YvYa%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20em%20Perdizes%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Limpeza%20de%20Pele%20%7C%20Preenchimento%20Facial%20%7C%20Ultrassom%20Microfocado%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975740970?text=Ol%C3%A1%2C%20YvYa%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20YvYa%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20em%20Perdizes%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Limpeza%20de%20Pele%20%7C%20Preenchimento%20Facial%20%7C%20Ultrassom%20Microfocado%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K87" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, YvYa Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para YvYa Clínica de Estética em Perdizes | Harmonização Facial | Limpeza de Pele | Preenchimento Facial | Ultrassom Microfocado, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para YvYa Clínica de Estética em Perdizes | Harmonização Facial | Limpeza de Pele | Preenchimento Facial | Ultrassom Microfocado, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="88" xml:space="preserve">
@@ -3738,19 +3725,19 @@
         <v>5,0</v>
       </c>
       <c r="H88" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I88" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J88" t="str">
-        <v>https://wa.me/5511913567195?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20avan%C3%A7ada%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11913567195?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20avan%C3%A7ada%20Perdizes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K88" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica Estética! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Estética avançada Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Estética avançada Perdizes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="89" xml:space="preserve">
@@ -3776,19 +3763,19 @@
         <v>5,0</v>
       </c>
       <c r="H89" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I89" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J89" t="str">
-        <v>https://wa.me/5511914800366?text=Ol%C3%A1%2C%20FIG%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20FIG%20Clinic%20-%20Dra.%20Manuela%20de%20Souza%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11914800366?text=Ol%C3%A1%2C%20FIG%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20FIG%20Clinic%20-%20Dra.%20Manuela%20de%20Souza%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K89" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, FIG Clinic! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para FIG Clinic - Dra. Manuela de Souza, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para FIG Clinic - Dra. Manuela de Souza, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -3814,19 +3801,19 @@
         <v>5,0</v>
       </c>
       <c r="H90" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I90" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dramadigiacomo?igsh=MTQzcHJnaXMxYnpiMQ==&amp;utm_source=qr</v>
       </c>
       <c r="J90" t="str">
-        <v>https://wa.me/5511972848524?text=Ol%C3%A1%2C%20Dra.%20Marcela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcela%20Di%20Giacomo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972848524?text=Ol%C3%A1%2C%20Dra.%20Marcela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcela%20Di%20Giacomo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K90" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Marcela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcela Di Giacomo - Estética Avançada, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcela Di Giacomo - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="91" xml:space="preserve">
@@ -3852,19 +3839,19 @@
         <v>5,0</v>
       </c>
       <c r="H91" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I91" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/dra.clairpessoa/</v>
       </c>
       <c r="J91" t="str">
-        <v>https://wa.me/5511954221740?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Facial!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Est%C3%A9tica%20Facial%20%26%20Rejuvenescimento%20%7C%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11954221740?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Facial!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Est%C3%A9tica%20Facial%20%26%20Rejuvenescimento%20%7C%20Perdizes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K91" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Estética Facial! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Estética Facial &amp; Rejuvenescimento | Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Estética Facial &amp; Rejuvenescimento | Perdizes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="92" xml:space="preserve">
@@ -3890,19 +3877,19 @@
         <v>4,2</v>
       </c>
       <c r="H92" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I92" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/ana-regina-alencar-santos/dermatologista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=50473&amp;utm_content=website</v>
       </c>
       <c r="J92" t="str">
-        <v>https://wa.me/5511960447173?text=Ol%C3%A1%2C%20Dra.%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C2%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Ana%20Regina%20Alencar%20Santos%2C%20Dermatologista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11960447173?text=Ol%C3%A1%2C%20Dra.%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C2%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Ana%20Regina%20Alencar%20Santos%2C%20Dermatologista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K92" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Ana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,2★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Ana Regina Alencar Santos, Dermatologista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,2★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Ana Regina Alencar Santos, Dermatologista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="93" xml:space="preserve">
@@ -3928,19 +3915,19 @@
         <v>5,0</v>
       </c>
       <c r="H93" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I93" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J93" t="str">
-        <v>https://wa.me/5511910324225?text=Ol%C3%A1%2C%20Dra%20Elisabeth!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Elisabeth%20Silveira%20-%20Dermatologia%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11910324225?text=Ol%C3%A1%2C%20Dra%20Elisabeth!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Elisabeth%20Silveira%20-%20Dermatologia%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K93" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Elisabeth! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Elisabeth Silveira - Dermatologia em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Elisabeth Silveira - Dermatologia em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="94" xml:space="preserve">
@@ -3966,19 +3953,19 @@
         <v>4,8</v>
       </c>
       <c r="H94" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I94" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J94" t="str">
-        <v>https://wa.me/5511993053569?text=Ol%C3%A1%2C%20Fernanda%20Lima!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Lima%20Queiroz%20Noya%20de%20Abreu%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993053569?text=Ol%C3%A1%2C%20Fernanda%20Lima!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Lima%20Queiroz%20Noya%20de%20Abreu%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K94" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Fernanda Lima! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Lima Queiroz Noya de Abreu, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Lima Queiroz Noya de Abreu, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="95" xml:space="preserve">
@@ -4004,19 +3991,19 @@
         <v>5,0</v>
       </c>
       <c r="H95" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I95" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/nutri.malubraidotti/</v>
       </c>
       <c r="J95" t="str">
-        <v>https://wa.me/5511945167295?text=Ol%C3%A1%2C%20Malu!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Malu%20Braidotti%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945167295?text=Ol%C3%A1%2C%20Malu!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Malu%20Braidotti%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K95" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Malu! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Malu Braidotti, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Malu Braidotti, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="96" xml:space="preserve">
@@ -4042,19 +4029,19 @@
         <v>5,0</v>
       </c>
       <c r="H96" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I96" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J96" t="str">
-        <v>https://wa.me/5511937287838?text=Ol%C3%A1%2C%20Centro%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20de%20Nutri%C3%A7%C3%A3o%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11937287838?text=Ol%C3%A1%2C%20Centro%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20de%20Nutri%C3%A7%C3%A3o%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K96" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Centro Nutrição! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro de Nutrição, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro de Nutrição, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="97" xml:space="preserve">
@@ -4080,19 +4067,19 @@
         <v>5,0</v>
       </c>
       <c r="H97" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I97" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J97" t="str">
-        <v>https://wa.me/5511997196772?text=Ol%C3%A1%2C%20Nutri%C3%A7%C3%A3o%20Personalizada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutri%C3%A7%C3%A3o%20Personalizada%20-%20Dra%20Fab%C3%ADola%20Estela%20Domingues%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11997196772?text=Ol%C3%A1%2C%20Nutri%C3%A7%C3%A3o%20Personalizada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutri%C3%A7%C3%A3o%20Personalizada%20-%20Dra%20Fab%C3%ADola%20Estela%20Domingues%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K97" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Nutrição Personalizada! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutrição Personalizada - Dra Fabíola Estela Domingues, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutrição Personalizada - Dra Fabíola Estela Domingues, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="98" xml:space="preserve">
@@ -4118,19 +4105,19 @@
         <v>5,0</v>
       </c>
       <c r="H98" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I98" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J98" t="str">
-        <v>https://wa.me/5511985928451?text=Ol%C3%A1%2C%20Esportivo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportivo%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11985928451?text=Ol%C3%A1%2C%20Esportivo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportivo%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K98" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Esportivo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportivo em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportivo em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="99" xml:space="preserve">
@@ -4156,19 +4143,19 @@
         <v>4,1</v>
       </c>
       <c r="H99" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I99" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J99" t="str">
-        <v>https://wa.me/5511974981031?text=Ol%C3%A1%2C%20Wesen%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C1%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Wesen%20Cl%C3%ADnica%20de%20Emagrecimento%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11974981031?text=Ol%C3%A1%2C%20Wesen%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C1%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Wesen%20Cl%C3%ADnica%20de%20Emagrecimento%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K99" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Wesen Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 4,1★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Wesen Clínica de Emagrecimento, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 4,1★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Wesen Clínica de Emagrecimento, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="100" xml:space="preserve">
@@ -4194,19 +4181,19 @@
         <v>5,0</v>
       </c>
       <c r="H100" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I100" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/larissafranco.nutri?igsh=MTE1MGZjenZvY3g3cw%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J100" t="str">
-        <v>https://wa.me/5511988957410?text=Ol%C3%A1%2C%20Larissa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Larissa%20Franco%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11988957410?text=Ol%C3%A1%2C%20Larissa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Larissa%20Franco%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K100" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Larissa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Larissa Franco, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Larissa Franco, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="101" xml:space="preserve">
@@ -4232,19 +4219,19 @@
         <v>5,0</v>
       </c>
       <c r="H101" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I101" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J101" t="str">
-        <v>https://wa.me/5511922183012?text=Ol%C3%A1%2C%20Larissa%20Monteiro!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Larissa%20Monteiro%20Nutricionista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11922183012?text=Ol%C3%A1%2C%20Larissa%20Monteiro!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Larissa%20Monteiro%20Nutricionista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K101" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Larissa Monteiro! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Larissa Monteiro Nutricionista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Larissa Monteiro Nutricionista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="102" xml:space="preserve">
@@ -4270,19 +4257,19 @@
         <v>5,0</v>
       </c>
       <c r="H102" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I102" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/nathalia.nutri/</v>
       </c>
       <c r="J102" t="str">
-        <v>https://wa.me/5511976575363?text=Ol%C3%A1%2C%20nos!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20nos%20Jardins%20-%20Nath%C3%A1lia%20D'Abruzzo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976575363?text=Ol%C3%A1%2C%20nos!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20nos%20Jardins%20-%20Nath%C3%A1lia%20D'Abruzzo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K102" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, nos! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista nos Jardins - Nathália D'Abruzzo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista nos Jardins - Nathália D'Abruzzo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="103" xml:space="preserve">
@@ -4308,19 +4295,19 @@
         <v>5,0</v>
       </c>
       <c r="H103" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I103" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/marisa-graca/nutricionista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=705957&amp;utm_content=website</v>
       </c>
       <c r="J103" t="str">
-        <v>https://wa.me/5511934427007?text=Ol%C3%A1%2C%20Dra.%20Marisa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marisa%20Diniz%20Gra%C3%A7a%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11934427007?text=Ol%C3%A1%2C%20Dra.%20Marisa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marisa%20Diniz%20Gra%C3%A7a%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K103" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra. Marisa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marisa Diniz Graça, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marisa Diniz Graça, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="104" xml:space="preserve">
@@ -4346,19 +4333,19 @@
         <v>5,0</v>
       </c>
       <c r="H104" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I104" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/5511921795550?text=Ol%C3%A1!%20Vim%20pelo%20Google%20e%20gostaria%20de%20mais%20informa%C3%A7%C3%B5es%20sobre%20a%20consulta%20nutricional!</v>
       </c>
       <c r="J104" t="str">
-        <v>https://wa.me/5511921795550?text=Ol%C3%A1%2C%20Rafael%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Rafael%20Morais%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11921795550?text=Ol%C3%A1%2C%20Rafael%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Rafael%20Morais%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K104" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Rafael Morais! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Rafael Morais, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Rafael Morais, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="105" xml:space="preserve">
@@ -4384,19 +4371,19 @@
         <v>5,0</v>
       </c>
       <c r="H105" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I105" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J105" t="str">
-        <v>https://wa.me/5511980982327?text=Ol%C3%A1%2C%20Dra%20Daniela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Daniela%20Mendon%C3%A7a%20-%20Nutricionista%20Esportiva%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11980982327?text=Ol%C3%A1%2C%20Dra%20Daniela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Daniela%20Mendon%C3%A7a%20-%20Nutricionista%20Esportiva%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K105" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Daniela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Daniela Mendonça - Nutricionista Esportiva, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Daniela Mendonça - Nutricionista Esportiva, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="106" xml:space="preserve">
@@ -4422,19 +4409,19 @@
         <v>5,0</v>
       </c>
       <c r="H106" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I106" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/5511964236252</v>
       </c>
       <c r="J106" t="str">
-        <v>https://wa.me/5511964236252?text=Ol%C3%A1%2C%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Jo%C3%A3o%20Pinheiro%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964236252?text=Ol%C3%A1%2C%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Jo%C3%A3o%20Pinheiro%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K106" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, João! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista João Pinheiro, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista João Pinheiro, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="107" xml:space="preserve">
@@ -4460,19 +4447,19 @@
         <v>5,0</v>
       </c>
       <c r="H107" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I107" t="str">
-        <v>Sem site próprio (Apenas api)</v>
+        <v>https://api.whatsapp.com/send?phone=5511981267772&amp;text=Ol%C3%A1%2C%20Andrea!%20Te%20encontrei%20no%20Google%20e%20gostaria%20de%20mais%20informa%C3%A7%C3%B5es%20sobre%20a%20consulta%20com%20voc%C3%AA.%20Obrigado.</v>
       </c>
       <c r="J107" t="str">
-        <v>https://wa.me/5511981267772?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Andrea%20Garrett%20Nutricionista%20no%20Itaim%20Bibi%20CRN3%2090979%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11981267772?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Andrea%20Garrett%20Nutricionista%20no%20Itaim%20Bibi%20CRN3%2090979%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K107" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Andrea Garrett Nutricionista no Itaim Bibi CRN3 90979, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Andrea Garrett Nutricionista no Itaim Bibi CRN3 90979, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="108" xml:space="preserve">
@@ -4498,19 +4485,19 @@
         <v>5,0</v>
       </c>
       <c r="H108" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I108" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/nutricionistaveronicanovais/</v>
       </c>
       <c r="J108" t="str">
-        <v>https://wa.me/5511952251414?text=Ol%C3%A1%2C%20Ver%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ver%C3%B4nica%20Novais%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11952251414?text=Ol%C3%A1%2C%20Ver%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ver%C3%B4nica%20Novais%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K108" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Verônica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Verônica Novais, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Verônica Novais, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="109" xml:space="preserve">
@@ -4536,19 +4523,19 @@
         <v>5,0</v>
       </c>
       <c r="H109" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I109" t="str">
-        <v>Sem site próprio (Apenas api)</v>
+        <v>https://api.whatsapp.com/send?phone=5511972163767</v>
       </c>
       <c r="J109" t="str">
-        <v>https://wa.me/5511972163767?text=Ol%C3%A1%2C%20Yuri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Yuri%20Gomes%20-%20Nutricionista%20Esportivo%20em%20Pinheiros%2C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972163767?text=Ol%C3%A1%2C%20Yuri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Yuri%20Gomes%20-%20Nutricionista%20Esportivo%20em%20Pinheiros%2C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K109" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Yuri! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Yuri Gomes - Nutricionista Esportivo em Pinheiros, São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Yuri Gomes - Nutricionista Esportivo em Pinheiros, São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="110" xml:space="preserve">
@@ -4574,19 +4561,19 @@
         <v>5,0</v>
       </c>
       <c r="H110" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I110" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/ellen-cortezi/nutricionista/sao-paulo</v>
       </c>
       <c r="J110" t="str">
-        <v>https://wa.me/5511971308828?text=Ol%C3%A1%2C%20Ellen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ellen%20Hiromi%20Cortezi%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11971308828?text=Ol%C3%A1%2C%20Ellen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ellen%20Hiromi%20Cortezi%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K110" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Ellen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Ellen Hiromi Cortezi, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Ellen Hiromi Cortezi, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="111" xml:space="preserve">
@@ -4612,19 +4599,19 @@
         <v>5,0</v>
       </c>
       <c r="H111" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I111" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J111" t="str">
-        <v>https://wa.me/5511982923609?text=Ol%C3%A1%2C%20Aline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Aline%20Rodrigues%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11982923609?text=Ol%C3%A1%2C%20Aline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Aline%20Rodrigues%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K111" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Aline! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Aline Rodrigues, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Aline Rodrigues, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="112" xml:space="preserve">
@@ -4650,19 +4637,19 @@
         <v>5,0</v>
       </c>
       <c r="H112" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I112" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/mayrachamas?igsh=MXN2M2xyeXB4Z28xcw%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J112" t="str">
-        <v>https://wa.me/5511995262251?text=Ol%C3%A1%2C%20Mayra%20Chamas!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mayra%20Chamas%20Nutricionista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11995262251?text=Ol%C3%A1%2C%20Mayra%20Chamas!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mayra%20Chamas%20Nutricionista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K112" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Mayra Chamas! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mayra Chamas Nutricionista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mayra Chamas Nutricionista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="113" xml:space="preserve">
@@ -4688,19 +4675,19 @@
         <v>5,0</v>
       </c>
       <c r="H113" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I113" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J113" t="str">
-        <v>https://wa.me/5511948082545?text=Ol%C3%A1%2C%20Mariana%20Sena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Sena%20-%20Nutricionista%20Cl%C3%ADnica%20Funcional%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11948082545?text=Ol%C3%A1%2C%20Mariana%20Sena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Sena%20-%20Nutricionista%20Cl%C3%ADnica%20Funcional%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K113" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Mariana Sena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Sena - Nutricionista Clínica Funcional, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Sena - Nutricionista Clínica Funcional, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="114" xml:space="preserve">
@@ -4726,19 +4713,19 @@
         <v>5,0</v>
       </c>
       <c r="H114" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I114" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/nutri_primazza/?hl=pt-br</v>
       </c>
       <c r="J114" t="str">
-        <v>https://wa.me/5511996792653?text=Ol%C3%A1%2C%20Vegetariana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Vegetariana%2F%20Vegana%20Priscilla%20Mazza%20(Vila%20Mariana)%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11996792653?text=Ol%C3%A1%2C%20Vegetariana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Vegetariana%2F%20Vegana%20Priscilla%20Mazza%20(Vila%20Mariana)%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K114" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Vegetariana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Vegetariana/ Vegana Priscilla Mazza (Vila Mariana), pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Vegetariana/ Vegana Priscilla Mazza (Vila Mariana), pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="115" xml:space="preserve">
@@ -4764,19 +4751,19 @@
         <v>5,0</v>
       </c>
       <c r="H115" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I115" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J115" t="str">
-        <v>https://wa.me/5511942228782?text=Ol%C3%A1%2C%20Priscila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Priscila%20Raso%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11942228782?text=Ol%C3%A1%2C%20Priscila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Priscila%20Raso%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K115" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Priscila! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Priscila Raso, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Priscila Raso, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="116" xml:space="preserve">
@@ -4802,19 +4789,19 @@
         <v>5,0</v>
       </c>
       <c r="H116" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I116" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J116" t="str">
-        <v>https://wa.me/5511947936739?text=Ol%C3%A1%2C%20Camila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Camila%20Hidani%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11947936739?text=Ol%C3%A1%2C%20Camila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Camila%20Hidani%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K116" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Camila! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Camila Hidani, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Camila Hidani, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="117" xml:space="preserve">
@@ -4840,19 +4827,19 @@
         <v>5,0</v>
       </c>
       <c r="H117" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I117" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J117" t="str">
-        <v>https://wa.me/5511989456640?text=Ol%C3%A1%2C%20Dra%20Pollana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Pollana%20Campos%20Moreira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11989456640?text=Ol%C3%A1%2C%20Dra%20Pollana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Pollana%20Campos%20Moreira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K117" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra Pollana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Pollana Campos Moreira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Pollana Campos Moreira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="118" xml:space="preserve">
@@ -4878,19 +4865,19 @@
         <v>5,0</v>
       </c>
       <c r="H118" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Subdomínio Wix gratuito)</v>
       </c>
       <c r="I118" t="str">
-        <v>Sem site próprio (Apenas wixsite)</v>
+        <v>https://julianagasulla.wixsite.com/nutricao</v>
       </c>
       <c r="J118" t="str">
-        <v>https://wa.me/5511975438419?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportiva%20Tatuap%C3%A9%20-%20Juliana%20Gasulla%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975438419?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportiva%20Tatuap%C3%A9%20-%20Juliana%20Gasulla%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K118" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Esportiva! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportiva Tatuapé - Juliana Gasulla, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportiva Tatuapé - Juliana Gasulla, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="119" xml:space="preserve">
@@ -4916,19 +4903,19 @@
         <v>5,0</v>
       </c>
       <c r="H119" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I119" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J119" t="str">
-        <v>https://wa.me/5511950262944?text=Ol%C3%A1%2C%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Cl%C3%ADnica%20e%20Esportiva%20-%20Mariana%20Saito%20-%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11950262944?text=Ol%C3%A1%2C%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Cl%C3%ADnica%20e%20Esportiva%20-%20Mariana%20Saito%20-%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K119" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Clínica e Esportiva - Mariana Saito - Tatuapé, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Clínica e Esportiva - Mariana Saito - Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="120" xml:space="preserve">
@@ -4954,19 +4941,19 @@
         <v>4,8</v>
       </c>
       <c r="H120" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I120" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/nutrijessicanogueira?r=nametag</v>
       </c>
       <c r="J120" t="str">
-        <v>https://wa.me/5511940152184?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20no%20Tatuap%C3%A9%20%7C%20J%C3%A9ssica%20Nogueira%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11940152184?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20no%20Tatuap%C3%A9%20%7C%20J%C3%A9ssica%20Nogueira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K120" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista no Tatuapé | Jéssica Nogueira, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista no Tatuapé | Jéssica Nogueira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="121" xml:space="preserve">
@@ -4992,19 +4979,19 @@
         <v>5,0</v>
       </c>
       <c r="H121" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I121" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/message/5PEST3D4ANFQB1</v>
       </c>
       <c r="J121" t="str">
-        <v>https://wa.me/5511976671105?text=Ol%C3%A1%2C%20Jessica%20Nascimento!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Jessica%20Nascimento%20%7C%20Nutricionista%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976671105?text=Ol%C3%A1%2C%20Jessica%20Nascimento!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Jessica%20Nascimento%20%7C%20Nutricionista%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K121" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Jessica Nascimento! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Jessica Nascimento | Nutricionista Tatuapé SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Jessica Nascimento | Nutricionista Tatuapé SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="122" xml:space="preserve">
@@ -5030,19 +5017,19 @@
         <v>5,0</v>
       </c>
       <c r="H122" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I122" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/nutrijulialinhares/</v>
       </c>
       <c r="J122" t="str">
-        <v>https://wa.me/5511933768718?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Julia%20Linhares%20-%20Cl%C3%ADnica%20e%20Esportiva%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11933768718?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Julia%20Linhares%20-%20Cl%C3%ADnica%20e%20Esportiva%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K122" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Julia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Julia Linhares - Clínica e Esportiva, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Julia Linhares - Clínica e Esportiva, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="123" xml:space="preserve">
@@ -5068,19 +5055,19 @@
         <v>4,0</v>
       </c>
       <c r="H123" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I123" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/susan-franca-guimaraes/nutricionista/sao-paulo</v>
       </c>
       <c r="J123" t="str">
-        <v>https://wa.me/5511993881567?text=Ol%C3%A1%2C%20Tatuap%C3%A9!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Tatuap%C3%A9%20%7C%20Susan%20Fran%C3%A7a%20Guimar%C3%A3es%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993881567?text=Ol%C3%A1%2C%20Tatuap%C3%A9!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Tatuap%C3%A9%20%7C%20Susan%20Fran%C3%A7a%20Guimar%C3%A3es%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K123" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Tatuapé! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 4,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Tatuapé | Susan França Guimarães, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 4,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Tatuapé | Susan França Guimarães, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="124" xml:space="preserve">
@@ -5106,19 +5093,19 @@
         <v>5,0</v>
       </c>
       <c r="H124" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I124" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>http://linktr.ee/victorpiekny</v>
       </c>
       <c r="J124" t="str">
-        <v>https://wa.me/5511942591826?text=Ol%C3%A1%2C%20Victor!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Victor%20Piekny%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11942591826?text=Ol%C3%A1%2C%20Victor!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Victor%20Piekny%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K124" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Victor! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Victor Piekny, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Victor Piekny, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="125" xml:space="preserve">
@@ -5144,19 +5131,19 @@
         <v>5,0</v>
       </c>
       <c r="H125" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I125" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>http://instagram.com/nutri.bruantonietti</v>
       </c>
       <c r="J125" t="str">
-        <v>https://wa.me/5511951573284?text=Ol%C3%A1%2C%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Bruna%20Antonietti%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951573284?text=Ol%C3%A1%2C%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Bruna%20Antonietti%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K125" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Bruna Antonietti, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Bruna Antonietti, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="126" xml:space="preserve">
@@ -5182,19 +5169,19 @@
         <v>5,0</v>
       </c>
       <c r="H126" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I126" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J126" t="str">
-        <v>https://wa.me/5511976893728?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Nutri%C3%A7%C3%A3o%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976893728?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Nutri%C3%A7%C3%A3o%20Perdizes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K126" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica Nutrição! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Nutrição Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Nutrição Perdizes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="127" xml:space="preserve">
@@ -5220,19 +5207,19 @@
         <v>5,0</v>
       </c>
       <c r="H127" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I127" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://instagram.com/monicaunzueta.nutri?igshid=1glrwzy5tmocd</v>
       </c>
       <c r="J127" t="str">
-        <v>https://wa.me/5511932300359?text=Ol%C3%A1%2C%20Emagrecimento%20Sa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Emagrecimento%20e%20Sa%C3%BAde%20da%20Mulher%2035%2B%20%7C%20Nutricionista%20Monica%20Valeria%20Palenque%20Unzueta%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11932300359?text=Ol%C3%A1%2C%20Emagrecimento%20Sa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Emagrecimento%20e%20Sa%C3%BAde%20da%20Mulher%2035%2B%20%7C%20Nutricionista%20Monica%20Valeria%20Palenque%20Unzueta%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K127" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Emagrecimento Saúde! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Emagrecimento e Saúde da Mulher 35+ | Nutricionista Monica Valeria Palenque Unzueta, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Emagrecimento e Saúde da Mulher 35+ | Nutricionista Monica Valeria Palenque Unzueta, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="128" xml:space="preserve">
@@ -5258,19 +5245,19 @@
         <v>5,0</v>
       </c>
       <c r="H128" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I128" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J128" t="str">
-        <v>https://wa.me/5511916477655?text=Ol%C3%A1%2C%20Dra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Dra%20Patr%C3%ADcia%20Neri%20Cavalcanti%20%7C%20Transformo%20a%20Sa%C3%BAde%20de%20Mulheres%20com%20Ci%C3%AAncia%20e%20Acolhimento.%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11916477655?text=Ol%C3%A1%2C%20Dra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Dra%20Patr%C3%ADcia%20Neri%20Cavalcanti%20%7C%20Transformo%20a%20Sa%C3%BAde%20de%20Mulheres%20com%20Ci%C3%AAncia%20e%20Acolhimento.%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K128" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Dra! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Dra Patrícia Neri Cavalcanti | Transformo a Saúde de Mulheres com Ciência e Acolhimento., pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Dra Patrícia Neri Cavalcanti | Transformo a Saúde de Mulheres com Ciência e Acolhimento., pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="129" xml:space="preserve">
@@ -5296,19 +5283,19 @@
         <v>5,0</v>
       </c>
       <c r="H129" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I129" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J129" t="str">
-        <v>https://wa.me/5511992192552?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Camila%20Moreira%20Nutricionista%20Esportiva%20Funcional%20-%20Cl%C3%ADnica%20Endocor%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11992192552?text=Ol%C3%A1%2C%20Esportiva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Camila%20Moreira%20Nutricionista%20Esportiva%20Funcional%20-%20Cl%C3%ADnica%20Endocor%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K129" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Esportiva! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Camila Moreira Nutricionista Esportiva Funcional - Clínica Endocor, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Camila Moreira Nutricionista Esportiva Funcional - Clínica Endocor, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="130" xml:space="preserve">
@@ -5334,19 +5321,19 @@
         <v>5,0</v>
       </c>
       <c r="H130" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I130" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J130" t="str">
-        <v>https://wa.me/5511932613077?text=Ol%C3%A1%2C%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Helena%20Fioravanti%20%7C%20Nutricionista%20em%20Perdizes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11932613077?text=Ol%C3%A1%2C%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Helena%20Fioravanti%20%7C%20Nutricionista%20em%20Perdizes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K130" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Helena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Helena Fioravanti | Nutricionista em Perdizes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Nutrição em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Helena Fioravanti | Nutricionista em Perdizes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="131" xml:space="preserve">
@@ -5372,19 +5359,19 @@
         <v>5,0</v>
       </c>
       <c r="H131" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I131" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J131" t="str">
-        <v>https://wa.me/5511972437354?text=Ol%C3%A1%2C%20Psi%20Yara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psi%20Yara%20Rodrigues%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972437354?text=Ol%C3%A1%2C%20Psi%20Yara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psi%20Yara%20Rodrigues%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K131" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Psi Yara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psi Yara Rodrigues, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psi Yara Rodrigues, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="132" xml:space="preserve">
@@ -5410,19 +5397,19 @@
         <v>5,0</v>
       </c>
       <c r="H132" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I132" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J132" t="str">
-        <v>https://wa.me/5511995828384?text=Ol%C3%A1%2C%20Luciane%20Bonfanti!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Luciane%20Bonfanti%20%7C%20Psic%C3%B3loga%20em%20Moema%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11995828384?text=Ol%C3%A1%2C%20Luciane%20Bonfanti!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Luciane%20Bonfanti%20%7C%20Psic%C3%B3loga%20em%20Moema%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K132" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Luciane Bonfanti! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Luciane Bonfanti | Psicóloga em Moema, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Luciane Bonfanti | Psicóloga em Moema, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="133" xml:space="preserve">
@@ -5448,19 +5435,19 @@
         <v>5,0</v>
       </c>
       <c r="H133" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I133" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J133" t="str">
-        <v>https://wa.me/5511952911744?text=Ol%C3%A1%2C%20Mariana%20Honorio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Honorio%20Psicologa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11952911744?text=Ol%C3%A1%2C%20Mariana%20Honorio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Honorio%20Psicologa%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K133" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Mariana Honorio! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Honorio Psicologa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Honorio Psicologa, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="134" xml:space="preserve">
@@ -5486,19 +5473,19 @@
         <v>5,0</v>
       </c>
       <c r="H134" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Subdomínio Wix gratuito)</v>
       </c>
       <c r="I134" t="str">
-        <v>Sem site próprio (Apenas wixsite)</v>
+        <v>https://psicologatayane.wixsite.com/website</v>
       </c>
       <c r="J134" t="str">
-        <v>https://wa.me/5511961879290?text=Ol%C3%A1%2C%20Tayane%20Teizen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Tayane%20Teizen%20-%20Psic%C3%B3loga%20Psicodin%C3%A2mica%20Psicanal%C3%ADtica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11961879290?text=Ol%C3%A1%2C%20Tayane%20Teizen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Tayane%20Teizen%20-%20Psic%C3%B3loga%20Psicodin%C3%A2mica%20Psicanal%C3%ADtica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K134" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Tayane Teizen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Tayane Teizen - Psicóloga Psicodinâmica Psicanalítica, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Tayane Teizen - Psicóloga Psicodinâmica Psicanalítica, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="135" xml:space="preserve">
@@ -5524,19 +5511,19 @@
         <v>5,0</v>
       </c>
       <c r="H135" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I135" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J135" t="str">
-        <v>https://wa.me/5511989304882?text=Ol%C3%A1%2C%20Adele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Adele%20Cestari%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11989304882?text=Ol%C3%A1%2C%20Adele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Adele%20Cestari%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K135" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Adele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Adele Cestari, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Adele Cestari, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="136" xml:space="preserve">
@@ -5562,19 +5549,19 @@
         <v>5,0</v>
       </c>
       <c r="H136" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I136" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J136" t="str">
-        <v>https://wa.me/5511993376425?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20psicologia%20%7C%20Gabriela%20Vaz%20Grzegorzewska%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993376425?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20psicologia%20%7C%20Gabriela%20Vaz%20Grzegorzewska%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K136" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Clínica psicologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de psicologia | Gabriela Vaz Grzegorzewska, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de psicologia | Gabriela Vaz Grzegorzewska, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="137" xml:space="preserve">
@@ -5600,19 +5587,19 @@
         <v>5,0</v>
       </c>
       <c r="H137" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I137" t="str">
-        <v>Sem site próprio (Apenas linktr)</v>
+        <v>https://linktr.ee/psi.giopermac</v>
       </c>
       <c r="J137" t="str">
-        <v>https://wa.me/5511998106227?text=Ol%C3%A1%2C%20Giovana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Giovana%20Pereira%20Macedo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11998106227?text=Ol%C3%A1%2C%20Giovana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Giovana%20Pereira%20Macedo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K137" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Giovana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Giovana Pereira Macedo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Giovana Pereira Macedo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="138" xml:space="preserve">
@@ -5638,19 +5625,19 @@
         <v>5,0</v>
       </c>
       <c r="H138" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I138" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J138" t="str">
-        <v>https://wa.me/5511948764737?text=Ol%C3%A1%2C%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologia%20-%20Profa%20Dra%20Gabriella%20Alvarenga%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11948764737?text=Ol%C3%A1%2C%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologia%20-%20Profa%20Dra%20Gabriella%20Alvarenga%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K138" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Psicologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologia - Profa Dra Gabriella Alvarenga, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologia - Profa Dra Gabriella Alvarenga, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="139" xml:space="preserve">
@@ -5676,19 +5663,19 @@
         <v>5,0</v>
       </c>
       <c r="H139" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site próprio oficial</v>
       </c>
       <c r="I139" t="str">
-        <v>Sem site próprio (Apenas wa)</v>
+        <v>https://wa.me/5511943493132</v>
       </c>
       <c r="J139" t="str">
-        <v>https://wa.me/5511943493132?text=Ol%C3%A1%2C%20CLAUDIO%20CARLOS!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20CLAUDIO%20CARLOS%20DE%20SOUZA%20-%20Psic%C3%B3logo%20Jardins%20Av.%20Paulista%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11943493132?text=Ol%C3%A1%2C%20CLAUDIO%20CARLOS!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20CLAUDIO%20CARLOS%20DE%20SOUZA%20-%20Psic%C3%B3logo%20Jardins%20Av.%20Paulista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K139" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, CLAUDIO CARLOS! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para CLAUDIO CARLOS DE SOUZA - Psicólogo Jardins Av. Paulista, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para CLAUDIO CARLOS DE SOUZA - Psicólogo Jardins Av. Paulista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="140" xml:space="preserve">
@@ -5714,19 +5701,19 @@
         <v>5,0</v>
       </c>
       <c r="H140" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I140" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J140" t="str">
-        <v>https://wa.me/5511996717876?text=Ol%C3%A1%2C%20Psicologa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11996717876?text=Ol%C3%A1%2C%20Psicologa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologa%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K140" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Psicologa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologa, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="141" xml:space="preserve">
@@ -5752,19 +5739,19 @@
         <v>5,0</v>
       </c>
       <c r="H141" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I141" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J141" t="str">
-        <v>https://wa.me/5511994413787?text=Ol%C3%A1%2C%20Fortun%C3%A9e%20Josiane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fortun%C3%A9e%20Josiane%20Zagha%20-%20Psic%C3%B3loga%20e%20Psicoterapeuta%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11994413787?text=Ol%C3%A1%2C%20Fortun%C3%A9e%20Josiane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fortun%C3%A9e%20Josiane%20Zagha%20-%20Psic%C3%B3loga%20e%20Psicoterapeuta%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K141" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Fortunée Josiane! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fortunée Josiane Zagha - Psicóloga e Psicoterapeuta, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fortunée Josiane Zagha - Psicóloga e Psicoterapeuta, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="142" xml:space="preserve">
@@ -5790,19 +5777,19 @@
         <v>5,0</v>
       </c>
       <c r="H142" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I142" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J142" t="str">
-        <v>https://wa.me/5511974992088?text=Ol%C3%A1%2C%20Marcela%20Pitombo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Marcela%20Pitombo%20Seixas%20-%20Psicologia%20Cl%C3%ADnica%20e%20Neuropsicologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11974992088?text=Ol%C3%A1%2C%20Marcela%20Pitombo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Marcela%20Pitombo%20Seixas%20-%20Psicologia%20Cl%C3%ADnica%20e%20Neuropsicologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K142" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Marcela Pitombo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Marcela Pitombo Seixas - Psicologia Clínica e Neuropsicologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Marcela Pitombo Seixas - Psicologia Clínica e Neuropsicologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="143" xml:space="preserve">
@@ -5828,19 +5815,19 @@
         <v>5,0</v>
       </c>
       <c r="H143" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I143" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J143" t="str">
-        <v>https://wa.me/5511982031569?text=Ol%C3%A1%2C%20Patr%C3%ADcia%20Camelatto!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Patr%C3%ADcia%20Camelatto%20-%20Psic%C3%B3loga%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11982031569?text=Ol%C3%A1%2C%20Patr%C3%ADcia%20Camelatto!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Patr%C3%ADcia%20Camelatto%20-%20Psic%C3%B3loga%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K143" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Patrícia Camelatto! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Patrícia Camelatto - Psicóloga, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Patrícia Camelatto - Psicóloga, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="144" xml:space="preserve">
@@ -5866,19 +5853,19 @@
         <v>5,0</v>
       </c>
       <c r="H144" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I144" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J144" t="str">
-        <v>https://wa.me/5511981559609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20e%20Psicanalista%20Thaina%20Santos%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11981559609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20e%20Psicanalista%20Thaina%20Santos%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K144" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga e Psicanalista Thaina Santos, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga e Psicanalista Thaina Santos, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="145" xml:space="preserve">
@@ -5904,19 +5891,19 @@
         <v>5,0</v>
       </c>
       <c r="H145" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I145" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J145" t="str">
-        <v>https://wa.me/5511995316010?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cristina%20Galv%C3%A3o%20Psic%C3%B3loga%20e%20Neuropsic%C3%B3loga%20Pinheiros%2FSP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11995316010?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cristina%20Galv%C3%A3o%20Psic%C3%B3loga%20e%20Neuropsic%C3%B3loga%20Pinheiros%2FSP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K145" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cristina Galvão Psicóloga e Neuropsicóloga Pinheiros/SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cristina Galvão Psicóloga e Neuropsicóloga Pinheiros/SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="146" xml:space="preserve">
@@ -5942,19 +5929,19 @@
         <v>3,7</v>
       </c>
       <c r="H146" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I146" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J146" t="str">
-        <v>https://wa.me/5511986209818?text=Ol%C3%A1%2C%20Psicologia%20Pinheiros!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%203%2C7%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologia%20Pinheiros%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11986209818?text=Ol%C3%A1%2C%20Psicologia%20Pinheiros!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%203%2C7%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psicologia%20Pinheiros%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K146" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Psicologia Pinheiros! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 3,7★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologia Pinheiros, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 3,7★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicologia Pinheiros, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="147" xml:space="preserve">
@@ -5980,19 +5967,19 @@
         <v>5,0</v>
       </c>
       <c r="H147" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I147" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/z/YixYVw</v>
       </c>
       <c r="J147" t="str">
-        <v>https://wa.me/5511984804578?text=Ol%C3%A1%2C%20em!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20em%20Pinheiros%20-%20Elianai%20Holanda%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11984804578?text=Ol%C3%A1%2C%20em!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20em%20Pinheiros%20-%20Elianai%20Holanda%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K147" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, em! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga em Pinheiros - Elianai Holanda, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga em Pinheiros - Elianai Holanda, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="148" xml:space="preserve">
@@ -6018,19 +6005,19 @@
         <v>5,0</v>
       </c>
       <c r="H148" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Subdomínio Wix gratuito)</v>
       </c>
       <c r="I148" t="str">
-        <v>Sem site próprio (Apenas wixsite)</v>
+        <v>https://fernandaataidepsic.wixsite.com/my-site-1</v>
       </c>
       <c r="J148" t="str">
-        <v>https://wa.me/5511993286995?text=Ol%C3%A1%2C%20Fernanda%20Ataide!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Ataide%20Psicologa%20Cl%C3%ADnica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993286995?text=Ol%C3%A1%2C%20Fernanda%20Ataide!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Ataide%20Psicologa%20Cl%C3%ADnica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K148" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Fernanda Ataide! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Ataide Psicologa Clínica, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Ataide Psicologa Clínica, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="149" xml:space="preserve">
@@ -6056,19 +6043,19 @@
         <v>5,0</v>
       </c>
       <c r="H149" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I149" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J149" t="str">
-        <v>https://wa.me/5511917252484?text=Ol%C3%A1%2C%20ZIL%C3%81%20GUIMAR%C3%83ES!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20ZIL%C3%81%20GUIMAR%C3%83ES-%20PSIC%C3%93LOGA-%20SP%20ITAIM%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11917252484?text=Ol%C3%A1%2C%20ZIL%C3%81%20GUIMAR%C3%83ES!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20ZIL%C3%81%20GUIMAR%C3%83ES-%20PSIC%C3%93LOGA-%20SP%20ITAIM%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K149" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, ZILÁ GUIMARÃES! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para ZILÁ GUIMARÃES- PSICÓLOGA- SP ITAIM, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para ZILÁ GUIMARÃES- PSICÓLOGA- SP ITAIM, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="150" xml:space="preserve">
@@ -6094,19 +6081,19 @@
         <v>5,0</v>
       </c>
       <c r="H150" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I150" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J150" t="str">
-        <v>https://wa.me/5511964682000?text=Ol%C3%A1%2C%20Consultorio%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consultorio%20de%20Psicologia%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964682000?text=Ol%C3%A1%2C%20Consultorio%20Psicologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consultorio%20de%20Psicologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K150" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Consultorio Psicologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultorio de Psicologia, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultorio de Psicologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="151" xml:space="preserve">
@@ -6132,19 +6119,19 @@
         <v>5,0</v>
       </c>
       <c r="H151" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I151" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/eric-heibel/psicologo-psicanalista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=711270&amp;utm_content=website</v>
       </c>
       <c r="J151" t="str">
-        <v>https://wa.me/5511983831705?text=Ol%C3%A1%2C%20Eric%20Heibel%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Eric%20Heibel%2C%20Psic%C3%B3logo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11983831705?text=Ol%C3%A1%2C%20Eric%20Heibel%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Eric%20Heibel%2C%20Psic%C3%B3logo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K151" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Eric Heibel,! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Eric Heibel, Psicólogo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Eric Heibel, Psicólogo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="152" xml:space="preserve">
@@ -6170,19 +6157,19 @@
         <v>5,0</v>
       </c>
       <c r="H152" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I152" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/psicocamilasantos</v>
       </c>
       <c r="J152" t="str">
-        <v>https://wa.me/5511987335609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20e%20neuropsic%C3%B3loga%20Camila%20Santos%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11987335609?text=Ol%C3%A1%2C%20e!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20e%20neuropsic%C3%B3loga%20Camila%20Santos%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K152" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, e! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga e neuropsicóloga Camila Santos, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga e neuropsicóloga Camila Santos, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="153" xml:space="preserve">
@@ -6208,19 +6195,19 @@
         <v>5,0</v>
       </c>
       <c r="H153" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I153" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J153" t="str">
-        <v>https://wa.me/5511983635226?text=Ol%C3%A1%2C%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Ana%20Florentino%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11983635226?text=Ol%C3%A1%2C%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Ana%20Florentino%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K153" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Ana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Ana Florentino, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Ana Florentino, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="154" xml:space="preserve">
@@ -6246,19 +6233,19 @@
         <v>5,0</v>
       </c>
       <c r="H154" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I154" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/psicologasuzane/</v>
       </c>
       <c r="J154" t="str">
-        <v>https://wa.me/5511987797093?text=Ol%C3%A1%2C%20Suzane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Suzane%20Rayssa%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11987797093?text=Ol%C3%A1%2C%20Suzane!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Suzane%20Rayssa%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K154" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Suzane! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Suzane Rayssa, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Suzane Rayssa, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="155" xml:space="preserve">
@@ -6284,19 +6271,19 @@
         <v>5,0</v>
       </c>
       <c r="H155" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I155" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J155" t="str">
-        <v>https://wa.me/5511987208987?text=Ol%C3%A1%2C%20Lilian!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Lilian%20Izzo%20%7C%20Tatuap%C3%A9%20-%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11987208987?text=Ol%C3%A1%2C%20Lilian!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Lilian%20Izzo%20%7C%20Tatuap%C3%A9%20-%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K155" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Lilian! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Lilian Izzo | Tatuapé - São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Lilian Izzo | Tatuapé - São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="156" xml:space="preserve">
@@ -6322,19 +6309,19 @@
         <v>5,0</v>
       </c>
       <c r="H156" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I156" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/solangemedina.psico/</v>
       </c>
       <c r="J156" t="str">
-        <v>https://wa.me/5511982743076?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20no%20Tatuap%C3%A9%20SP%20%7C%20Terapia%20de%20Casal%2C%20Ansiedade%2C%20Depress%C3%A3o%20e%20Autoconhecimento%20-%20Solange%20Medina%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11982743076?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20no%20Tatuap%C3%A9%20SP%20%7C%20Terapia%20de%20Casal%2C%20Ansiedade%2C%20Depress%C3%A3o%20e%20Autoconhecimento%20-%20Solange%20Medina%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K156" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga no Tatuapé SP | Terapia de Casal, Ansiedade, Depressão e Autoconhecimento - Solange Medina, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga no Tatuapé SP | Terapia de Casal, Ansiedade, Depressão e Autoconhecimento - Solange Medina, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="157" xml:space="preserve">
@@ -6360,19 +6347,19 @@
         <v>5,0</v>
       </c>
       <c r="H157" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas Instagram/Linktree)</v>
       </c>
       <c r="I157" t="str">
-        <v>Sem site próprio (Apenas instagram)</v>
+        <v>https://www.instagram.com/psi.daylanesilva/</v>
       </c>
       <c r="J157" t="str">
-        <v>https://wa.me/5511983150090?text=Ol%C3%A1%2C%20Daylane%20Silva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Daylane%20Silva%20%7C%20Psic%C3%B3loga%20Cl%C3%ADnica%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11983150090?text=Ol%C3%A1%2C%20Daylane%20Silva!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Daylane%20Silva%20%7C%20Psic%C3%B3loga%20Cl%C3%ADnica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K157" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Daylane Silva! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Daylane Silva | Psicóloga Clínica, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Daylane Silva | Psicóloga Clínica, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="158" xml:space="preserve">
@@ -6398,19 +6385,19 @@
         <v>5,0</v>
       </c>
       <c r="H158" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I158" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J158" t="str">
-        <v>https://wa.me/5511974441262?text=Ol%C3%A1%2C%20La%C3%ADs%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20La%C3%ADs%20Fernandes%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11974441262?text=Ol%C3%A1%2C%20La%C3%ADs%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20La%C3%ADs%20Fernandes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K158" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Laís Fernandes! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Laís Fernandes, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Laís Fernandes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="159" xml:space="preserve">
@@ -6436,19 +6423,19 @@
         <v>5,0</v>
       </c>
       <c r="H159" t="str">
-        <v>Avaliações no Google</v>
+        <v>Sem site próprio (Apenas perfil Doctoralia)</v>
       </c>
       <c r="I159" t="str">
-        <v>Sem site próprio (Apenas doctoralia)</v>
+        <v>https://www.doctoralia.com.br/z/woij1Y</v>
       </c>
       <c r="J159" t="str">
-        <v>https://wa.me/5511994158972?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Julia%20Ribas%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11994158972?text=Ol%C3%A1%2C%20Julia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Julia%20Ribas%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K159" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Julia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Julia Ribas, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Julia Ribas, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="160" xml:space="preserve">
@@ -6474,19 +6461,19 @@
         <v>5,0</v>
       </c>
       <c r="H160" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I160" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J160" t="str">
-        <v>https://wa.me/5511987558867?text=Ol%C3%A1%2C%20Valquiria%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Valquiria%20Fernandes%20-%20Psic%C3%B3loga%20Integrativa%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11987558867?text=Ol%C3%A1%2C%20Valquiria%20Fernandes!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Valquiria%20Fernandes%20-%20Psic%C3%B3loga%20Integrativa%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K160" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Valquiria Fernandes! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Valquiria Fernandes - Psicóloga Integrativa em São Paulo, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Valquiria Fernandes - Psicóloga Integrativa em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
     <row r="161" xml:space="preserve">
@@ -6512,19 +6499,19 @@
         <v>5,0</v>
       </c>
       <c r="H161" t="str">
-        <v>Avaliações no Google</v>
+        <v>100% Sem site no Google (Zero Link)</v>
       </c>
       <c r="I161" t="str">
-        <v>Sem site próprio (Sem site cadastrado)</v>
+        <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J161" t="str">
-        <v>https://wa.me/5511987046526?text=Ol%C3%A1%2C%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pela%20reputa%C3%A7%C3%A3o%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Marina%20Araujo%20%7C%20Perdizes%20SP%2C%20pensado%20para%20apresentar%20seu%20trabalho%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20cadastrada%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11987046526?text=Ol%C3%A1%2C%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Psicologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Psic%C3%B3loga%20Marina%20Araujo%20%7C%20Perdizes%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
       </c>
       <c r="K161" t="str" xml:space="preserve">
         <v xml:space="preserve">Olá, Marina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pela reputação e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Marina Araujo | Perdizes SP, pensado para apresentar seu trabalho com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem uma página oficial própria cadastrada no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+Acompanho as referências de Psicologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
+Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Psicóloga Marina Araujo | Perdizes SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
+Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(prospeccao): aplica roteiro comercial focado em Perda de Dinheiro, Google x Instagram (marketing de intencao) e 50% OFF
</commit_message>
<xml_diff>
--- a/prospeccao_160_leads_sp.xlsx
+++ b/prospeccao_160_leads_sp.xlsx
@@ -463,13 +463,14 @@
         <v>https://linktr.ee/drafefernandes</v>
       </c>
       <c r="J2" t="str">
-        <v>https://wa.me/11991307186?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Fernandes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991307186?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Moema%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Fernandes%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K2" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Fernandes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Moema para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Fernanda Fernandes, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -501,13 +502,14 @@
         <v>https://linktr.ee/drasamaraoliveira_?utm_source=ig&amp;utm_medium=social&amp;utm_content=link_in_bio&amp;fbclid=PAZXh0bgNhZW0CMTEAc3J0YwZhcHBfaWQPOTM2NjE5NzQzMzkyNDU5AAGnfH1dXc14yvpmnoJ4k1irpfNClsn3d8yKB1Fov3MFQvQ8wKwpsOIMBgLt9XQ_aem_nMyhVMbErrB6Z85L6mXYkw</v>
       </c>
       <c r="J3" t="str">
-        <v>https://wa.me/11964799591?text=Ol%C3%A1%2C%20Dra.%20Samara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Samara%20Oliveira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964799591?text=Ol%C3%A1%2C%20Dra.%20Samara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Moema%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Samara%20Oliveira%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K3" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Samara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Samara Oliveira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Samara! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Moema para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Samara Oliveira, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="4" xml:space="preserve">
@@ -539,13 +541,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J4" t="str">
-        <v>https://wa.me/11940394742?text=Ol%C3%A1%2C%20Odontoreli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontoreli%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11940394742?text=Ol%C3%A1%2C%20Odontoreli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Moema%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Odontoreli%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K4" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontoreli! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontoreli, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Odontoreli! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Moema para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Odontoreli, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="5" xml:space="preserve">
@@ -577,13 +580,14 @@
         <v>https://www.doctoralia.com.br/marcia-ayres/dentista/sao-paulo</v>
       </c>
       <c r="J5" t="str">
-        <v>https://wa.me/11971268686?text=Ol%C3%A1%2C%20Dra.%20Marcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcia%20Ayres%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11971268686?text=Ol%C3%A1%2C%20Dra.%20Marcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Moema%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Marcia%20Ayres%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K5" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marcia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcia Ayres, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Marcia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Moema para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Marcia Ayres, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
@@ -615,13 +619,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J6" t="str">
-        <v>https://wa.me/11984843250?text=Ol%C3%A1%2C%20Dr.%20Paulo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Dent%C3%A1rio%20Dr.%20Paulo%20Rog%C3%A9rio%20Barbosa%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11984843250?text=Ol%C3%A1%2C%20Dr.%20Paulo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Pinheiros%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Dent%C3%A1rio%20Dr.%20Paulo%20Rog%C3%A9rio%20Barbosa%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K6" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. Paulo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Dentário Dr. Paulo Rogério Barbosa, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dr. Paulo! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Pinheiros para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Consultório Dentário Dr. Paulo Rogério Barbosa, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="7" xml:space="preserve">
@@ -653,13 +658,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J7" t="str">
-        <v>https://wa.me/11925683124?text=Ol%C3%A1%2C%20Oral%20Premium!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Oral%20Premium%20Implantes%20Pinheiros%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11925683124?text=Ol%C3%A1%2C%20Oral%20Premium!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Pinheiros%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Oral%20Premium%20Implantes%20Pinheiros%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K7" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Oral Premium! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Oral Premium Implantes Pinheiros, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Oral Premium! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Pinheiros para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Oral Premium Implantes Pinheiros, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="8" xml:space="preserve">
@@ -691,13 +697,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J8" t="str">
-        <v>https://wa.me/11944502942?text=Ol%C3%A1%2C%20Cairo%20Martinelli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cairo%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11944502942?text=Ol%C3%A1%2C%20Cairo%20Martinelli!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Pinheiros%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cairo%20Martinelli%20Odontologia%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K8" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Cairo Martinelli! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Cairo Martinelli Odontologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Cairo Martinelli! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Pinheiros para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Cairo Martinelli Odontologia, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="9" xml:space="preserve">
@@ -729,13 +736,14 @@
         <v>http://instagram.com/dr.viniciusbibiano</v>
       </c>
       <c r="J9" t="str">
-        <v>https://wa.me/11993616602?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20Bibiano%20%7C%20Dentista%20em%20Pinheiros%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993616602?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Pinheiros%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20Bibiano%20%7C%20Dentista%20em%20Pinheiros%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K9" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Pinheiros e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica Bibiano | Dentista em Pinheiros, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Pinheiros para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clínica Odontológica Bibiano | Dentista em Pinheiros, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="10" xml:space="preserve">
@@ -767,13 +775,14 @@
         <v>https://wa.me/message/H22QFMB4FZMYD1</v>
       </c>
       <c r="J10" t="str">
-        <v>https://wa.me/11950060220?text=Ol%C3%A1%2C%20Dra.%20J%C3%A9ssica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20J%C3%A9ssica%20Mattos%20de%20Britto%20-%20Odontologia%20Est%C3%A9tica%20e%20Restauradora%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11950060220?text=Ol%C3%A1%2C%20Dra.%20J%C3%A9ssica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Jardins%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20J%C3%A9ssica%20Mattos%20de%20Britto%20-%20Odontologia%20Est%C3%A9tica%20e%20Restauradora%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K10" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Jéssica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Jéssica Mattos de Britto - Odontologia Estética e Restauradora, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Jéssica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Jardins para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Jéssica Mattos de Britto - Odontologia Estética e Restauradora, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="11" xml:space="preserve">
@@ -805,13 +814,14 @@
         <v>http://instagram.com/dramariagoncalves</v>
       </c>
       <c r="J11" t="str">
-        <v>https://wa.me/11910995184?text=Ol%C3%A1%2C%20Dra%20Maria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Maria%20Eduarda%20Gon%C3%A7alves%20%7C%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11910995184?text=Ol%C3%A1%2C%20Dra%20Maria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Jardins%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Maria%20Eduarda%20Gon%C3%A7alves%20%7C%20Cirurgi%C3%A3%20Dentista%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K11" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Maria! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Maria Eduarda Gonçalves | Cirurgiã Dentista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Maria! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Jardins para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Maria Eduarda Gonçalves | Cirurgiã Dentista, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -843,13 +853,14 @@
         <v>https://www.instagram.com/drgalsander?igsh=MXRwZ3JlZXQ3cXN3Yg==</v>
       </c>
       <c r="J12" t="str">
-        <v>https://wa.me/11976253586?text=Ol%C3%A1%2C%20Dr.%20Galsander!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Galsander%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976253586?text=Ol%C3%A1%2C%20Dr.%20Galsander!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Itaim%20Bibi%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dr.%20Galsander%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K12" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. Galsander! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Galsander, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dr. Galsander! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Itaim Bibi para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dr. Galsander, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="13" xml:space="preserve">
@@ -881,13 +892,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J13" t="str">
-        <v>https://wa.me/11964008778?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20AR%20Odontologia%20-%20Dr.%20C%C3%A9sar%20e%20Equipe%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964008778?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Vila%20Mariana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20AR%20Odontologia%20-%20Dr.%20C%C3%A9sar%20e%20Equipe%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K13" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica AR Odontologia - Dr. César e Equipe, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clínica Odontologia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Vila Mariana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clínica AR Odontologia - Dr. César e Equipe, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="14" xml:space="preserve">
@@ -919,13 +931,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J14" t="str">
-        <v>https://wa.me/11947647807?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20LK%20%7C%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11947647807?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Odontol%C3%B3gica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Vila%20Mariana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Odontol%C3%B3gica%20LK%20%7C%20Vila%20Mariana%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K14" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Odontológica LK | Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clínica Odontológica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Vila Mariana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clínica Odontológica LK | Vila Mariana, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="15" xml:space="preserve">
@@ -957,13 +970,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J15" t="str">
-        <v>https://wa.me/11999919290?text=Ol%C3%A1%2C%20Dra.%20Carolina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Carolina%20Oliveira%20-%20Endodontia%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11999919290?text=Ol%C3%A1%2C%20Dra.%20Carolina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Vila%20Mariana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Carolina%20Oliveira%20-%20Endodontia%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20na%20Vila%20Mariana%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K15" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Carolina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Carolina Oliveira - Endodontia e Harmonização Facial na Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Carolina! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Vila Mariana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Carolina Oliveira - Endodontia e Harmonização Facial na Vila Mariana, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="16" xml:space="preserve">
@@ -995,13 +1009,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J16" t="str">
-        <v>https://wa.me/11958187028?text=Ol%C3%A1%2C%20Odontologico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontologico%20na%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11958187028?text=Ol%C3%A1%2C%20Odontologico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Vila%20Mariana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontologico%20na%20Vila%20Mariana%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K16" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontologico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontologico na Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Odontologico! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Vila Mariana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Consultório Odontologico na Vila Mariana, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="17" xml:space="preserve">
@@ -1033,13 +1048,14 @@
         <v>https://www.google.com/url?sa=t&amp;source=web&amp;rct=j&amp;url=https://dentista-dra-andreia-serra.negocio.site/&amp;ved=2ahUKEwjc5ueF7v_nAhWjLLkGHd-pDB0QFjAZegQIBxAB&amp;usg=AOvVaw23N10dPXvHyJEkdydgJi0X</v>
       </c>
       <c r="J17" t="str">
-        <v>https://wa.me/11975911100?text=Ol%C3%A1%2C%20Dra.%20Andreia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Andreia%20Serra%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975911100?text=Ol%C3%A1%2C%20Dra.%20Andreia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Vila%20Mariana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Andreia%20Serra%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K17" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Andreia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Vila Mariana e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Andreia Serra, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Andreia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Vila Mariana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Andreia Serra, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="18" xml:space="preserve">
@@ -1071,13 +1087,14 @@
         <v>https://l.instagram.com/?u=https://linktr.ee/dramarciaharumimurata&amp;e=AT1N9YDKEugyBbEwe94G4hO-NzSWSyHgF1RhzSumj7pTZk2roJYnt2LifhIyfVpvgBMPU_BNIypnIsxCYq9APoSsmxxIDJQmdYcOiodw1AyXxK6TeRLfyw</v>
       </c>
       <c r="J18" t="str">
-        <v>https://wa.me/11976088594?text=Ol%C3%A1%2C%20Dentista!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20-%20Tatuap%C3%A9%20-%20Dra.%20Marcia%20Harumi%20Murata%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976088594?text=Ol%C3%A1%2C%20Dentista!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dentista%20-%20Tatuap%C3%A9%20-%20Dra.%20Marcia%20Harumi%20Murata%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K18" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista - Tatuapé - Dra. Marcia Harumi Murata, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dentista! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dentista - Tatuapé - Dra. Marcia Harumi Murata, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="19" xml:space="preserve">
@@ -1109,13 +1126,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J19" t="str">
-        <v>https://wa.me/11930252702?text=Ol%C3%A1%2C%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra%20Regiane%20Carvalheiro%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11930252702?text=Ol%C3%A1%2C%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra%20Regiane%20Carvalheiro%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K19" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontológico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra Regiane Carvalheiro, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Odontológico! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Consultório Odontológico Dra Regiane Carvalheiro, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="20" xml:space="preserve">
@@ -1147,13 +1165,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J20" t="str">
-        <v>https://wa.me/11951406244?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Faustino%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951406244?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Faustino%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K20" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Faustino, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Gabriela Faustino, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="21" xml:space="preserve">
@@ -1185,13 +1204,14 @@
         <v>https://instagram.com/dra_annacarolina</v>
       </c>
       <c r="J21" t="str">
-        <v>https://wa.me/11985969605?text=Ol%C3%A1%2C%20Dra%20Anna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Anna%20Carolina%20%7C%20Dentista%20%7C%20Harmoniza%C3%A7%C3%A3o%20%7C%20Aparelho%20invis%C3%ADvel%20-%20sousmile%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11985969605?text=Ol%C3%A1%2C%20Dra%20Anna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Anna%20Carolina%20%7C%20Dentista%20%7C%20Harmoniza%C3%A7%C3%A3o%20%7C%20Aparelho%20invis%C3%ADvel%20-%20sousmile%20%7C%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K21" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Anna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Anna Carolina | Dentista | Harmonização | Aparelho invisível - sousmile | Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Anna! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Anna Carolina | Dentista | Harmonização | Aparelho invisível - sousmile | Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="22" xml:space="preserve">
@@ -1223,13 +1243,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J22" t="str">
-        <v>https://wa.me/11985133002?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20S%C3%A3o%20Paulo%20Dra%20Bianca%20Assis%20Cirurgi%C3%A3%20Dentista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11985133002?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dentista%20S%C3%A3o%20Paulo%20Dra%20Bianca%20Assis%20Cirurgi%C3%A3%20Dentista%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K22" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista São Paulo Dra Bianca Assis Cirurgiã Dentista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dentista São Paulo Dra Bianca Assis Cirurgiã Dentista, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="23" xml:space="preserve">
@@ -1261,13 +1282,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J23" t="str">
-        <v>https://wa.me/11976103809?text=Ol%C3%A1%2C%20Dra.%20Daniella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Daniella%20Plaza%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976103809?text=Ol%C3%A1%2C%20Dra.%20Daniella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Daniella%20Plaza%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K23" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Daniella! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Daniella Plaza, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Daniella! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Daniella Plaza, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="24" xml:space="preserve">
@@ -1299,13 +1321,14 @@
         <v>https://instagram.com/dratamymenezes?igshid=MzMyNGUyNmU2YQ==</v>
       </c>
       <c r="J24" t="str">
-        <v>https://wa.me/11945231034?text=Ol%C3%A1%2C%20Clinica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Odontologia%20Especializada%20-%20Dra%20Thamiris%20Menezes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945231034?text=Ol%C3%A1%2C%20Clinica%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%204%2C8%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Tatuap%C3%A9%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Odontologia%20Especializada%20-%20Dra%20Thamiris%20Menezes%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K24" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clinica Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Tatuapé e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Odontologia Especializada - Dra Thamiris Menezes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clinica Odontologia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 4,8★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Tatuapé para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clinica de Odontologia Especializada - Dra Thamiris Menezes, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="25" xml:space="preserve">
@@ -1337,13 +1360,14 @@
         <v>https://www.instagram.com/dradanielleoliveiraa?igsh=MW5oc3U0YWQ4Mmcyag==&amp;utm_source=qr</v>
       </c>
       <c r="J25" t="str">
-        <v>https://wa.me/11991519479?text=Ol%C3%A1%2C%20Dra.%20Danielle!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Danielle%20Oliveira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991519479?text=Ol%C3%A1%2C%20Dra.%20Danielle!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Perdizes%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Danielle%20Oliveira%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K25" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Danielle! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Danielle Oliveira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Danielle! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Perdizes para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Danielle Oliveira, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="26" xml:space="preserve">
@@ -1375,13 +1399,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J26" t="str">
-        <v>https://wa.me/11992918335?text=Ol%C3%A1%2C%20Dra.%20Isadora!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Isadora%20Martinelli%20Odontologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11992918335?text=Ol%C3%A1%2C%20Dra.%20Isadora!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Perdizes%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Isadora%20Martinelli%20Odontologia%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K26" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Isadora! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Isadora Martinelli Odontologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Isadora! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Perdizes para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Isadora Martinelli Odontologia, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="27" xml:space="preserve">
@@ -1413,13 +1438,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J27" t="str">
-        <v>https://wa.me/11963239000?text=Ol%C3%A1%2C%20Dra%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Helena%20Pires%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11963239000?text=Ol%C3%A1%2C%20Dra%20Helena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Perdizes%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Helena%20Pires%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K27" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Helena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Helena Pires, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Helena! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Perdizes para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Helena Pires, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="28" xml:space="preserve">
@@ -1451,13 +1477,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J28" t="str">
-        <v>https://wa.me/11939011103?text=Ol%C3%A1%2C%20Dra%20Giovanna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Giovanna%20Dourado%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11939011103?text=Ol%C3%A1%2C%20Dra%20Giovanna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%204%2C8%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Perdizes%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Giovanna%20Dourado%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K28" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Giovanna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Giovanna Dourado, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Giovanna! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 4,8★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Perdizes para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Giovanna Dourado, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="29" xml:space="preserve">
@@ -1489,13 +1516,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J29" t="str">
-        <v>https://wa.me/11988877098?text=Ol%C3%A1%2C%20Dra.Leticia%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Leticia%20Morais%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11988877098?text=Ol%C3%A1%2C%20Dra.Leticia%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%204%2C8%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Perdizes%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.Leticia%20Morais%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K29" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra.Leticia Morais! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Leticia Morais, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra.Leticia Morais! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 4,8★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Perdizes para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra.Leticia Morais, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="30" xml:space="preserve">
@@ -1527,13 +1555,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J30" t="str">
-        <v>https://wa.me/11996040673?text=Ol%C3%A1%2C%20Dra.%20Monique!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Monique%20Fai%C3%A3o%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11996040673?text=Ol%C3%A1%2C%20Dra.%20Monique!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Perdizes%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Monique%20Fai%C3%A3o%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K30" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Monique! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Monique Faião, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Monique! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Perdizes para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Monique Faião, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="31" xml:space="preserve">
@@ -1565,13 +1594,14 @@
         <v>https://www.instagram.com/dra.luanavieiraa?igsh=cGRzNHNpOTJ4MXkw&amp;utm_source=qr</v>
       </c>
       <c r="J31" t="str">
-        <v>https://wa.me/11978738749?text=Ol%C3%A1%2C%20Dentista%20Santana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20Santana%20-%20Dra%20Luana%20Vieira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11978738749?text=Ol%C3%A1%2C%20Dentista%20Santana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Santana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Santana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dentista%20em%20Santana%20-%20Dra%20Luana%20Vieira%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K31" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista Santana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em Santana - Dra Luana Vieira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dentista Santana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Santana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Santana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dentista em Santana - Dra Luana Vieira, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="32" xml:space="preserve">
@@ -1603,13 +1633,14 @@
         <v>https://instagram.com/dralourdesspereira?igshid=MzRlODBiNWFlZA==</v>
       </c>
       <c r="J32" t="str">
-        <v>https://wa.me/11956566650?text=Ol%C3%A1%2C%20Odontologia%20%2FSa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Odontologia%20%2FSa%C3%BAde%20e%20bem%20estar%20Dra%20Lourdes%20S.Pereira%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11956566650?text=Ol%C3%A1%2C%20Odontologia%20%2FSa%C3%BAde!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Santana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Santana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Odontologia%20%2FSa%C3%BAde%20e%20bem%20estar%20Dra%20Lourdes%20S.Pereira%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K32" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Odontologia /Saúde! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Odontologia /Saúde e bem estar Dra Lourdes S.Pereira, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Odontologia /Saúde! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Santana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Santana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Odontologia /Saúde e bem estar Dra Lourdes S.Pereira, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="33" xml:space="preserve">
@@ -1641,13 +1672,14 @@
         <v>https://www.instagram.com/draluciana.dentista</v>
       </c>
       <c r="J33" t="str">
-        <v>https://wa.me/11993273559?text=Ol%C3%A1%2C%20Dra%20Luciana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luciana%20Espejo%20%7C%20Dentista%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993273559?text=Ol%C3%A1%2C%20Dra%20Luciana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Santana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Santana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Luciana%20Espejo%20%7C%20Dentista%20em%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K33" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Luciana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luciana Espejo | Dentista em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Luciana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Santana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Santana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Luciana Espejo | Dentista em São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="34" xml:space="preserve">
@@ -1679,13 +1711,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J34" t="str">
-        <v>https://wa.me/11991252211?text=Ol%C3%A1%2C%20Dra%20Alessandra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Alessandra%20Parisi%20%7C%20Dentista%20%7C%20Santana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991252211?text=Ol%C3%A1%2C%20Dra%20Alessandra!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Santana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Santana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Alessandra%20Parisi%20%7C%20Dentista%20%7C%20Santana%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K34" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Alessandra! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Alessandra Parisi | Dentista | Santana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Alessandra! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Santana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Santana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Alessandra Parisi | Dentista | Santana, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="35" xml:space="preserve">
@@ -1717,13 +1750,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J35" t="str">
-        <v>https://wa.me/11915333818?text=Ol%C3%A1%2C%20Dra.%20Thabata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Santana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra.%20Thabata%20L%C3%ADvia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11915333818?text=Ol%C3%A1%2C%20Dra.%20Thabata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Santana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Santana%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Consult%C3%B3rio%20Odontol%C3%B3gico%20Dra.%20Thabata%20L%C3%ADvia%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K35" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Thabata! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Santana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Consultório Odontológico Dra. Thabata Lívia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Thabata! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Santana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Santana para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Consultório Odontológico Dra. Thabata Lívia, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="36" xml:space="preserve">
@@ -1755,13 +1789,14 @@
         <v>https://www.instagram.com/centroodontomorumbi/</v>
       </c>
       <c r="J36" t="str">
-        <v>https://wa.me/11966400022?text=Ol%C3%A1%2C%20Centro%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20Odontol%C3%B3gico%20Morumbi%20-%20Dra%20Renata%20Ramos%20e%20Equipe%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11966400022?text=Ol%C3%A1%2C%20Centro%20Odontol%C3%B3gico!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Morumbi%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Morumbi%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Centro%20Odontol%C3%B3gico%20Morumbi%20-%20Dra%20Renata%20Ramos%20e%20Equipe%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K36" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Centro Odontológico! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro Odontológico Morumbi - Dra Renata Ramos e Equipe, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Centro Odontológico! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Morumbi (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Morumbi para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Centro Odontológico Morumbi - Dra Renata Ramos e Equipe, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="37" xml:space="preserve">
@@ -1793,13 +1828,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J37" t="str">
-        <v>https://wa.me/11951307605?text=Ol%C3%A1%2C%20Dentista%20Morumbi%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Morumbi%2C%20S%C3%A3o%20Paulo%20-%20Dra%20Larissa%20Tavares%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951307605?text=Ol%C3%A1%2C%20Dentista%20Morumbi%2C!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Morumbi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Morumbi%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dentista%20Morumbi%2C%20S%C3%A3o%20Paulo%20-%20Dra%20Larissa%20Tavares%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K37" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista Morumbi,! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Morumbi, São Paulo - Dra Larissa Tavares, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dentista Morumbi,! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Morumbi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Morumbi para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dentista Morumbi, São Paulo - Dra Larissa Tavares, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="38" xml:space="preserve">
@@ -1831,13 +1867,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J38" t="str">
-        <v>https://wa.me/11959391155?text=Ol%C3%A1%2C%20Dr.%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20Dr.%20Jo%C3%A3o%20Vila%20-%20Morumbi%20-%20Vila%20Progredior%20-%20Jd%20Guedala%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11959391155?text=Ol%C3%A1%2C%20Dr.%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Morumbi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Morumbi%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dentista%20Dr.%20Jo%C3%A3o%20Vila%20-%20Morumbi%20-%20Vila%20Progredior%20-%20Jd%20Guedala%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K38" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. João! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista Dr. João Vila - Morumbi - Vila Progredior - Jd Guedala, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dr. João! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Morumbi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Morumbi para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dentista Dr. João Vila - Morumbi - Vila Progredior - Jd Guedala, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="39" xml:space="preserve">
@@ -1869,13 +1906,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J39" t="str">
-        <v>https://wa.me/11958978174?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dentista%20em%20S%C3%A3o%20Paulo%20-%20Dra%20Bruna%20Del%20Mestre%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11958978174?text=Ol%C3%A1%2C%20Dentista%20S%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Morumbi%20(nota%204%2C7%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Morumbi%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dentista%20em%20S%C3%A3o%20Paulo%20-%20Dra%20Bruna%20Del%20Mestre%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K39" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 4,7★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dentista em São Paulo - Dra Bruna Del Mestre, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dentista São! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Morumbi (nota 4,7★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Morumbi para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dentista em São Paulo - Dra Bruna Del Mestre, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="40" xml:space="preserve">
@@ -1907,13 +1945,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J40" t="str">
-        <v>https://wa.me/11949420235?text=Ol%C3%A1%2C%20Dra.%20Tayna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Morumbi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Tayna%20Bastos%20%7C%20Dentista%20no%20Morumbi%20-%20S%C3%A3o%20Paulo%20%7C%20Pr%C3%B3tese%2C%20est%C3%A9tica%20e%20urg%C3%AAncia.%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11949420235?text=Ol%C3%A1%2C%20Dra.%20Tayna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Morumbi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Morumbi%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Tayna%20Bastos%20%7C%20Dentista%20no%20Morumbi%20-%20S%C3%A3o%20Paulo%20%7C%20Pr%C3%B3tese%2C%20est%C3%A9tica%20e%20urg%C3%AAncia.%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K40" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Tayna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Morumbi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Tayna Bastos | Dentista no Morumbi - São Paulo | Prótese, estética e urgência., pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Tayna! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Morumbi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Morumbi para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Tayna Bastos | Dentista no Morumbi - São Paulo | Prótese, estética e urgência., focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="41" xml:space="preserve">
@@ -1945,13 +1984,14 @@
         <v>https://www.instagram.com/dra_mayaracardoso/</v>
       </c>
       <c r="J41" t="str">
-        <v>https://wa.me/11947930542?text=Ol%C3%A1%2C%20Dra%20Mayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Mayara%20Cardoso%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11947930542?text=Ol%C3%A1%2C%20Dra%20Mayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Mayara%20Cardoso%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K41" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Mayara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Mayara Cardoso, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Mayara! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Mayara Cardoso, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="42" xml:space="preserve">
@@ -1983,13 +2023,14 @@
         <v>https://www.doctoralia.com.br/nayara-freitas/dentista/sao-paulo</v>
       </c>
       <c r="J42" t="str">
-        <v>https://wa.me/11972871378?text=Ol%C3%A1%2C%20Dra%20Nayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Nayara%20Freitas%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972871378?text=Ol%C3%A1%2C%20Dra%20Nayara!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Nayara%20Freitas%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K42" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Nayara! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Nayara Freitas, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Nayara! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Nayara Freitas, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="43" xml:space="preserve">
@@ -2021,13 +2062,14 @@
         <v>https://www.instagram.com/dr.alexandrewon/</v>
       </c>
       <c r="J43" t="str">
-        <v>https://wa.me/11940696509?text=Ol%C3%A1%2C%20Won%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Won%20Odontologia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11940696509?text=Ol%C3%A1%2C%20Won%20Odontologia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Won%20Odontologia%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K43" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Won Odontologia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Won Odontologia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Won Odontologia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Won Odontologia, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="44" xml:space="preserve">
@@ -2059,13 +2101,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J44" t="str">
-        <v>https://wa.me/11945216642?text=Ol%C3%A1%2C%20Dr.%20Marcello!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr.%20Marcello%20Barone%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%20e%20Odontologia%20est%C3%A9tica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945216642?text=Ol%C3%A1%2C%20Dr.%20Marcello!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dr.%20Marcello%20Barone%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%20e%20Odontologia%20est%C3%A9tica%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K44" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dr. Marcello! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr. Marcello Barone - Harmonização Orofacial e Odontologia estética, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dr. Marcello! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dr. Marcello Barone - Harmonização Orofacial e Odontologia estética, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="45" xml:space="preserve">
@@ -2097,13 +2140,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J45" t="str">
-        <v>https://wa.me/11998978621?text=Ol%C3%A1%2C%20Dra.%20Cecilia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cecilia%20Sena%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11998978621?text=Ol%C3%A1%2C%20Dra.%20Cecilia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Cecilia%20Sena%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K45" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Cecilia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cecilia Sena, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Cecilia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Cecilia Sena, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="46" xml:space="preserve">
@@ -2135,13 +2179,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J46" t="str">
-        <v>https://wa.me/11984157966?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Rodrigues%20Santos%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11984157966?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Rodrigues%20Santos%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K46" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Rodrigues Santos, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Luana Rodrigues Santos, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="47" xml:space="preserve">
@@ -2173,13 +2218,14 @@
         <v>https://instagram.com/drasilviaarruda?utm_medium=copy_link</v>
       </c>
       <c r="J47" t="str">
-        <v>https://wa.me/11998439008?text=Ol%C3%A1%2C%20Dra%20Silvia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Odontologia%20em%20Higien%C3%B3polis%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C3%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Silvia%20Gajardoni%20Arruda%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11998439008?text=Ol%C3%A1%2C%20Dra%20Silvia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Higien%C3%B3polis%20(nota%204%2C3%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20est%C3%A1%20com%20dor%20de%20dente%20ou%20precisa%20de%20um%20tratamento%20urgente%20n%C3%A3o%20vai%20procurar%20no%20Instagram%3A%20a%20pessoa%20pesquisa%20direto%20no%20Google%20buscando%20um%20dentista%20aqui%20em%20Higien%C3%B3polis%20para%20resolver%20na%20hora.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20pacientes%20prontos%20para%20agendar%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20cl%C3%ADnicas%20concorrentes%20da%20regi%C3%A3o.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Silvia%20Gajardoni%20Arruda%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K47" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Silvia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Odontologia em Higienópolis e encontrei o seu perfil no Google com nota 4,3★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Silvia Gajardoni Arruda, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Silvia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Higienópolis (nota 4,3★ no Google, parabéns!).
+Te mandei mensagem porque quem está com dor de dente ou precisa de um tratamento urgente não vai procurar no Instagram: a pessoa pesquisa direto no Google buscando um dentista aqui em Higienópolis para resolver na hora. Como você está sem um site próprio cadastrado, você acaba perdendo esses pacientes prontos para agendar e perdendo dinheiro todos os dias para clínicas concorrentes da região.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Silvia Gajardoni Arruda, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="48" xml:space="preserve">
@@ -2211,13 +2257,14 @@
         <v>https://www.instagram.com/draraphaela.maia/</v>
       </c>
       <c r="J48" t="str">
-        <v>https://wa.me/11993878167?text=Ol%C3%A1%2C%20Dra%20Raphaela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raphaela%20Maia%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20em%20Moema%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993878167?text=Ol%C3%A1%2C%20Dra%20Raphaela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Moema.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Raphaela%20Maia%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20em%20Moema%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K48" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Raphaela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raphaela Maia - Harmonização Facial em Moema, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Raphaela! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Moema. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Raphaela Maia - Harmonização Facial em Moema, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="49" xml:space="preserve">
@@ -2249,13 +2296,14 @@
         <v>https://linktr.ee/drafeliramonteiro</v>
       </c>
       <c r="J49" t="str">
-        <v>https://wa.me/11988571847?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Lira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Zona%20Sul%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11988571847?text=Ol%C3%A1%2C%20Dra.%20Fernanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Moema.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Fernanda%20Lira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Zona%20Sul%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K49" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Fernanda Lira | Harmonização Facial | Zona Sul São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Fernanda! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Moema. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Fernanda Lira | Harmonização Facial | Zona Sul São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="50" xml:space="preserve">
@@ -2287,13 +2335,14 @@
         <v>https://www.instagram.com/dramendoncagabriela?igsh=MTE5MThiMGVhcXV2MQ==</v>
       </c>
       <c r="J50" t="str">
-        <v>https://wa.me/11965850611?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Mendon%C3%A7a%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11965850611?text=Ol%C3%A1%2C%20Dra%20Gabriela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Gabriela%20Mendon%C3%A7a%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K50" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Gabriela Mendonça - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Gabriela! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Gabriela Mendonça - Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="51" xml:space="preserve">
@@ -2325,13 +2374,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J51" t="str">
-        <v>https://wa.me/11975815099?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Avan%C3%A7ada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20AC%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975815099?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Avan%C3%A7ada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20AC%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K51" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Estética Avançada! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para AC Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Estética Avançada! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para AC Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="52" xml:space="preserve">
@@ -2363,13 +2413,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J52" t="str">
-        <v>https://wa.me/11958882681?text=Ol%C3%A1%2C%20Dra%20Fl%C3%A1via!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Fl%C3%A1via%20Roma%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11958882681?text=Ol%C3%A1%2C%20Dra%20Fl%C3%A1via!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Fl%C3%A1via%20Roma%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K52" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Flávia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Flávia Roma Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Flávia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Flávia Roma Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="53" xml:space="preserve">
@@ -2401,13 +2452,14 @@
         <v>https://www.instagram.com/estetica_monicamuchante?igsh=M2syNWtzY2t3b3k4</v>
       </c>
       <c r="J53" t="str">
-        <v>https://wa.me/11951008872?text=Ol%C3%A1%2C%20Dra.%20M%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20M%C3%B4nica%20Muchante%20Biom%C3%A9dica%20Esteta%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11951008872?text=Ol%C3%A1%2C%20Dra.%20M%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20M%C3%B4nica%20Muchante%20Biom%C3%A9dica%20Esteta%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K53" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Mônica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Mônica Muchante Biomédica Esteta | Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Mônica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Mônica Muchante Biomédica Esteta | Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="54" xml:space="preserve">
@@ -2439,13 +2491,14 @@
         <v>https://www.instagram.com/dragiulianafranca/</v>
       </c>
       <c r="J54" t="str">
-        <v>https://wa.me/11977440161?text=Ol%C3%A1%2C%20Dra.%20Giuliana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Giuliana%20Fran%C3%A7a%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11977440161?text=Ol%C3%A1%2C%20Dra.%20Giuliana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Giuliana%20Fran%C3%A7a%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K54" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Giuliana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Giuliana França Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Giuliana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Giuliana França Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="55" xml:space="preserve">
@@ -2477,13 +2530,14 @@
         <v>https://api.whatsapp.com/message/CDJPK6KBGJXNE1?autoload=1&amp;app_absent=0</v>
       </c>
       <c r="J55" t="str">
-        <v>https://wa.me/11966291967?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Mello%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11966291967?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Mello%20%7C%20Est%C3%A9tica%20Avan%C3%A7ada%20SP%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K55" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Mello | Estética Avançada SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Letícia Mello | Estética Avançada SP, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="56" xml:space="preserve">
@@ -2515,13 +2569,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J56" t="str">
-        <v>https://wa.me/11952805419?text=Ol%C3%A1%2C%20Dra%20Leticia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Leticia%20Papp%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11952805419?text=Ol%C3%A1%2C%20Dra%20Leticia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Leticia%20Papp%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K56" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Leticia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Leticia Papp - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Leticia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Leticia Papp - Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="57" xml:space="preserve">
@@ -2553,13 +2608,14 @@
         <v>https://www.instagram.com/dra_amandaomartins/</v>
       </c>
       <c r="J57" t="str">
-        <v>https://wa.me/11975791298?text=Ol%C3%A1%2C%20Lemu%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Lemu%20Clinic%20%7C%20Dra.%20Amanda%20Martins%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975791298?text=Ol%C3%A1%2C%20Lemu%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Lemu%20Clinic%20%7C%20Dra.%20Amanda%20Martins%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K57" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Lemu Clinic! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Lemu Clinic | Dra. Amanda Martins | Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Lemu Clinic! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Lemu Clinic | Dra. Amanda Martins | Harmonização Facial, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="58" xml:space="preserve">
@@ -2591,13 +2647,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J58" t="str">
-        <v>https://wa.me/11976971573?text=Ol%C3%A1%2C%20Dra%20Stephanie!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Stephanie%20Milagre%20-%20Cl%C3%ADnica%20de%20est%C3%A9tica%20avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976971573?text=Ol%C3%A1%2C%20Dra%20Stephanie!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Jardins.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Stephanie%20Milagre%20-%20Cl%C3%ADnica%20de%20est%C3%A9tica%20avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K58" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Stephanie! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Stephanie Milagre - Clínica de estética avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Stephanie! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Jardins. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Stephanie Milagre - Clínica de estética avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="59" xml:space="preserve">
@@ -2629,13 +2686,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J59" t="str">
-        <v>https://wa.me/11954537661?text=Ol%C3%A1%2C%20Dra%20Renata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Renata%20Queiroz%20-%20Biomedicina%20Est%C3%A9tica%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11954537661?text=Ol%C3%A1%2C%20Dra%20Renata!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Pinheiros.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Renata%20Queiroz%20-%20Biomedicina%20Est%C3%A9tica%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K59" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Renata! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Renata Queiroz - Biomedicina Estética, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Renata! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Pinheiros. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Renata Queiroz - Biomedicina Estética, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="60" xml:space="preserve">
@@ -2667,13 +2725,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J60" t="str">
-        <v>https://wa.me/11962612208?text=Ol%C3%A1%2C%20Nathalia%20Nastri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dr%20Nathalia%20Nastri%20-%20Biomedicina%20Est%C3%A9tica-%20Pinheiros%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11962612208?text=Ol%C3%A1%2C%20Nathalia%20Nastri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Pinheiros.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dr%20Nathalia%20Nastri%20-%20Biomedicina%20Est%C3%A9tica-%20Pinheiros%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K60" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Nathalia Nastri! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dr Nathalia Nastri - Biomedicina Estética- Pinheiros São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Nathalia Nastri! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Pinheiros. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dr Nathalia Nastri - Biomedicina Estética- Pinheiros São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="61" xml:space="preserve">
@@ -2705,13 +2764,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J61" t="str">
-        <v>https://wa.me/11914566745?text=Ol%C3%A1%2C%20Dra.Igma%20Araujo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.Igma%20Araujo%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11914566745?text=Ol%C3%A1%2C%20Dra.Igma%20Araujo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Itaim%20Bibi.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.Igma%20Araujo%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K61" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra.Igma Araujo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra.Igma Araujo | Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra.Igma Araujo! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Itaim Bibi. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra.Igma Araujo | Harmonização Facial, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="62" xml:space="preserve">
@@ -2743,13 +2803,14 @@
         <v>https://wa.me/5511988399169</v>
       </c>
       <c r="J62" t="str">
-        <v>https://wa.me/11991646740?text=Ol%C3%A1%2C%20Dra%20Carmen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carmen%20Barge%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Corporal%20%7C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991646740?text=Ol%C3%A1%2C%20Dra%20Carmen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Itaim%20Bibi.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Carmen%20Barge%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Corporal%20%7C%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K62" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Carmen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carmen Barge | Harmonização Facial e Corporal | São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Carmen! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Itaim Bibi. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Carmen Barge | Harmonização Facial e Corporal | São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="63" xml:space="preserve">
@@ -2781,13 +2842,14 @@
         <v>https://www.instagram.com/dralaismarquesa/</v>
       </c>
       <c r="J63" t="str">
-        <v>https://wa.me/11954742132?text=Ol%C3%A1%2C%20Dra.%20La%C3%ADs!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20La%C3%ADs%20Marques%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11954742132?text=Ol%C3%A1%2C%20Dra.%20La%C3%ADs!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Itaim%20Bibi.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20La%C3%ADs%20Marques%20-%20Harmoniza%C3%A7%C3%A3o%20Orofacial%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K63" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Laís! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Laís Marques - Harmonização Orofacial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Laís! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Itaim Bibi. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Laís Marques - Harmonização Orofacial, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="64" xml:space="preserve">
@@ -2819,13 +2881,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J64" t="str">
-        <v>https://wa.me/11944625222?text=Ol%C3%A1%2C%20Clinica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Est%C3%A9tica-%20Elaine%20Vasconcelos-%20Harmoniza%C3%A7%C3%A3o%20Facial-%20Itaim%20Bibi%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11944625222?text=Ol%C3%A1%2C%20Clinica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Itaim%20Bibi.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Clinica%20de%20Est%C3%A9tica-%20Elaine%20Vasconcelos-%20Harmoniza%C3%A7%C3%A3o%20Facial-%20Itaim%20Bibi%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K64" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clinica Estética! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clinica de Estética- Elaine Vasconcelos- Harmonização Facial- Itaim Bibi, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clinica Estética! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Itaim Bibi. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clinica de Estética- Elaine Vasconcelos- Harmonização Facial- Itaim Bibi, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="65" xml:space="preserve">
@@ -2857,13 +2920,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J65" t="str">
-        <v>https://wa.me/11961662005?text=Ol%C3%A1%2C%20Dra.%20Alyne!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Alyne%20Souza%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20-%20Vila%20Ol%C3%ADmpia%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11961662005?text=Ol%C3%A1%2C%20Dra.%20Alyne!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Itaim%20Bibi.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Alyne%20Souza%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20-%20Vila%20Ol%C3%ADmpia%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K65" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Alyne! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Alyne Souza | Harmonização Facial - Vila Olímpia, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Alyne! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Itaim Bibi. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Alyne Souza | Harmonização Facial - Vila Olímpia, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="66" xml:space="preserve">
@@ -2895,13 +2959,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J66" t="str">
-        <v>https://wa.me/11917440783?text=Ol%C3%A1%2C%20Dra.%20Thayn%C3%A1!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Thayn%C3%A1%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11917440783?text=Ol%C3%A1%2C%20Dra.%20Thayn%C3%A1!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Itaim%20Bibi.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Thayn%C3%A1%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K66" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Thayná! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Thayná Rosa | Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Thayná! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Itaim Bibi. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Thayná Rosa | Harmonização Facial, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="67" xml:space="preserve">
@@ -2933,13 +2998,14 @@
         <v>https://www.instagram.com/clinicabellalinea?igsh=MXVmMngxNm05aXdlZQ%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J67" t="str">
-        <v>https://wa.me/11991236080?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Bella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C7%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Bella%20Linea%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11991236080?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Bella!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%204%2C7%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Vila%20Mariana.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Bella%20Linea%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K67" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Bella! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 4,7★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Bella Linea, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clínica Bella! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 4,7★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Vila Mariana. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clínica Bella Linea, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="68" xml:space="preserve">
@@ -2971,13 +3037,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J68" t="str">
-        <v>https://wa.me/11992442685?text=Ol%C3%A1%2C%20Dra%20Raquel!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Raquel%20Camargo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11992442685?text=Ol%C3%A1%2C%20Dra%20Raquel!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Vila%20Mariana.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Raquel%20Camargo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K68" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Raquel! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Raquel Camargo - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Raquel! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Vila Mariana. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Raquel Camargo - Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="69" xml:space="preserve">
@@ -3009,13 +3076,14 @@
         <v>https://wa.me/5511965833614</v>
       </c>
       <c r="J69" t="str">
-        <v>https://wa.me/11965833614?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Botox%20na%20Vila%20Mariana%20Dra.%20Bruna%20Ferreira%20Esteta%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11965833614?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Vila%20Mariana.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Botox%20na%20Vila%20Mariana%20Dra.%20Bruna%20Ferreira%20Esteta%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K69" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Botox na Vila Mariana Dra. Bruna Ferreira Esteta, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Vila Mariana. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Botox na Vila Mariana Dra. Bruna Ferreira Esteta, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="70" xml:space="preserve">
@@ -3047,13 +3115,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J70" t="str">
-        <v>https://wa.me/11994003820?text=Ol%C3%A1%2C%20Nadia%20Ces%C3%A1rio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nadia%20Ces%C3%A1rio%20-%20Est%C3%A9tica%20Especializada%20%7CDrenagem%20Linf%C3%A1tica%20Vila%20Mariana%20%7CLimpeza%20de%20pele%20%7CLipedema%7C%20P%C3%B3s%20Operat%C3%B3rio%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11994003820?text=Ol%C3%A1%2C%20Nadia%20Ces%C3%A1rio!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Vila%20Mariana.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nadia%20Ces%C3%A1rio%20-%20Est%C3%A9tica%20Especializada%20%7CDrenagem%20Linf%C3%A1tica%20Vila%20Mariana%20%7CLimpeza%20de%20pele%20%7CLipedema%7C%20P%C3%B3s%20Operat%C3%B3rio%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K70" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Nadia Cesário! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nadia Cesário - Estética Especializada |Drenagem Linfática Vila Mariana |Limpeza de pele |Lipedema| Pós Operatório, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Nadia Cesário! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Vila Mariana. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nadia Cesário - Estética Especializada |Drenagem Linfática Vila Mariana |Limpeza de pele |Lipedema| Pós Operatório, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="71" xml:space="preserve">
@@ -3085,13 +3154,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J71" t="str">
-        <v>https://wa.me/11999985553?text=Ol%C3%A1%2C%20Dra.%20Mage!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Dra.%20Mage%20Mantovani%20Est%C3%A9tica%20Avan%C3%A7ada%20Vila%20Mariana%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11999985553?text=Ol%C3%A1%2C%20Dra.%20Mage!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Vila%20Mariana.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20Dra.%20Mage%20Mantovani%20Est%C3%A9tica%20Avan%C3%A7ada%20Vila%20Mariana%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K71" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Mage! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica Dra. Mage Mantovani Estética Avançada Vila Mariana, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Mage! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Vila Mariana. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clínica Dra. Mage Mantovani Estética Avançada Vila Mariana, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="72" xml:space="preserve">
@@ -3123,13 +3193,14 @@
         <v>https://www.instagram.com/dra.amandarubio?igsh=MTI5NmJkZWU2d2VlMw==&amp;utm_source=qr</v>
       </c>
       <c r="J72" t="str">
-        <v>https://wa.me/11974771241?text=Ol%C3%A1%2C%20Dra%20Amanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Amanda%20Rubio%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11974771241?text=Ol%C3%A1%2C%20Dra%20Amanda!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Vila%20Mariana.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Amanda%20Rubio%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20e%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K72" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Amanda! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Amanda Rubio - Harmonização Facial e Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Amanda! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Vila Mariana. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Amanda Rubio - Harmonização Facial e Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="73" xml:space="preserve">
@@ -3161,13 +3232,14 @@
         <v>https://wa.me//5511993736844?text=Ol%C3%A1!%20Encontrei%20no%20Google%20e%20quero%20saber%20mais.</v>
       </c>
       <c r="J73" t="str">
-        <v>https://wa.me/11993736844?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Bruna%20Martinez%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993736844?text=Ol%C3%A1%2C%20Dra.%20Bruna!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Bruna%20Martinez%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%20SP%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K73" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Bruna Martinez - Harmonização Facial Tatuapé SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Bruna! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Bruna Martinez - Harmonização Facial Tatuapé SP, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="74" xml:space="preserve">
@@ -3199,13 +3271,14 @@
         <v>https://wa.me/message/CIUHJ3HBXIETA1</v>
       </c>
       <c r="J74" t="str">
-        <v>https://wa.me/11994073067?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Guimar%C3%A3es%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11994073067?text=Ol%C3%A1%2C%20Dra%20Luana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Luana%20Guimar%C3%A3es%20Rosa%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K74" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Luana Guimarães Rosa | Harmonização Facial Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Luana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Luana Guimarães Rosa | Harmonização Facial Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="75" xml:space="preserve">
@@ -3237,13 +3310,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J75" t="str">
-        <v>https://wa.me/11953634975?text=Ol%C3%A1%2C%20Dra.%20Vit%C3%B3ria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Vit%C3%B3ria%20Caldeira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11953634975?text=Ol%C3%A1%2C%20Dra.%20Vit%C3%B3ria!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Vit%C3%B3ria%20Caldeira%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K75" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Vitória! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Vitória Caldeira | Harmonização Facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Vitória! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Vitória Caldeira | Harmonização Facial no Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="76" xml:space="preserve">
@@ -3275,13 +3349,14 @@
         <v>https://wa.me/5511945950480</v>
       </c>
       <c r="J76" t="str">
-        <v>https://wa.me/11945950480?text=Ol%C3%A1%2C%20Dra.%20Gisele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Gisele%20Neves%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%20%7C%20Botox%20%7C%20Ultraformer%20%7C%20Sculptra%20%7C%20Radiesse%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945950480?text=Ol%C3%A1%2C%20Dra.%20Gisele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Gisele%20Neves%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%20%7C%20Botox%20%7C%20Ultraformer%20%7C%20Sculptra%20%7C%20Radiesse%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K76" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Gisele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Gisele Neves - Harmonização Facial no Tatuapé | Botox | Ultraformer | Sculptra | Radiesse, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Gisele! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Gisele Neves - Harmonização Facial no Tatuapé | Botox | Ultraformer | Sculptra | Radiesse, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="77" xml:space="preserve">
@@ -3313,13 +3388,14 @@
         <v>https://linktr.ee/dracarla.bocuto?fbclid=PAAabVkC7D5GvCg526Viljb7iD7leQoFXx5zYuUVFUNXw_8gCHOeAkCW2DXSw</v>
       </c>
       <c r="J77" t="str">
-        <v>https://wa.me/11982885834?text=Ol%C3%A1%2C%20Dra%20Carla!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Carla%20Bocuto%20Harmoniza%C3%A7%C3%A3o%20Natural%20-%20Botox%20Tatuap%C3%A9%2C%20Mind%20Est%C3%A9tica.%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11982885834?text=Ol%C3%A1%2C%20Dra%20Carla!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Carla%20Bocuto%20Harmoniza%C3%A7%C3%A3o%20Natural%20-%20Botox%20Tatuap%C3%A9%2C%20Mind%20Est%C3%A9tica.%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K77" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Carla! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Carla Bocuto Harmonização Natural - Botox Tatuapé, Mind Estética., pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Carla! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Carla Bocuto Harmonização Natural - Botox Tatuapé, Mind Estética., focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="78" xml:space="preserve">
@@ -3351,13 +3427,14 @@
         <v>https://www.instagram.com/dra.marinaferreira</v>
       </c>
       <c r="J78" t="str">
-        <v>https://wa.me/11983714557?text=Ol%C3%A1%2C%20Dra.%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marina%20Ferreira%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20%7C%20Tatuap%C3%A9%2FAn%C3%A1lia%20Franco%20SP%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11983714557?text=Ol%C3%A1%2C%20Dra.%20Marina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Marina%20Ferreira%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20%7C%20Tatuap%C3%A9%2FAn%C3%A1lia%20Franco%20SP%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K78" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marina Ferreira | Harmonização facial | Tatuapé/Anália Franco SP, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Marina! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Marina Ferreira | Harmonização facial | Tatuapé/Anália Franco SP, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="79" xml:space="preserve">
@@ -3389,13 +3466,14 @@
         <v>https://www.instagram.com/dra.leticiaforstner/</v>
       </c>
       <c r="J79" t="str">
-        <v>https://wa.me/11963070502?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Forstner%20%7C%20Otomodela%C3%A7%C3%A3o%20%E2%80%A2%20Preenchimento%20Labial%20%E2%80%A2%20Botox%20%E2%80%A2%20Harmoniza%C3%A7%C3%A3o%20Facial%20%E2%80%93%20Tatuap%C3%A9%20SP%20%7C%20Line%20Skin%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11963070502?text=Ol%C3%A1%2C%20Dra.%20Let%C3%ADcia!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Let%C3%ADcia%20Forstner%20%7C%20Otomodela%C3%A7%C3%A3o%20%E2%80%A2%20Preenchimento%20Labial%20%E2%80%A2%20Botox%20%E2%80%A2%20Harmoniza%C3%A7%C3%A3o%20Facial%20%E2%80%93%20Tatuap%C3%A9%20SP%20%7C%20Line%20Skin%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K79" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Letícia Forstner | Otomodelação • Preenchimento Labial • Botox • Harmonização Facial – Tatuapé SP | Line Skin, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Letícia! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Letícia Forstner | Otomodelação • Preenchimento Labial • Botox • Harmonização Facial – Tatuapé SP | Line Skin, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="80" xml:space="preserve">
@@ -3427,13 +3505,14 @@
         <v>https://instagram.com/dra.carolinelopess?igshid=MzMyNGUyNmU2YQ==</v>
       </c>
       <c r="J80" t="str">
-        <v>https://wa.me/11969170606?text=Ol%C3%A1%2C%20Dra.%20Caroline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Caroline%20Lopes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11969170606?text=Ol%C3%A1%2C%20Dra.%20Caroline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Caroline%20Lopes%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K80" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Caroline! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Caroline Lopes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Caroline! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Caroline Lopes, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="81" xml:space="preserve">
@@ -3465,13 +3544,14 @@
         <v>https://www.instagram.com/dra.micheleneri?igsh=ajcyeXp0Nm1xM3Zk&amp;utm_source=qr</v>
       </c>
       <c r="J81" t="str">
-        <v>https://wa.me/11942945433?text=Ol%C3%A1%2C%20Dra.%20Michele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Michele%20Neri%20%E2%80%93%20Harmoniza%C3%A7%C3%A3o%20Facial%20%26%20Corporal%20%7C%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11942945433?text=Ol%C3%A1%2C%20Dra.%20Michele!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Michele%20Neri%20%E2%80%93%20Harmoniza%C3%A7%C3%A3o%20Facial%20%26%20Corporal%20%7C%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K81" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Michele! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Michele Neri – Harmonização Facial &amp; Corporal | Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Michele! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Michele Neri – Harmonização Facial &amp; Corporal | Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="82" xml:space="preserve">
@@ -3503,13 +3583,14 @@
         <v>http://www.instagram.com/draandressalopes</v>
       </c>
       <c r="J82" t="str">
-        <v>https://wa.me/11932253874?text=Ol%C3%A1%2C%20Dra%20Andressa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Andressa%20Lopes%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11932253874?text=Ol%C3%A1%2C%20Dra%20Andressa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Andressa%20Lopes%20-%20Harmoniza%C3%A7%C3%A3o%20Facial%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K82" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Andressa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Andressa Lopes - Harmonização Facial, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Andressa! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Andressa Lopes - Harmonização Facial, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="83" xml:space="preserve">
@@ -3541,13 +3622,14 @@
         <v>https://www.instagram.com/drasuellenalbuquerque/</v>
       </c>
       <c r="J83" t="str">
-        <v>https://wa.me/11918467067?text=Ol%C3%A1%2C%20Dra%20Su%C3%A9llen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Su%C3%A9llen%20Albuquerque%20-%20Cl%C3%ADnica%20de%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11918467067?text=Ol%C3%A1%2C%20Dra%20Su%C3%A9llen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Su%C3%A9llen%20Albuquerque%20-%20Cl%C3%ADnica%20de%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K83" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Suéllen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Suéllen Albuquerque - Clínica de Harmonização Facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Suéllen! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Suéllen Albuquerque - Clínica de Harmonização Facial no Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="84" xml:space="preserve">
@@ -3579,13 +3661,14 @@
         <v>https://www.instagram.com/dratalita.trevisan/</v>
       </c>
       <c r="J84" t="str">
-        <v>https://wa.me/11913257440?text=Ol%C3%A1%2C%20Dra%20Talita!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Talita%20Trevisan%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11913257440?text=Ol%C3%A1%2C%20Dra%20Talita!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Talita%20Trevisan%20%7C%20Harmoniza%C3%A7%C3%A3o%20facial%20no%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K84" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Talita! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Talita Trevisan | Harmonização facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Talita! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Talita Trevisan | Harmonização facial no Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="85" xml:space="preserve">
@@ -3617,13 +3700,14 @@
         <v>https://www.instagram.com/dragreicekelli?igsh=MWFicHZibDl6bjJ3dw%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J85" t="str">
-        <v>https://wa.me/11999627447?text=Ol%C3%A1%2C%20Dra.%20Greice!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Tatuap%C3%A9%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Greice%20Keli-%20Est%C3%A9tica%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11999627447?text=Ol%C3%A1%2C%20Dra.%20Greice!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Tatuap%C3%A9%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Tatuap%C3%A9.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Greice%20Keli-%20Est%C3%A9tica%20e%20Harmoniza%C3%A7%C3%A3o%20Facial%20no%20Tatuap%C3%A9%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K85" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Greice! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Tatuapé e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Greice Keli- Estética e Harmonização Facial no Tatuapé, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Greice! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Tatuapé (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Tatuapé. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Greice Keli- Estética e Harmonização Facial no Tatuapé, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="86" xml:space="preserve">
@@ -3655,13 +3739,14 @@
         <v>https://linktr.ee/dra.cristinaizabel.s</v>
       </c>
       <c r="J86" t="str">
-        <v>https://wa.me/11962892115?text=Ol%C3%A1%2C%20Dra.%20Cristina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Cristina%20Silva%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11962892115?text=Ol%C3%A1%2C%20Dra.%20Cristina!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Perdizes.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Cristina%20Silva%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K86" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Cristina! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Cristina Silva - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Cristina! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Perdizes. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Cristina Silva - Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="87" xml:space="preserve">
@@ -3693,13 +3778,14 @@
         <v>https://www.instagram.com/yvya_estetica/</v>
       </c>
       <c r="J87" t="str">
-        <v>https://wa.me/11975740970?text=Ol%C3%A1%2C%20YvYa%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C9%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20YvYa%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20em%20Perdizes%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Limpeza%20de%20Pele%20%7C%20Preenchimento%20Facial%20%7C%20Ultrassom%20Microfocado%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11975740970?text=Ol%C3%A1%2C%20YvYa%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%204%2C9%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Perdizes.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20YvYa%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20em%20Perdizes%20%7C%20Harmoniza%C3%A7%C3%A3o%20Facial%20%7C%20Limpeza%20de%20Pele%20%7C%20Preenchimento%20Facial%20%7C%20Ultrassom%20Microfocado%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K87" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, YvYa Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 4,9★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para YvYa Clínica de Estética em Perdizes | Harmonização Facial | Limpeza de Pele | Preenchimento Facial | Ultrassom Microfocado, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, YvYa Clínica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 4,9★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Perdizes. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para YvYa Clínica de Estética em Perdizes | Harmonização Facial | Limpeza de Pele | Preenchimento Facial | Ultrassom Microfocado, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="88" xml:space="preserve">
@@ -3731,13 +3817,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J88" t="str">
-        <v>https://wa.me/11913567195?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20avan%C3%A7ada%20Perdizes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11913567195?text=Ol%C3%A1%2C%20Cl%C3%ADnica%20Est%C3%A9tica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Perdizes.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Cl%C3%ADnica%20de%20Est%C3%A9tica%20avan%C3%A7ada%20Perdizes%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K88" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Clínica Estética! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Clínica de Estética avançada Perdizes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Clínica Estética! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Perdizes. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Clínica de Estética avançada Perdizes, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="89" xml:space="preserve">
@@ -3769,13 +3856,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J89" t="str">
-        <v>https://wa.me/11914800366?text=Ol%C3%A1%2C%20FIG%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20FIG%20Clinic%20-%20Dra.%20Manuela%20de%20Souza%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11914800366?text=Ol%C3%A1%2C%20FIG%20Clinic!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Perdizes.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20FIG%20Clinic%20-%20Dra.%20Manuela%20de%20Souza%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K89" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, FIG Clinic! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para FIG Clinic - Dra. Manuela de Souza, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, FIG Clinic! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Perdizes. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para FIG Clinic - Dra. Manuela de Souza, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -3807,13 +3895,14 @@
         <v>https://www.instagram.com/dramadigiacomo?igsh=MTQzcHJnaXMxYnpiMQ==&amp;utm_source=qr</v>
       </c>
       <c r="J90" t="str">
-        <v>https://wa.me/11972848524?text=Ol%C3%A1%2C%20Dra.%20Marcela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marcela%20Di%20Giacomo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972848524?text=Ol%C3%A1%2C%20Dra.%20Marcela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Perdizes.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Marcela%20Di%20Giacomo%20-%20Est%C3%A9tica%20Avan%C3%A7ada%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K90" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marcela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marcela Di Giacomo - Estética Avançada, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Marcela! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Perdizes. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Marcela Di Giacomo - Estética Avançada, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="91" xml:space="preserve">
@@ -3845,13 +3934,14 @@
         <v>https://www.instagram.com/dra.clairpessoa/</v>
       </c>
       <c r="J91" t="str">
-        <v>https://wa.me/11954221740?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Facial!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Perdizes%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Est%C3%A9tica%20Facial%20%26%20Rejuvenescimento%20%7C%20Perdizes%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11954221740?text=Ol%C3%A1%2C%20Est%C3%A9tica%20Facial!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Perdizes%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Perdizes.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Est%C3%A9tica%20Facial%20%26%20Rejuvenescimento%20%7C%20Perdizes%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K91" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Estética Facial! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Perdizes e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Estética Facial &amp; Rejuvenescimento | Perdizes, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Estética Facial! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Perdizes (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Perdizes. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Estética Facial &amp; Rejuvenescimento | Perdizes, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="92" xml:space="preserve">
@@ -3883,13 +3973,14 @@
         <v>https://www.doctoralia.com.br/ana-regina-alencar-santos/dermatologista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=50473&amp;utm_content=website</v>
       </c>
       <c r="J92" t="str">
-        <v>https://wa.me/11960447173?text=Ol%C3%A1%2C%20Dra.%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C2%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Ana%20Regina%20Alencar%20Santos%2C%20Dermatologista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11960447173?text=Ol%C3%A1%2C%20Dra.%20Ana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%204%2C2%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Moema.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Ana%20Regina%20Alencar%20Santos%2C%20Dermatologista%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K92" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Ana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,2★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Ana Regina Alencar Santos, Dermatologista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Ana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 4,2★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Moema. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Ana Regina Alencar Santos, Dermatologista, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="93" xml:space="preserve">
@@ -3921,13 +4012,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J93" t="str">
-        <v>https://wa.me/11910324225?text=Ol%C3%A1%2C%20Dra%20Elisabeth!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Elisabeth%20Silveira%20-%20Dermatologia%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11910324225?text=Ol%C3%A1%2C%20Dra%20Elisabeth!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Moema.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Elisabeth%20Silveira%20-%20Dermatologia%20em%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K93" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Elisabeth! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Elisabeth Silveira - Dermatologia em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Elisabeth! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Moema. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Elisabeth Silveira - Dermatologia em São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="94" xml:space="preserve">
@@ -3959,13 +4051,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J94" t="str">
-        <v>https://wa.me/11993053569?text=Ol%C3%A1%2C%20Fernanda%20Lima!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Est%C3%A9tica%20%26%20Harmoniza%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C8%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Fernanda%20Lima%20Queiroz%20Noya%20de%20Abreu%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11993053569?text=Ol%C3%A1%2C%20Fernanda%20Lima!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%204%2C8%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quem%20decide%20fazer%20um%20procedimento%20est%C3%A9tico%20ou%20harmoniza%C3%A7%C3%A3o%20com%20dinheiro%20na%20m%C3%A3o%20pesquisa%20refer%C3%AAncias%20e%20cl%C3%ADnicas%20no%20Google%20aqui%20em%20Moema.%20O%20Instagram%20ajuda%20a%20mostrar%20fotos%2C%20mas%20no%20Google%20o%20cliente%20est%C3%A1%20na%20fase%20de%20decis%C3%A3o%20de%20compra.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20no%20Google%2C%20voc%C3%AA%20acaba%20perdendo%20esses%20agendamentos%20de%20alto%20valor%20e%20perdendo%20dinheiro%20todos%20os%20dias%20para%20outras%20cl%C3%ADnicas.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Fernanda%20Lima%20Queiroz%20Noya%20de%20Abreu%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K94" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Fernanda Lima! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Estética &amp; Harmonização em Moema e encontrei o seu perfil no Google com nota 4,8★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Fernanda Lima Queiroz Noya de Abreu, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Fernanda Lima! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 4,8★ no Google, parabéns!).
+Te mandei mensagem porque quem decide fazer um procedimento estético ou harmonização com dinheiro na mão pesquisa referências e clínicas no Google aqui em Moema. O Instagram ajuda a mostrar fotos, mas no Google o cliente está na fase de decisão de compra. Como você está sem um site próprio no Google, você acaba perdendo esses agendamentos de alto valor e perdendo dinheiro todos os dias para outras clínicas.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Fernanda Lima Queiroz Noya de Abreu, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="95" xml:space="preserve">
@@ -3997,13 +4090,14 @@
         <v>https://www.instagram.com/nutri.malubraidotti/</v>
       </c>
       <c r="J95" t="str">
-        <v>https://wa.me/11945167295?text=Ol%C3%A1%2C%20Malu!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Malu%20Braidotti%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11945167295?text=Ol%C3%A1%2C%20Malu!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Moema.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Malu%20Braidotti%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K95" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Malu! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Malu Braidotti, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Malu! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Moema. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Malu Braidotti, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="96" xml:space="preserve">
@@ -4035,13 +4129,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J96" t="str">
-        <v>https://wa.me/11937287838?text=Ol%C3%A1%2C%20Centro%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Centro%20de%20Nutri%C3%A7%C3%A3o%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11937287838?text=Ol%C3%A1%2C%20Centro%20Nutri%C3%A7%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Moema.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Centro%20de%20Nutri%C3%A7%C3%A3o%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K96" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Centro Nutrição! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Centro de Nutrição, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Centro Nutrição! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Moema. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Centro de Nutrição, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="97" xml:space="preserve">
@@ -4073,13 +4168,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J97" t="str">
-        <v>https://wa.me/11997196772?text=Ol%C3%A1%2C%20Nutri%C3%A7%C3%A3o%20Personalizada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutri%C3%A7%C3%A3o%20Personalizada%20-%20Dra%20Fab%C3%ADola%20Estela%20Domingues%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11997196772?text=Ol%C3%A1%2C%20Nutri%C3%A7%C3%A3o%20Personalizada!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Moema.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutri%C3%A7%C3%A3o%20Personalizada%20-%20Dra%20Fab%C3%ADola%20Estela%20Domingues%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K97" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Nutrição Personalizada! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutrição Personalizada - Dra Fabíola Estela Domingues, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Nutrição Personalizada! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Moema. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutrição Personalizada - Dra Fabíola Estela Domingues, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="98" xml:space="preserve">
@@ -4111,13 +4207,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J98" t="str">
-        <v>https://wa.me/11985928451?text=Ol%C3%A1%2C%20Esportivo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportivo%20em%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11985928451?text=Ol%C3%A1%2C%20Esportivo!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Moema.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Esportivo%20em%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K98" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Esportivo! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Esportivo em São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Esportivo! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Moema. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Esportivo em São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="99" xml:space="preserve">
@@ -4149,13 +4246,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J99" t="str">
-        <v>https://wa.me/11974981031?text=Ol%C3%A1%2C%20Wesen%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Moema%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%204%2C1%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Wesen%20Cl%C3%ADnica%20de%20Emagrecimento%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11974981031?text=Ol%C3%A1%2C%20Wesen%20Cl%C3%ADnica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Moema%20(nota%204%2C1%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Moema.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Wesen%20Cl%C3%ADnica%20de%20Emagrecimento%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K99" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Wesen Clínica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Moema e encontrei o seu perfil no Google com nota 4,1★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Wesen Clínica de Emagrecimento, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Wesen Clínica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Moema (nota 4,1★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Moema. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Wesen Clínica de Emagrecimento, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="100" xml:space="preserve">
@@ -4187,13 +4285,14 @@
         <v>https://www.instagram.com/larissafranco.nutri?igsh=MTE1MGZjenZvY3g3cw%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J100" t="str">
-        <v>https://wa.me/11988957410?text=Ol%C3%A1%2C%20Larissa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Larissa%20Franco%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11988957410?text=Ol%C3%A1%2C%20Larissa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Jardins.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Larissa%20Franco%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K100" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Larissa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Larissa Franco, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Larissa! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Jardins. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Larissa Franco, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="101" xml:space="preserve">
@@ -4225,13 +4324,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J101" t="str">
-        <v>https://wa.me/11922183012?text=Ol%C3%A1%2C%20Larissa%20Monteiro!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Larissa%20Monteiro%20Nutricionista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11922183012?text=Ol%C3%A1%2C%20Larissa%20Monteiro!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Jardins.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Larissa%20Monteiro%20Nutricionista%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K101" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Larissa Monteiro! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Larissa Monteiro Nutricionista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Larissa Monteiro! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Jardins. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Larissa Monteiro Nutricionista, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="102" xml:space="preserve">
@@ -4263,13 +4363,14 @@
         <v>https://www.instagram.com/nathalia.nutri/</v>
       </c>
       <c r="J102" t="str">
-        <v>https://wa.me/11976575363?text=Ol%C3%A1%2C%20nos!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20nos%20Jardins%20-%20Nath%C3%A1lia%20D'Abruzzo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11976575363?text=Ol%C3%A1%2C%20nos!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Jardins.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20nos%20Jardins%20-%20Nath%C3%A1lia%20D'Abruzzo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K102" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, nos! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista nos Jardins - Nathália D'Abruzzo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, nos! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Jardins. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista nos Jardins - Nathália D'Abruzzo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="103" xml:space="preserve">
@@ -4301,13 +4402,14 @@
         <v>https://www.doctoralia.com.br/marisa-graca/nutricionista/sao-paulo?utm_source=google&amp;utm_medium=gmb&amp;utm_campaign=705957&amp;utm_content=website</v>
       </c>
       <c r="J103" t="str">
-        <v>https://wa.me/11934427007?text=Ol%C3%A1%2C%20Dra.%20Marisa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Jardins%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra.%20Marisa%20Diniz%20Gra%C3%A7a%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11934427007?text=Ol%C3%A1%2C%20Dra.%20Marisa!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Jardins%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Jardins.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra.%20Marisa%20Diniz%20Gra%C3%A7a%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K103" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra. Marisa! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Jardins e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra. Marisa Diniz Graça, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra. Marisa! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Jardins (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Jardins. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra. Marisa Diniz Graça, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="104" xml:space="preserve">
@@ -4339,13 +4441,14 @@
         <v>https://wa.me/5511921795550?text=Ol%C3%A1!%20Vim%20pelo%20Google%20e%20gostaria%20de%20mais%20informa%C3%A7%C3%B5es%20sobre%20a%20consulta%20nutricional!</v>
       </c>
       <c r="J104" t="str">
-        <v>https://wa.me/11921795550?text=Ol%C3%A1%2C%20Rafael%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Rafael%20Morais%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11921795550?text=Ol%C3%A1%2C%20Rafael%20Morais!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Itaim%20Bibi.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Rafael%20Morais%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K104" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Rafael Morais! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Rafael Morais, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Rafael Morais! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Itaim Bibi. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Rafael Morais, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="105" xml:space="preserve">
@@ -4377,13 +4480,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J105" t="str">
-        <v>https://wa.me/11980982327?text=Ol%C3%A1%2C%20Dra%20Daniela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Dra%20Daniela%20Mendon%C3%A7a%20-%20Nutricionista%20Esportiva%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11980982327?text=Ol%C3%A1%2C%20Dra%20Daniela!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Itaim%20Bibi.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Dra%20Daniela%20Mendon%C3%A7a%20-%20Nutricionista%20Esportiva%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K105" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Dra Daniela! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Dra Daniela Mendonça - Nutricionista Esportiva, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Dra Daniela! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Itaim Bibi. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Dra Daniela Mendonça - Nutricionista Esportiva, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="106" xml:space="preserve">
@@ -4415,13 +4519,14 @@
         <v>https://wa.me/5511964236252</v>
       </c>
       <c r="J106" t="str">
-        <v>https://wa.me/11964236252?text=Ol%C3%A1%2C%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Jo%C3%A3o%20Pinheiro%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11964236252?text=Ol%C3%A1%2C%20Jo%C3%A3o!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Itaim%20Bibi.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Jo%C3%A3o%20Pinheiro%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K106" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, João! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista João Pinheiro, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, João! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Itaim Bibi. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista João Pinheiro, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="107" xml:space="preserve">
@@ -4453,13 +4558,14 @@
         <v>https://api.whatsapp.com/send?phone=5511981267772&amp;text=Ol%C3%A1%2C%20Andrea!%20Te%20encontrei%20no%20Google%20e%20gostaria%20de%20mais%20informa%C3%A7%C3%B5es%20sobre%20a%20consulta%20com%20voc%C3%AA.%20Obrigado.</v>
       </c>
       <c r="J107" t="str">
-        <v>https://wa.me/11981267772?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Itaim%20Bibi%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Andrea%20Garrett%20Nutricionista%20no%20Itaim%20Bibi%20CRN3%2090979%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11981267772?text=Ol%C3%A1%2C%20no!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Itaim%20Bibi%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Itaim%20Bibi.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Andrea%20Garrett%20Nutricionista%20no%20Itaim%20Bibi%20CRN3%2090979%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K107" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Itaim Bibi e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Andrea Garrett Nutricionista no Itaim Bibi CRN3 90979, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, no! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Itaim Bibi (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Itaim Bibi. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Andrea Garrett Nutricionista no Itaim Bibi CRN3 90979, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="108" xml:space="preserve">
@@ -4491,13 +4597,14 @@
         <v>https://www.instagram.com/nutricionistaveronicanovais/</v>
       </c>
       <c r="J108" t="str">
-        <v>https://wa.me/11952251414?text=Ol%C3%A1%2C%20Ver%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ver%C3%B4nica%20Novais%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11952251414?text=Ol%C3%A1%2C%20Ver%C3%B4nica!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Pinheiros.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ver%C3%B4nica%20Novais%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K108" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Verônica! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Verônica Novais, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Verônica! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Pinheiros. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Verônica Novais, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="109" xml:space="preserve">
@@ -4529,13 +4636,14 @@
         <v>https://api.whatsapp.com/send?phone=5511972163767</v>
       </c>
       <c r="J109" t="str">
-        <v>https://wa.me/11972163767?text=Ol%C3%A1%2C%20Yuri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Yuri%20Gomes%20-%20Nutricionista%20Esportivo%20em%20Pinheiros%2C%20S%C3%A3o%20Paulo%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11972163767?text=Ol%C3%A1%2C%20Yuri!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Pinheiros.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Yuri%20Gomes%20-%20Nutricionista%20Esportivo%20em%20Pinheiros%2C%20S%C3%A3o%20Paulo%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K109" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Yuri! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Yuri Gomes - Nutricionista Esportivo em Pinheiros, São Paulo, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Yuri! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Pinheiros. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Yuri Gomes - Nutricionista Esportivo em Pinheiros, São Paulo, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="110" xml:space="preserve">
@@ -4567,13 +4675,14 @@
         <v>https://www.doctoralia.com.br/ellen-cortezi/nutricionista/sao-paulo</v>
       </c>
       <c r="J110" t="str">
-        <v>https://wa.me/11971308828?text=Ol%C3%A1%2C%20Ellen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ellen%20Hiromi%20Cortezi%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20institucional%20pr%C3%B3prio%20cadastrado%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11971308828?text=Ol%C3%A1%2C%20Ellen!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Pinheiros.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Ellen%20Hiromi%20Cortezi%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K110" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Ellen! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Ellen Hiromi Cortezi, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como você está sem um site institucional próprio cadastrado no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Ellen! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Pinheiros. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Ellen Hiromi Cortezi, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="111" xml:space="preserve">
@@ -4605,13 +4714,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J111" t="str">
-        <v>https://wa.me/11982923609?text=Ol%C3%A1%2C%20Aline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Aline%20Rodrigues%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11982923609?text=Ol%C3%A1%2C%20Aline!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Pinheiros.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Aline%20Rodrigues%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K111" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Aline! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Aline Rodrigues, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Aline! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Pinheiros. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Aline Rodrigues, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="112" xml:space="preserve">
@@ -4643,13 +4753,14 @@
         <v>https://www.instagram.com/mayrachamas?igsh=MXN2M2xyeXB4Z28xcw%3D%3D&amp;utm_source=qr</v>
       </c>
       <c r="J112" t="str">
-        <v>https://wa.me/11995262251?text=Ol%C3%A1%2C%20Mayra%20Chamas!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Pinheiros%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mayra%20Chamas%20Nutricionista%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11995262251?text=Ol%C3%A1%2C%20Mayra%20Chamas!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Pinheiros%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Pinheiros.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Mayra%20Chamas%20Nutricionista%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K112" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Mayra Chamas! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Pinheiros e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mayra Chamas Nutricionista, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Mayra Chamas! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Pinheiros (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Pinheiros. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Mayra Chamas Nutricionista, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="113" xml:space="preserve">
@@ -4681,13 +4792,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J113" t="str">
-        <v>https://wa.me/11948082545?text=Ol%C3%A1%2C%20Mariana%20Sena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Mariana%20Sena%20-%20Nutricionista%20Cl%C3%ADnica%20Funcional%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11948082545?text=Ol%C3%A1%2C%20Mariana%20Sena!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Vila%20Mariana.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Mariana%20Sena%20-%20Nutricionista%20Cl%C3%ADnica%20Funcional%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K113" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Mariana Sena! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Mariana Sena - Nutricionista Clínica Funcional, pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você está sem nenhum site cadastrado no perfil do Google Maps, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Mariana Sena! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Vila Mariana. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Mariana Sena - Nutricionista Clínica Funcional, focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="114" xml:space="preserve">
@@ -4719,13 +4831,14 @@
         <v>https://www.instagram.com/nutri_primazza/?hl=pt-br</v>
       </c>
       <c r="J114" t="str">
-        <v>https://wa.me/11996792653?text=Ol%C3%A1%2C%20Vegetariana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Vegetariana%2F%20Vegana%20Priscilla%20Mazza%20(Vila%20Mariana)%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20utiliza%20apenas%20link%20de%20rede%20social%20e%20est%C3%A1%20sem%20uma%20p%C3%A1gina%20oficial%20pr%C3%B3pria%20no%20Google%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11996792653?text=Ol%C3%A1%2C%20Vegetariana!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fica%20esperando%20post%20no%20feed%3A%20pesquisa%20direto%20no%20Google%20nutricionistas%20em%20Vila%20Mariana.%20Como%20voc%C3%AA%20est%C3%A1%20sem%20um%20site%20pr%C3%B3prio%20cadastrado%2C%20esses%20pacientes%20prontos%20para%20agendar%20acabam%20indo%20para%20outros%20consult%C3%B3rios%20e%20voc%C3%AA%20perde%20dinheiro%20todo%20m%C3%AAs.%0A%0APara%20resolver%20isso%20de%20forma%20imediata%2C%20selecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20com%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20j%C3%A1%20pronto%20e%20exclusivo%20para%20Nutricionista%20Vegetariana%2F%20Vegana%20Priscilla%20Mazza%20(Vila%20Mariana)%2C%20focado%20justamente%20em%20captar%20essas%20buscas%20com%20inten%C3%A7%C3%A3o%20de%20compra%20no%20Google%20e%20converter%20direto%20no%20seu%20WhatsApp.%0A%0APosso%20te%20enviar%20o%20link%20para%20voc%C3%AA%20dar%20uma%20olhada%20de%201%20minutinho%20sem%20compromisso%3F%20Faz%20sentido%20para%20voc%C3%AA%3F</v>
       </c>
       <c r="K114" t="str" xml:space="preserve">
-        <v xml:space="preserve">Olá, Vegetariana! Tudo bem? Sou o Gabriel, trabalho com criação de sites aqui em São Paulo.
-Acompanho as referências de Nutrição em Vila Mariana e encontrei o seu perfil no Google com nota 5,0★. Parabéns pelo trabalho e avaliações!
-Selecionei você para uma ação promocional exclusiva de 50% de desconto e preparei um novo modelo de site pronto e exclusivo para Nutricionista Vegetariana/ Vegana Priscilla Mazza (Vila Mariana), pensado para apresentar seus serviços com máxima autoridade no celular e facilitar o agendamento direto pelo WhatsApp.
-Como vi que você utiliza apenas link de rede social e está sem uma página oficial própria no Google, esse modelo já está estruturado para colocar no ar. Se você tiver 1 minutinho, gostaria de dar uma olhada sem compromisso para ver como ficou?</v>
+        <v xml:space="preserve">Olá, Vegetariana! Tudo bem? Sou o Gabriel, especialista em criação de sites e posicionamento no Google aqui em São Paulo.
+Acompanho o seu trabalho em Vila Mariana (nota 5,0★ no Google, parabéns!).
+Te mandei mensagem porque quando alguém decide cuidar da saúde, emagrecer ou precisa de um nutricionista com urgência, ela não fica esperando post no feed: pesquisa direto no Google nutricionistas em Vila Mariana. Como você está sem um site próprio cadastrado, esses pacientes prontos para agendar acabam indo para outros consultórios e você perde dinheiro todo mês.
+Para resolver isso de forma imediata, selecionei você para uma ação promocional com 50% de desconto e preparei um novo modelo de site já pronto e exclusivo para Nutricionista Vegetariana/ Vegana Priscilla Mazza (Vila Mariana), focado justamente em captar essas buscas com intenção de compra no Google e converter direto no seu WhatsApp.
+Posso te enviar o link para você dar uma olhada de 1 minutinho sem compromisso? Faz sentido para você?</v>
       </c>
     </row>
     <row r="115" xml:space="preserve">
@@ -4757,13 +4870,14 @@
         <v>Nenhum link cadastrado (Sem site)</v>
       </c>
       <c r="J115" t="str">
-        <v>https://wa.me/11942228782?text=Ol%C3%A1%2C%20Priscila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20trabalho%20com%20cria%C3%A7%C3%A3o%20de%20sites%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20as%20refer%C3%AAncias%20de%20Nutri%C3%A7%C3%A3o%20em%20Vila%20Mariana%20e%20encontrei%20o%20seu%20perfil%20no%20Google%20com%20nota%205%2C0%E2%98%85.%20Parab%C3%A9ns%20pelo%20trabalho%20e%20avalia%C3%A7%C3%B5es!%0A%0ASelecionei%20voc%C3%AA%20para%20uma%20a%C3%A7%C3%A3o%20promocional%20exclusiva%20de%2050%25%20de%20desconto%20e%20preparei%20um%20novo%20modelo%20de%20site%20pronto%20e%20exclusivo%20para%20Nutricionista%20Priscila%20Raso%2C%20pensado%20para%20apresentar%20seus%20servi%C3%A7os%20com%20m%C3%A1xima%20autoridade%20no%20celular%20e%20facilitar%20o%20agendamento%20direto%20pelo%20WhatsApp.%0A%0AComo%20vi%20que%20voc%C3%AA%20est%C3%A1%20sem%20nenhum%20site%20cadastrado%20no%20perfil%20do%20Google%20Maps%2C%20esse%20modelo%20j%C3%A1%20est%C3%A1%20estruturado%20para%20colocar%20no%20ar.%20Se%20voc%C3%AA%20tiver%201%20minutinho%2C%20gostaria%20de%20dar%20uma%20olhada%20sem%20compromisso%20para%20ver%20como%20ficou%3F</v>
+        <v>https://wa.me/11942228782?text=Ol%C3%A1%2C%20Priscila!%20Tudo%20bem%3F%20Sou%20o%20Gabriel%2C%20especialista%20em%20cria%C3%A7%C3%A3o%20de%20sites%20e%20posicionamento%20no%20Google%20aqui%20em%20S%C3%A3o%20Paulo.%0A%0AAcompanho%20o%20seu%20trabalho%20em%20Vila%20Mariana%20(nota%205%2C0%E2%98%85%20no%20Google%2C%20parab%C3%A9ns!).%0A%0ATe%20mandei%20mensagem%20porque%20quando%20algu%C3%A9m%20decide%20cuidar%20da%20sa%C3%BAde%2C%20emagrecer%20ou%20precisa%20de%20um%20nutricionista%20com%20urg%C3%AAncia%2C%20ela%20n%C3%A3o%20fic